<commit_message>
feat: humanização do bot para não cair no reCAPTCHA
</commit_message>
<xml_diff>
--- a/bcoDados.xlsx
+++ b/bcoDados.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -891,6 +891,96 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>10063021</v>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>1006.30.21</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="inlineStr">
+        <is>
+          <t>1006.30.21 — Polido ou brunido</t>
+        </is>
+      </c>
+      <c r="D11" s="1" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+      <c r="E11" s="1" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+      <c r="F11" s="1" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+      <c r="G11" s="1" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+      <c r="H11" s="1" t="inlineStr">
+        <is>
+          <t>Cumulativo / Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="I11" s="1" t="inlineStr">
+        <is>
+          <t>Cum: Lei nº 10.925/2004, artigo 1º, inciso V | N.Cum: Lei nº 10.925/2004, artigo 1º, inciso V</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n">
+        <v>87082999</v>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>8708.29.99</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>8708.29.99 — Outros</t>
+        </is>
+      </c>
+      <c r="D12" s="1" t="inlineStr">
+        <is>
+          <t>0,65%</t>
+        </is>
+      </c>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>3,00%</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="inlineStr">
+        <is>
+          <t>1,65%</t>
+        </is>
+      </c>
+      <c r="G12" s="1" t="inlineStr">
+        <is>
+          <t>7,60%</t>
+        </is>
+      </c>
+      <c r="H12" s="1" t="inlineStr">
+        <is>
+          <t>Monofásico</t>
+        </is>
+      </c>
+      <c r="I12" s="1" t="inlineStr">
+        <is>
+          <t>Cum: Lei nº 9.715/98, artigo 8º, inciso I; Lei nº 9.718/98, artigo 8º | N.Cum: Lei nº 10.637/2002, artigo 2º; Lei nº 10.833/2003, artigo 2º</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
feat(scraper): modo --todos com detecção de mudanças e sheet Histórico
- ler_ncms(apenas_incompletos) suporta dois modos de operação
- ler_dados_existentes() captura snapshot dos dados antes da execução
- _registrar_historico() compara campo a campo e grava diferenças
- salvar_excel() cria/atualiza sheet "Histórico" com data, NCM, campo, valor anterior e novo
- main() lê flag --todos para ativar verificação completa

Uso:
  python econet_scraper.py          # apenas NCMs incompletos (padrão)
  python econet_scraper.py --todos  # todos os NCMs + histórico de mudanças

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bcoDados.xlsx
+++ b/bcoDados.xlsx
@@ -7,6 +7,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Histórico" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -65,7 +66,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -75,6 +76,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -709,7 +713,7 @@
           <t>Bebidas Frias (Monofásico)</t>
         </is>
       </c>
-      <c r="I6" s="1" t="n"/>
+      <c r="I6" s="1" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
@@ -987,4 +991,52 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Data/Hora</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>NCM</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Campo</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Valor Anterior</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Valor Novo</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: funcao na skill para buscar todos ou incompletos
</commit_message>
<xml_diff>
--- a/bcoDados.xlsx
+++ b/bcoDados.xlsx
@@ -74,11 +74,11 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -157,8 +157,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tbNcm" displayName="tbNcm" ref="A1:A15" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:A15"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tbNcm" displayName="tbNcm" ref="A1:A17" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A1:A17"/>
   <tableColumns count="1">
     <tableColumn id="1" name="NCM"/>
   </tableColumns>
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -448,47 +448,47 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>NCM</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>NCM Econet</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Descrição</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>PIS Cumulativo</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>COFINS Cumulativo</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>PIS Não Cumulativo</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>COFINS Não Cumulativo</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>Regime</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>Legislação</t>
         </is>
@@ -980,6 +980,231 @@
         </is>
       </c>
       <c r="I12" s="1" t="inlineStr">
+        <is>
+          <t>Cum: Lei nº 9.715/98, artigo 8º, inciso I; Lei nº 9.718/98, artigo 8º | N.Cum: Lei nº 10.637/2002, artigo 2º; Lei nº 10.833/2003, artigo 2º</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30.75" customHeight="1">
+      <c r="A13" s="1" t="n">
+        <v>2071400</v>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>0207.14.00</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>0207.14.11 — Peitos</t>
+        </is>
+      </c>
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+      <c r="G13" s="1" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+      <c r="H13" s="1" t="inlineStr">
+        <is>
+          <t>Cumulativo / Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="I13" s="1" t="inlineStr">
+        <is>
+          <t>Cum: Lei nº 10.925/2004, artigo 1º, inciso XIX e § 4º | N.Cum: Lei nº 10.925/2004, artigo 1º, inciso XIX e § 4º</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="n">
+        <v>15079011</v>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>1507.90.11</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t>1507.90.11 — Em recipientes com capacidade inferior ou igual a 5 l</t>
+        </is>
+      </c>
+      <c r="D14" s="1" t="inlineStr">
+        <is>
+          <t>0,65%</t>
+        </is>
+      </c>
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t>3,00%</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="inlineStr">
+        <is>
+          <t>1,65%</t>
+        </is>
+      </c>
+      <c r="G14" s="1" t="inlineStr">
+        <is>
+          <t>7,60%</t>
+        </is>
+      </c>
+      <c r="H14" s="1" t="inlineStr">
+        <is>
+          <t>Cumulativo / Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="I14" s="1" t="inlineStr">
+        <is>
+          <t>Cum: Lei nº 9.715/98, artigo 8º, inciso I; Lei nº 9.718/98, artigo 8º | N.Cum: Lei nº 10.637/2002, artigo 2º; Lei nº 10.833/2003, artigo 2º</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="n">
+        <v>27101932</v>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>2710.19.32</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>2710.19.32 — Com aditivos</t>
+        </is>
+      </c>
+      <c r="D15" s="1" t="inlineStr">
+        <is>
+          <t>0,65%</t>
+        </is>
+      </c>
+      <c r="E15" s="1" t="inlineStr">
+        <is>
+          <t>3,00%</t>
+        </is>
+      </c>
+      <c r="F15" s="1" t="inlineStr">
+        <is>
+          <t>1,65%</t>
+        </is>
+      </c>
+      <c r="G15" s="1" t="inlineStr">
+        <is>
+          <t>7,60%</t>
+        </is>
+      </c>
+      <c r="H15" s="1" t="inlineStr">
+        <is>
+          <t>Cumulativo / Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="I15" s="1" t="inlineStr">
+        <is>
+          <t>Cum: Lei nº 9.715/98, artigo 8º, inciso I; Lei nº 9.718/98, artigo 8º | N.Cum: Lei nº 10.637/2002, artigo 2º; Lei nº 10.833/2003, artigo 2º</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="n">
+        <v>39269090</v>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
+        <is>
+          <t>3926.90.90</t>
+        </is>
+      </c>
+      <c r="C16" s="1" t="inlineStr">
+        <is>
+          <t>3926.90.90 — Outras</t>
+        </is>
+      </c>
+      <c r="D16" s="1" t="inlineStr">
+        <is>
+          <t>0,65%</t>
+        </is>
+      </c>
+      <c r="E16" s="1" t="inlineStr">
+        <is>
+          <t>3,00%</t>
+        </is>
+      </c>
+      <c r="F16" s="1" t="inlineStr">
+        <is>
+          <t>1,65%</t>
+        </is>
+      </c>
+      <c r="G16" s="1" t="inlineStr">
+        <is>
+          <t>7,60%</t>
+        </is>
+      </c>
+      <c r="H16" s="1" t="inlineStr">
+        <is>
+          <t>Cumulativo / Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="I16" s="1" t="inlineStr">
+        <is>
+          <t>Cum: Lei nº 9.715/98, artigo 8º, inciso I; Lei nº 9.718/98, artigo 8º | N.Cum: Lei nº 10.637/2002, artigo 2º; Lei nº 10.833/2003, artigo 2º</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="n">
+        <v>94036000</v>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>9403.60.00</t>
+        </is>
+      </c>
+      <c r="C17" s="1" t="inlineStr">
+        <is>
+          <t>9403.60.00 — Outros móveis de madeira</t>
+        </is>
+      </c>
+      <c r="D17" s="1" t="inlineStr">
+        <is>
+          <t>0,65%</t>
+        </is>
+      </c>
+      <c r="E17" s="1" t="inlineStr">
+        <is>
+          <t>3,00%</t>
+        </is>
+      </c>
+      <c r="F17" s="1" t="inlineStr">
+        <is>
+          <t>1,65%</t>
+        </is>
+      </c>
+      <c r="G17" s="1" t="inlineStr">
+        <is>
+          <t>7,60%</t>
+        </is>
+      </c>
+      <c r="H17" s="1" t="inlineStr">
+        <is>
+          <t>Cumulativo / Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="I17" s="1" t="inlineStr">
         <is>
           <t>Cum: Lei nº 9.715/98, artigo 8º, inciso I; Lei nº 9.718/98, artigo 8º | N.Cum: Lei nº 10.637/2002, artigo 2º; Lei nº 10.833/2003, artigo 2º</t>
         </is>
@@ -999,40 +1224,683 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="4" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Data/Hora</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>NCM</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Campo</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Valor Anterior</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Valor Novo</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-04-17 14:30</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1507.90.11</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1507.90.11 — Em recipientes com capacidade inferior ou igual a 5 l</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-04-17 14:30</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1507.90.11</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>PIS Cumulativo</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0,65%</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-04-17 14:30</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1507.90.11</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>COFINS Cumulativo</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>3,00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-04-17 14:30</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>1507.90.11</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>PIS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1,65%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-04-17 14:30</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1507.90.11</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>COFINS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>7,60%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-04-17 14:30</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1507.90.11</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Regime</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Cumulativo / Não Cumulativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-04-17 14:30</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1507.90.11</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Legislação</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Cum: Lei nº 9.715/98, artigo 8º, inciso I; Lei nº 9.718/98, artigo 8º | N.Cum: Lei nº 10.637/2002, artigo 2º; Lei nº 10.833/2003, artigo 2º</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-04-17 14:30</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2710.19.32</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2710.19.32 — Com aditivos</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-04-17 14:30</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2710.19.32</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>PIS Cumulativo</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>0,65%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-04-17 14:30</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2710.19.32</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>COFINS Cumulativo</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>3,00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-04-17 14:30</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2710.19.32</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>PIS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>1,65%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-04-17 14:30</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2710.19.32</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>COFINS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>7,60%</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-04-17 14:30</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2710.19.32</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Regime</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Cumulativo / Não Cumulativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-04-17 14:30</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2710.19.32</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Legislação</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Cum: Lei nº 9.715/98, artigo 8º, inciso I; Lei nº 9.718/98, artigo 8º | N.Cum: Lei nº 10.637/2002, artigo 2º; Lei nº 10.833/2003, artigo 2º</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-04-17 14:30</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>3926.90.90</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>3926.90.90 — Outras</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-04-17 14:30</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>3926.90.90</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>PIS Cumulativo</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>0,65%</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-04-17 14:30</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>3926.90.90</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>COFINS Cumulativo</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>3,00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-04-17 14:30</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>3926.90.90</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>PIS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>1,65%</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-04-17 14:30</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>3926.90.90</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>COFINS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>7,60%</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-04-17 14:30</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>3926.90.90</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Regime</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Cumulativo / Não Cumulativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-04-17 14:30</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>3926.90.90</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Legislação</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Cum: Lei nº 9.715/98, artigo 8º, inciso I; Lei nº 9.718/98, artigo 8º | N.Cum: Lei nº 10.637/2002, artigo 2º; Lei nº 10.833/2003, artigo 2º</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-04-17 14:30</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>9403.60.00</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>9403.60.00 — Outros móveis de madeira</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-04-17 14:30</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>9403.60.00</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>PIS Cumulativo</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>0,65%</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-04-17 14:30</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>9403.60.00</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>COFINS Cumulativo</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>3,00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-04-17 14:30</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>9403.60.00</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>PIS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>1,65%</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-04-17 14:30</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>9403.60.00</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>COFINS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>7,60%</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-04-17 14:30</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>9403.60.00</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Regime</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Cumulativo / Não Cumulativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-04-17 14:30</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>9403.60.00</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Legislação</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Cum: Lei nº 9.715/98, artigo 8º, inciso I; Lei nº 9.718/98, artigo 8º | N.Cum: Lei nº 10.637/2002, artigo 2º; Lei nº 10.833/2003, artigo 2º</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: adições na tabela
</commit_message>
<xml_diff>
--- a/bcoDados.xlsx
+++ b/bcoDados.xlsx
@@ -157,8 +157,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tbNcm" displayName="tbNcm" ref="A1:A17" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:A17"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tbNcm" displayName="tbNcm" ref="A1:A19" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A1:A19"/>
   <tableColumns count="1">
     <tableColumn id="1" name="NCM"/>
   </tableColumns>
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1210,6 +1210,96 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="1" t="n">
+        <v>85171231</v>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
+        <is>
+          <t>8517.12.31</t>
+        </is>
+      </c>
+      <c r="C18" s="1" t="inlineStr">
+        <is>
+          <t>8517.11.00 — Aparelhos telefônicos por fio com unidade auscultador-microfone sem fio</t>
+        </is>
+      </c>
+      <c r="D18" s="1" t="inlineStr">
+        <is>
+          <t>0,65%</t>
+        </is>
+      </c>
+      <c r="E18" s="1" t="inlineStr">
+        <is>
+          <t>3,00%</t>
+        </is>
+      </c>
+      <c r="F18" s="1" t="inlineStr">
+        <is>
+          <t>1,65%</t>
+        </is>
+      </c>
+      <c r="G18" s="1" t="inlineStr">
+        <is>
+          <t>7,60%</t>
+        </is>
+      </c>
+      <c r="H18" s="1" t="inlineStr">
+        <is>
+          <t>Cumulativo / Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="I18" s="1" t="inlineStr">
+        <is>
+          <t>Cum: Lei nº 9.715/98, artigo 8º, inciso I; Lei nº 9.718/98, artigo 8º | N.Cum: Lei nº 10.637/2002, artigo 2º; Lei nº 10.833/2003, artigo 2º</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n">
+        <v>4022110</v>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
+        <is>
+          <t>0402.21.10</t>
+        </is>
+      </c>
+      <c r="C19" s="1" t="inlineStr">
+        <is>
+          <t>0402.21.10 — Leite integral</t>
+        </is>
+      </c>
+      <c r="D19" s="1" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+      <c r="E19" s="1" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+      <c r="F19" s="1" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+      <c r="G19" s="1" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+      <c r="H19" s="1" t="inlineStr">
+        <is>
+          <t>Cumulativo / Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="I19" s="1" t="inlineStr">
+        <is>
+          <t>Cum: Lei nº 10.925/2004, artigo 1º, inciso XI | N.Cum: Lei nº 10.925/2004, artigo 1º, inciso XI</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -1224,13 +1314,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="5"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1246,15 +1337,20 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
           <t>Campo</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Valor Anterior</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Valor Novo</t>
         </is>
@@ -1271,13 +1367,12 @@
           <t>1507.90.11</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Descrição</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>1507.90.11 — Em recipientes com capacidade inferior ou igual a 5 l</t>
         </is>
@@ -1294,13 +1389,12 @@
           <t>1507.90.11</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>PIS Cumulativo</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>0,65%</t>
         </is>
@@ -1317,13 +1411,12 @@
           <t>1507.90.11</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>COFINS Cumulativo</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>3,00%</t>
         </is>
@@ -1340,13 +1433,12 @@
           <t>1507.90.11</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>PIS Não Cumulativo</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>1,65%</t>
         </is>
@@ -1363,13 +1455,12 @@
           <t>1507.90.11</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>COFINS Não Cumulativo</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>7,60%</t>
         </is>
@@ -1386,13 +1477,12 @@
           <t>1507.90.11</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Regime</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Cumulativo / Não Cumulativo</t>
         </is>
@@ -1409,13 +1499,12 @@
           <t>1507.90.11</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>Legislação</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Cum: Lei nº 9.715/98, artigo 8º, inciso I; Lei nº 9.718/98, artigo 8º | N.Cum: Lei nº 10.637/2002, artigo 2º; Lei nº 10.833/2003, artigo 2º</t>
         </is>
@@ -1432,13 +1521,12 @@
           <t>2710.19.32</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>Descrição</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>2710.19.32 — Com aditivos</t>
         </is>
@@ -1455,13 +1543,12 @@
           <t>2710.19.32</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>PIS Cumulativo</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>0,65%</t>
         </is>
@@ -1478,13 +1565,12 @@
           <t>2710.19.32</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>COFINS Cumulativo</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>3,00%</t>
         </is>
@@ -1501,13 +1587,12 @@
           <t>2710.19.32</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>PIS Não Cumulativo</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>1,65%</t>
         </is>
@@ -1524,13 +1609,12 @@
           <t>2710.19.32</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>COFINS Não Cumulativo</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>7,60%</t>
         </is>
@@ -1547,13 +1631,12 @@
           <t>2710.19.32</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>Regime</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>Cumulativo / Não Cumulativo</t>
         </is>
@@ -1570,13 +1653,12 @@
           <t>2710.19.32</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>Legislação</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>Cum: Lei nº 9.715/98, artigo 8º, inciso I; Lei nº 9.718/98, artigo 8º | N.Cum: Lei nº 10.637/2002, artigo 2º; Lei nº 10.833/2003, artigo 2º</t>
         </is>
@@ -1593,13 +1675,12 @@
           <t>3926.90.90</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>Descrição</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>3926.90.90 — Outras</t>
         </is>
@@ -1616,13 +1697,12 @@
           <t>3926.90.90</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>PIS Cumulativo</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>0,65%</t>
         </is>
@@ -1639,13 +1719,12 @@
           <t>3926.90.90</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>COFINS Cumulativo</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>3,00%</t>
         </is>
@@ -1662,13 +1741,12 @@
           <t>3926.90.90</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>PIS Não Cumulativo</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>1,65%</t>
         </is>
@@ -1685,13 +1763,12 @@
           <t>3926.90.90</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>COFINS Não Cumulativo</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>7,60%</t>
         </is>
@@ -1708,13 +1785,12 @@
           <t>3926.90.90</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>Regime</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>Cumulativo / Não Cumulativo</t>
         </is>
@@ -1731,13 +1807,12 @@
           <t>3926.90.90</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>Legislação</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>Cum: Lei nº 9.715/98, artigo 8º, inciso I; Lei nº 9.718/98, artigo 8º | N.Cum: Lei nº 10.637/2002, artigo 2º; Lei nº 10.833/2003, artigo 2º</t>
         </is>
@@ -1754,13 +1829,12 @@
           <t>9403.60.00</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>Descrição</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>9403.60.00 — Outros móveis de madeira</t>
         </is>
@@ -1777,13 +1851,12 @@
           <t>9403.60.00</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>PIS Cumulativo</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>0,65%</t>
         </is>
@@ -1800,13 +1873,12 @@
           <t>9403.60.00</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>COFINS Cumulativo</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>3,00%</t>
         </is>
@@ -1823,13 +1895,12 @@
           <t>9403.60.00</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>PIS Não Cumulativo</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>1,65%</t>
         </is>
@@ -1846,13 +1917,12 @@
           <t>9403.60.00</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>COFINS Não Cumulativo</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>7,60%</t>
         </is>
@@ -1869,13 +1939,12 @@
           <t>9403.60.00</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>Regime</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>Cumulativo / Não Cumulativo</t>
         </is>
@@ -1892,15 +1961,462 @@
           <t>9403.60.00</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>Legislação</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>Cum: Lei nº 9.715/98, artigo 8º, inciso I; Lei nº 9.718/98, artigo 8º | N.Cum: Lei nº 10.637/2002, artigo 2º; Lei nº 10.833/2003, artigo 2º</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-04-17 15:18</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>8517.12.31</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>8517.11.00 — Aparelhos telefônicos por fio com unidade auscultador-microfone sem fio</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-04-17 15:18</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>8517.12.31</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>PIS Cumulativo</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>0,65%</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-04-17 15:18</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>8517.12.31</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>COFINS Cumulativo</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>3,00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-04-17 15:18</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>8517.12.31</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>PIS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>1,65%</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-04-17 15:18</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>8517.12.31</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>COFINS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>7,60%</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-04-17 15:18</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>8517.12.31</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Regime</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Cumulativo / Não Cumulativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-04-17 15:18</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>8517.12.31</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Legislação</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Cum: Lei nº 9.715/98, artigo 8º, inciso I; Lei nº 9.718/98, artigo 8º | N.Cum: Lei nº 10.637/2002, artigo 2º; Lei nº 10.833/2003, artigo 2º</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-04-17 15:28</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>0402.21.10</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>0402.21.10 — Leite integral</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-04-17 15:28</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>0402.21.10</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>PIS Cumulativo</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-04-17 15:28</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>0402.21.10</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>COFINS Cumulativo</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-04-17 15:28</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>0402.21.10</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>PIS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-04-17 15:28</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>0402.21.10</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>COFINS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-04-17 15:28</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>0402.21.10</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Regime</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Cumulativo / Não Cumulativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-04-17 15:28</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>0402.21.10</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Legislação</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Cum: Lei nº 10.925/2004, artigo 1º, inciso XI | N.Cum: Lei nº 10.925/2004, artigo 1º, inciso XI</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: extração multi-aba — Suspensão, ZFM e Observações por NCM
Expande buscar_ncm() para capturar dados de três abas (Regra Geral,
Suspensão, ZFM) extraindo seções Descrição, Alíquota e Observações.
Exclui CST e EFD-Contribuições conforme solicitado.

Novas colunas J–R no Excel: Observações (RG), Suspensão PIS/COFINS/
Legislação/Observações, ZFM PIS/COFINS/Legislação/Observações.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bcoDados.xlsx
+++ b/bcoDados.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:R19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -445,6 +445,15 @@
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="28" customWidth="1" min="8" max="8"/>
     <col width="65" customWidth="1" min="9" max="9"/>
+    <col width="55" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="55" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="50" customWidth="1" min="17" max="17"/>
+    <col width="55" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -493,6 +502,51 @@
           <t>Legislação</t>
         </is>
       </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Observações (Regra Geral)</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>Suspensão - PIS</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>Suspensão - COFINS</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>Suspensão - Legislação</t>
+        </is>
+      </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
+          <t>Suspensão - Observações</t>
+        </is>
+      </c>
+      <c r="O1" s="4" t="inlineStr">
+        <is>
+          <t>ZFM - PIS</t>
+        </is>
+      </c>
+      <c r="P1" s="4" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS</t>
+        </is>
+      </c>
+      <c r="Q1" s="4" t="inlineStr">
+        <is>
+          <t>ZFM - Legislação</t>
+        </is>
+      </c>
+      <c r="R1" s="4" t="inlineStr">
+        <is>
+          <t>ZFM - Observações</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
@@ -538,6 +592,96 @@
           <t>Cum: Lei nº 9.715/98, artigo 8º, inciso I; Lei nº 9.718/98, artigo 8º | N.Cum: Lei nº 10.637/2002, artigo 2º; Lei nº 10.833/2003, artigo 2º</t>
         </is>
       </c>
+      <c r="J2" s="1" t="inlineStr">
+        <is>
+          <t>ALTERAÇÃO NA NCM - A reclassificação dos códigos NCM promovida pelo Decreto nº 11.158/2022 não faz com que o produto sofra alteração de tributação prevista na legislação mencionada anteriormente.
+Desta forma, a definição da NCM deverá seguir o disposto no artigo 16 do RIPI (Decreto nº 7.212/2010). Para verificar se houve reclassificação utilize a ferramenta Correlação da NCM.
+REGRA GERAL - O código NCM pesquisado não se encontra dentre os produtos com benefícios fiscais de PIS e COFINS previstos em legislação. Antes de aplicar as alíquotas correspondentes ao regime tributário da pessoa jurídica é recomendado analisar as outras guias.
+CONDIÇÃO DO ADQUIRENTE - Antes de aplicar a alíquota básica, é importante verificar se a pessoa jurídica adquirente é habilitada em algum regime especial, se está localizada na Zona Franca de Manaus (ZFM) ou em Área de Livre Comércio (ALC), e se a receita é proveniente de exportação de mercadorias.
+SIMPLES NACIONAL - A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+DARF - As empresas optantes pelo regime cumulativo recolherão o PIS e a COFINS em DARF, nos códigos 8109 e 2172, respectivamente.
+Para o regime não cumulativo os códigos serão 6912 e 5856.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
+      <c r="K2" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="L2" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="M2" s="1" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+      <c r="N2" s="1" t="inlineStr">
+        <is>
+          <t>ALTERAÇÃO NA NCM - A reclassificação dos códigos NCM promovida pelo Decreto nº 11.158/2022 não faz com que o produto sofra alteração de tributação prevista na legislação mencionada anteriormente.
+Desta forma, a definição da NCM deverá seguir o disposto no artigo 16 do RIPI (Decreto nº 7.212/2010). Para verificar se houve reclassificação utilize a ferramenta Correlação da NCM.
+SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da suspensão do PIS e da COFINS sobre as receitas de vendas de mercadorias, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+REGIME CUMULATIVO / NÃO CUMULATIVO - Aplica-se a suspensão do PIS e da COFINS:
+a) na venda realizada para pessoa jurídica beneficiária do Regime Especial de Aquisição de bens de Capital para Empresas Exportadoras (RECAP), para incorporação ao seu ativo imobilizado (Lei nº 11.196/2005, artigo 12; Decreto nº 5.789/2006);
+b) na venda para pessoa jurídica beneficiária do RECAP, sobre os bens adquiridos ou importados por estaleiro naval brasileiro (Lei nº 11.196/2005, artigo 13, § 3º, inciso II; Decreto nº 5.788/2006). Essa suspensão aplica-se somente quando os referidos bens forem destinados às atividades de construção, conservação, modernização, conversão e reparo de embarcações pré-registradas ou registradas no Registro Especial Brasileiro (REB), instituído pela Lei nº 9.432/97;
+c) na venda realizada a pessoa jurídica inscrita no Regime Especial de Tributação para Desenvolvimento da Atividade de Exibição Cinematográfica (RECINE) (Lei nº 12.599/2012, artigos 12 a 15; Decreto nº 7.729/2012).
+Prazo de vigência do benefício do RECINE: Até 31.12.2029 (Lei nº 13.594/2018);
+d) na venda de bens novos, destinados ao desenvolvimento, no País, de software e de serviços de tecnologia da informação, quando os referidos bens forem adquiridos por pessoa jurídica beneficiária do Regime Especial de Tributação para a Plataforma de Exportação de Serviços de Tecnologia da Informação (REPES) para incorporação ao seu ativo imobilizado (Lei nº 11.196/2005, artigos 4º e 11; Decreto nº 5.713/2006, artigo 1º).
+A partir de 01.04.2026, os incentivos e benefícios federais de natureza tributária são reduzidos, sendo aqueles de alíquota zero mediante a aplicação de alíquota correspondente a 10% da alíquota do sistema padrão de tributação. Desta forma, tendo em vista que para o PIS e a Cofins existem dois regimes de tributação, as alíquotas devem corresponder a 10% das alíquotas padrão de cada um dos regimes:
+a) Regime cumulativo - PIS: 0,065%; Cofins: 0,3%;
+b) Regime não cumulativo - PIS: 0,165%; Cofins: 0,76%. (Lei Complementar nº 224/2025, artigo 4º, caput e § 4º, inciso I)
+Ressalta-se que o § 1°, do artigo 2°, da IN RFB n° 2.305/2025 limita a redução dos benefícios àqueles discriminados no demonstrativo de gastos tributários anexo à Lei Orçamentária Anual de 2026. O Recine está discriminado, sofrendo redução do benefício.
+O Recap e o Repes não estão discriminados no demonstrativo de gastos tributários, não se sujeitando à redução estabelecida na Lei Complementar nº 224/2025.
+Quanto à aplicação da redução dos benefícios, no caso da suspensão, o artigo 6°, da IN RFB n° 2.305/2025 estabelece que a redução não se aplica aos benefícios de suspensão em que se verifique apenas um diferimento temporal no recolhimento do tributo. Logo, tendo em vista que o inciso II, do § 3°, do artigo 14, da Lei n° 12.599/2012 estabelece que a suspensão do PIS/Cofins converte-se em alíquota zero após a incorporação do bem ou material de construção no ativo imobilizado ou sua utilização no complexo de exibição cinematográfica ou cinema itinerante, situação na qual a operação fica sujeita à redução do benefício disposto na Lei Complementar nº 224/2025.
+Preventivamente, a sugestão é de que no cálculo para demonstrar o aumento da carga deve ser aplicado 10% das alíquotas do sistema padrão de PIS/Cofins sobre as vendas ou importação, baseado no artigo 7° da IN RFB 2.305/2025. Tal sugestão é um entendimento que poderá ser confirmado ou reformulado mediante esclarecimento da RFB.
+Visto que essas informações não estão claras na legislação, recomenda-se ao contribuinte buscar o serviço do Receita Soluciona, por meio das Confederações Nacionais de Representação de Categorias Econômicas, às Centrais Sindicais, aos Órgãos de Registro de Classe com atuação nacional e Organizações Associativas Patronais e Empresarias.</t>
+        </is>
+      </c>
+      <c r="O2" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="P2" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="Q2" s="1" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+      <c r="R2" s="1" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+ZONA FRANCA DE MANAUS (ZFM) - Para os regimes cumulativo e não cumulativo, ficam reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas de vendas de mercadorias destinadas ao consumo (utilizadas diretamente ou para comercialização por atacado ou a varejo) ou à industrialização na Zona Franca de Manaus, por pessoa jurídica estabelecida fora da ZFM (Lei nº 10.996/2004, artigo 2º).
+Nas notas fiscais relativas à venda, deverá constar a expressão "Venda de mercadoria efetuada com alíquota zero da Contribuição para o PIS/Pasep e da COFINS - Lei nº 10.996/2004, artigo 2º".
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, terão a alíquota do PIS e da COFINS reduzidas a zero, exceto nas vendas de mercadorias que tenham como destinatárias pessoas jurídicas atacadistas e varejistas, sujeitas ao regime de apuração não cumulativa do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, §§ 3º e 4º). As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+MATÉRIAS-PRIMAS, PRODUTOS INTERMEDIÁRIOS E MATERIAIS DE EMBALAGEM - São reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas decorrentes da comercialização de matérias-primas, produtos intermediários e materiais de embalagem, produzidos na Zona Franca de Manaus para emprego em processo de industrialização por estabelecimentos industriais dos regimes cumulativo ou não cumulativo ali instalados, consoante projetos aprovados pelo Conselho de Administração da Superintendência da Zona Franca de Manaus (SUFRAMA) (Lei nº 10.637/2002, artigo 5º-A).
+REGIME NÃO CUMULATIVO - As alíquotas especiais para vendas realizadas por pessoa jurídica optante pelo regime não cumulativo estabelecida na Zona Franca de Manaus estão dispostas abaixo do item "Solução de Consulta".</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -583,6 +727,60 @@
           <t>Cum: Lei nº 9.715/98, artigo 8º, inciso I; Lei nº 9.718/98, artigo 8º | N.Cum: Lei nº 10.637/2002, artigo 2º; Lei nº 10.833/2003, artigo 2º</t>
         </is>
       </c>
+      <c r="J3" s="1" t="inlineStr">
+        <is>
+          <t>REGRA GERAL - O código NCM pesquisado pode enquadrar-se dentre os produtos com benefícios fiscais de PIS e COFINS previstos em legislação. Antes de aplicar as alíquotas correspondentes ao regime tributário da pessoa jurídica é recomendado analisar as outras guias.
+CONDIÇÃO DO ADQUIRENTE - Antes de aplicar a alíquota básica, é importante verificar se a pessoa jurídica adquirente é habilitada em algum regime especial, se está localizada na Zona Franca de Manaus (ZFM) ou em Área de Livre Comércio (ALC), e se a receita é proveniente de exportação de mercadorias.
+SIMPLES NACIONAL - A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+DARF - As empresas optantes pelo regime cumulativo recolherão o PIS e a COFINS em DARF, nos códigos 8109 e 2172, respectivamente.
+Para o regime não cumulativo os códigos serão 6912 e 5856.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
+      <c r="K3" s="1" t="inlineStr"/>
+      <c r="L3" s="1" t="inlineStr"/>
+      <c r="M3" s="1" t="inlineStr"/>
+      <c r="N3" s="1" t="inlineStr"/>
+      <c r="O3" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="P3" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="Q3" s="1" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+      <c r="R3" s="1" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+ZONA FRANCA DE MANAUS (ZFM) - Para os regimes cumulativo e não cumulativo, ficam reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas de vendas de mercadorias destinadas ao consumo (utilizadas diretamente ou para comercialização por atacado ou a varejo) ou à industrialização na Zona Franca de Manaus, por pessoa jurídica estabelecida fora da ZFM (Lei nº 10.996/2004, artigo 2º).
+Nas notas fiscais relativas à venda, deverá constar a expressão "Venda de mercadoria efetuada com alíquota zero da Contribuição para o PIS/Pasep e da COFINS - Lei nº 10.996/2004, artigo 2º".
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, terão a alíquota do PIS e da COFINS reduzidas a zero, exceto nas vendas de mercadorias que tenham como destinatárias pessoas jurídicas atacadistas e varejistas, sujeitas ao regime de apuração não cumulativa do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, §§ 3º e 4º). As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+MATÉRIAS-PRIMAS, PRODUTOS INTERMEDIÁRIOS E MATERIAIS DE EMBALAGEM - São reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas decorrentes da comercialização de matérias-primas, produtos intermediários e materiais de embalagem, produzidos na Zona Franca de Manaus para emprego em processo de industrialização por estabelecimentos industriais dos regimes cumulativo ou não cumulativo ali instalados, consoante projetos aprovados pelo Conselho de Administração da Superintendência da Zona Franca de Manaus (SUFRAMA) (Lei nº 10.637/2002, artigo 5º-A).
+REGIME NÃO CUMULATIVO - As alíquotas especiais para vendas realizadas por pessoa jurídica optante pelo regime não cumulativo estabelecida na Zona Franca de Manaus estão dispostas abaixo do item "Solução de Consulta".</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
@@ -628,6 +826,60 @@
           <t>Cum: Lei nº 9.715/98, artigo 8º, inciso I; Lei nº 9.718/98, artigo 8º | N.Cum: Lei nº 10.637/2002, artigo 2º; Lei nº 10.833/2003, artigo 2º</t>
         </is>
       </c>
+      <c r="J4" s="1" t="inlineStr">
+        <is>
+          <t>REGRA GERAL - O código NCM pesquisado não se encontra dentre os produtos com benefícios fiscais de PIS e COFINS previstos em legislação. Antes de aplicar as alíquotas correspondentes ao regime tributário da pessoa jurídica é recomendado analisar as outras guias.
+CONDIÇÃO DO ADQUIRENTE - Antes de aplicar a alíquota básica, é importante verificar se a pessoa jurídica adquirente é habilitada em algum regime especial, se está localizada na Zona Franca de Manaus (ZFM) ou em Área de Livre Comércio (ALC), e se a receita é proveniente de exportação de mercadorias.
+SIMPLES NACIONAL - A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+DARF - As empresas optantes pelo regime cumulativo recolherão o PIS e a COFINS em DARF, nos códigos 8109 e 2172, respectivamente.
+Para o regime não cumulativo os códigos serão 6912 e 5856.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
+      <c r="K4" s="1" t="inlineStr"/>
+      <c r="L4" s="1" t="inlineStr"/>
+      <c r="M4" s="1" t="inlineStr"/>
+      <c r="N4" s="1" t="inlineStr"/>
+      <c r="O4" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="P4" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="Q4" s="1" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+      <c r="R4" s="1" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+ZONA FRANCA DE MANAUS (ZFM) - Para os regimes cumulativo e não cumulativo, ficam reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas de vendas de mercadorias destinadas ao consumo (utilizadas diretamente ou para comercialização por atacado ou a varejo) ou à industrialização na Zona Franca de Manaus, por pessoa jurídica estabelecida fora da ZFM (Lei nº 10.996/2004, artigo 2º).
+Nas notas fiscais relativas à venda, deverá constar a expressão "Venda de mercadoria efetuada com alíquota zero da Contribuição para o PIS/Pasep e da COFINS - Lei nº 10.996/2004, artigo 2º".
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, terão a alíquota do PIS e da COFINS reduzidas a zero, exceto nas vendas de mercadorias que tenham como destinatárias pessoas jurídicas atacadistas e varejistas, sujeitas ao regime de apuração não cumulativa do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, §§ 3º e 4º). As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+MATÉRIAS-PRIMAS, PRODUTOS INTERMEDIÁRIOS E MATERIAIS DE EMBALAGEM - São reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas decorrentes da comercialização de matérias-primas, produtos intermediários e materiais de embalagem, produzidos na Zona Franca de Manaus para emprego em processo de industrialização por estabelecimentos industriais dos regimes cumulativo ou não cumulativo ali instalados, consoante projetos aprovados pelo Conselho de Administração da Superintendência da Zona Franca de Manaus (SUFRAMA) (Lei nº 10.637/2002, artigo 5º-A).
+REGIME NÃO CUMULATIVO - As alíquotas especiais para vendas realizadas por pessoa jurídica optante pelo regime não cumulativo estabelecida na Zona Franca de Manaus estão dispostas abaixo do item "Solução de Consulta".</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
@@ -673,6 +925,71 @@
           <t>Cum: Lei nº 10.485/2002, artigo 1º | N.Cum: Lei nº 10.485/2002, artigo 1º</t>
         </is>
       </c>
+      <c r="J5" s="1" t="inlineStr">
+        <is>
+          <t>CONCEITO DE INCIDÊNCIA MONOFÁSICA - O sistema de tributação monofásica é um tratamento tributário próprio e específico, previsto em relação ao PIS e a COFINS incidentes sobre a receita bruta decorrente da venda de determinados produtos, geralmente a fim de concentrar a tributação nas etapas de produção e importação, desonerando as etapas subsequentes de comercialização.
+A concentração da tributação ocorre com a aplicação de alíquotas maiores que as usualmente aplicadas na tributação das demais receitas.
+O álcool e as bebidas frias relacionadas no artigo 14 da Lei nº 13.097/2015 são exceções à regra, visto que o distribuidor também é responsável pelo recolhimento do PIS e da COFINS.
+SIMPLES NACIONAL - As leis que estabelecem a incidência monofásica não trazem dispensa no recolhimento da alíquota concentrada quando se trata de importador ou fabricante optante pelo Simples Nacional. Deste modo, o importador e o fabricante deverão proceder o recolhimento do PIS e da COFINS em DARF separado, mediante a aplicação das alíquotas diferenciadas previstas em legislação própria conforme o produto.
+Deve ser destacada a receita decorrente da venda desse produto, aplicando-se, sobre tal receita, a alíquota efetiva calculada com base no Anexo II da Lei Complementar nº 123/2006, mas sem considerar os percentuais destinados ao PIS e a COFINS.
+Para tanto, o importador e a indústria devem selecionar a atividade de "venda de mercadorias industrializadas, com substituição tributária/tributação monofásica", indicando a opção tributação monofásica em relação ao PIS e a COFINS, a fim de que o aplicativo desconsidere os percentuais desses tributos sobre a receita destacada, ou seja, o recolhimento não será realizado pelo DAS e sim em DARF separado (Lei Complementar nº 123/2006, artigo 18, § 4º-A, inciso I).
+Desde 01.01.2018, a atividade de produção e venda no atacado de bebidas alcoólicas não está vedada ao ingresso ao Simples Nacional, desde que praticada por:
+a) micro e pequenas cervejarias;
+b) micro e pequenas vinícolas;
+c) produtores de licores;
+d) micro e pequenas destilarias.
+As ME e EPP optantes pelo Simples Nacional deverão obrigatoriamente estar registradas no Ministério da Agricultura, Pecuária e Abastecimento e obedecerão também à regulamentação da Agência Nacional de Vigilância Sanitária e da Secretaria da Receita Federal do Brasil quanto à produção e à comercialização de bebidas alcoólicas (Lei Complementar nº 123/2006, artigo 17, § 5º).
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+REGIME CUMULATIVO / NÃO CUMULATIVO (IMPORTADOR OU INDÚSTRIA) - A receita bruta auferida por importador ou por indústria, optantes pelos regimes cumulativo ou não cumulativo, sujeita-se à incidência monofásica do PIS e da COFINS sobre os produtos constantes nos artigos 1º e 3º da Lei nº 10.485/2002.
+PRODUTOS USADOS - Os produtos usados não estão sujeitos a incidência monofásica do PIS e da COFINS (Lei nº 10.485/2002, artigo 6º).
+INDUSTRIALIZAÇÃO POR ENCOMENDA - Na industrialização por encomenda, exceto sobre os medicamentos relacionados no artigo 1º, inciso I, alíneas "a" e "b" da Lei nº 10.147/2000, o PIS e a COFINS incidirão sobre a receita auferida pela pessoa jurídica executora da encomenda às alíquotas de 1,65% (PIS) e 7,60% (COFINS), independentemente do regime de apuração a que está submetida a pessoa jurídica. O encomendante deve recolher o PIS e a COFINS mediante as alíquotas monofásicas (Lei nº 11.051/2004, artigo 10, § 2º e Lei nº 10.833/2003, artigo 25, inciso I).
+DARF - As empresas optantes pelo Simples Nacional recolherão o PIS e a COFINS em DARF, nos códigos 8109 e 2172, respectivamente (Lei nº 10.833/2003, artigo 10, inciso III).
+Para as empresas optantes pelo regime cumulativo, o recolhimento será nos códigos 8109 e 2172 e para as optantes pelo regime não cumulativo, será nos códigos 6912 e 5856.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
+      <c r="K5" s="1" t="inlineStr"/>
+      <c r="L5" s="1" t="inlineStr"/>
+      <c r="M5" s="1" t="inlineStr"/>
+      <c r="N5" s="1" t="inlineStr"/>
+      <c r="O5" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="P5" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="Q5" s="1" t="inlineStr">
+        <is>
+          <t>Lei nº 10.485/2002, artigo 1º; Lei nº 11.196/2005, artigo 65</t>
+        </is>
+      </c>
+      <c r="R5" s="1" t="inlineStr">
+        <is>
+          <t>ALÍQUOTA - O fabricante ou importador dos produtos monofásicos citados no artigo 65 da Lei nº 11.196/2005 estabelecido fora da ZFM, fica obrigado a cobrar e recolher como substituto tributário o PIS e a COFINS devidos pela pessoa jurídica estabelecida na ZFM.
+Até 24.09.2020, as alíquotas eram de 2% (PIS) e de 9,6% (COFINS) (Lei nº 11.196/2005, artigo 65, § 1º, inciso III e Lei nº 10.485/2002, artigo 1º).
+A partir da vinculação da ADI nº 4.254, em 25.09.2020, o Supremo Tribunal Federal (STF) declarou a inconstitucionalidade das alíquotas majoradas citadas no artigo 65 da Lei nº 11.196/2005 e, em decorrência desse julgamento, o Ministro proferiu decisão determinando a aplicação das alíquotas gerais de 1,65% (PIS) e 7,6% (COFINS) para suprir a lacuna legislativa.
+Posteriormente, emitiu-se o Parecer SEI nº 298/2023 com vigência a partir de 30.03.2023, que concluiu pela inaplicabilidade legal das alíquotas estabelecidas pelo Ministro do STF e, determinou não ser possível a tributação sobre a revenda realizada pelas empresas situadas na ZFM, e consequentemente a substituição tributária pelo fabricante/importador, até que nova legislação fosse promulgada para fixar tais percentuais.
+Embora tenha sido publicada no DOU de 18.07.2023, a Instrução Normativa RFB nº 2.152/2023 consolidando no § 2º do artigo 545 e § 2º do artigo 551 da Instrução Normativa RFB nº 2.121/2022 a utilização das alíquotas de 1,65% (PIS) e 7,6% (COFINS), no mesmo sentido da ADI. Contudo, pela leitura do relatório complementar das Soluções de Consulta Cosit nº 271/2023 (item 20 do relatório) e nº 176/2024 (item 18 do relatório), a autoridade fiscal reconhece a necessidade de atualização do texto da Instrução Normativa para que ela seja adequada à redação do Parecer SEI nº 298/2023.
+Assim, interpreta-se que as alíquotas para o fabricante/importador na substituição tributária são:
+a) até 24.09.2020: 2% (PIS) e de 9,6% (COFINS) - Lei nº 11.196/2005, artigo 65, § 1º, inciso III;
+b) de 25.09.2020 em diante: inexistência de alíquotas para o importador/fabricante em decorrência de lacuna normativa, essa a ensejar, atualmente, a ausência de tributação na operação de revenda pela pessoa jurídica localizada na ZFM. - ADI nº 4.254; Parecer SEI nº 298/2023; SC Cosit nº 271/2023 e nº 176/2024.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica estabelecida fora dessas áreas, terão o mesmo tratamento da substituição tributária prevista para fabricante ou importador estabelecido fora da Zona Franca de Manaus. Porém, a redução a zero e a respectiva substituição tributária não se aplicam às vendas para adquirente atacadista ou varejista sujeito ao regime não cumulativo situado nas ALC (Lei nº 11.196/2005, artigos 2º, § 4º.
+As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+TRIBUTAÇÃO - A tributação de produtos monofásicos destinados ao consumo ou industrialização a Pessoas Jurídicas localizadas na ZFM possuirá dois momentos: a contribuição própria do vendedor localizado fora da área incentivada (redução a zero conforme prevê a Lei nº 10.996/2004, artigo 2º) e a contribuição como sujeito passivo por substituição tributária (responsável tributário), recolhendo antecipadamente o PIS e a COFINS do contribuinte situado na ZFM onde aplicará alíquotas de acordo com a legislação pertinente ao produto (Lei nº 11.196/2005, artigos 64 e 65; ADI nº 4.254).
+VENDA A MONTADORAS DE VEÍCULOS - Não haverá recolhimento da substituição tributária de PIS e COFINS nas vendas para montadoras de veículos situadas na ZFM, em relação as vendas das autopeças relacionadas nos Anexos I e II da Lei nº 10.485/2002 (Lei nº 11.196/2005, artigo 65, § 6º).
+DARF - As empresas optantes pelo regime cumulativo e não cumulativo recolherão o PIS e a COFINS em DARF, sobre as receitas de vendas à Zona Franca de Manaus (Substituição Tributária), nos códigos 1921 e 1840, respectivamente.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -714,6 +1031,55 @@
         </is>
       </c>
       <c r="I6" s="1" t="inlineStr"/>
+      <c r="J6" s="1" t="inlineStr">
+        <is>
+          <t>CONCEITO DE INCIDÊNCIA MONOFÁSICA - As bebidas frias listadas no artigo 14 da Lei nº 13.097/2015 estão sujeitas a incidência monofásica, conforme prevê o artigo 25 da referida Lei. O sistema de tributação monofásica é um tratamento tributário próprio e específico, previsto em relação ao PIS e a COFINS incidentes sobre a receita bruta decorrente da venda de determinados produtos, onde usualmente a tributação ocorre de forma concentrada no produtor e importador, e no caso das bebidas frias ocorrerá também no atacadista, desonerando as etapas subsequentes de comercialização. A concentração da tributação ocorre com a aplicação de alíquotas maiores que as usualmente aplicadas na tributação das demais receitas.
+Em relação aos produtos classificados nas posições 22.01 e 22.02 da Tipi, o alcance da incidência monofásica é exclusivamente para água e refrigerantes, refrescos, cerveja sem álcool, repositores hidroeletrolíticos, bebidas energéticas e compostos líquidos prontos para o consumo que contenham como ingrediente principal inositol, glucoronolactona, taurina ou cafeína, segundo o parágrafo único do artigo 1º do Decreto nº 8.442/2015.
+SIMPLES NACIONAL - Para os fabricantes, importadores e distribuidores, a tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento, pois neste regime tributário não caberá a aplicação das alíquotas correspondentes à incidência monofásica em função do disposto no artigo 25, § 2º da Lei nº 13.097/2015.
+Cabe destacar que a atividade de produção e venda no atacado de bebidas alcoólicas estava terminantemente vedada ao Simples Nacional até 31/12/2017, passando a ser autorizada nos casos excepcionais de produção ou venda no atacado por micro e pequenos produtores. A atividade de produção e venda no atacado de cervejas sem álcool permanecerá vedada mesmo após 31/12/2017 (Lei Complementar nº 123/2006, artigo 17, inciso X, alíneas "b" e "c").
+Já na venda a varejo (nos moldes do conceito de varejista abaixo), ficam reduzidas a zero as alíquotas do PIS e da COFINS, de modo que estes contribuintes poderão segregar a receita e desonerar os percentuais efetivos das contribuições. (Lei nº 13.097/2015, artigo 28, § 2º).
+RECOLHIMENTO - São responsáveis pelo recolhimento do PIS e da COFINS, os importadores, fabricantes e atacadistas dos produtos relacionados no artigo 14 da Lei nº 13.097/2015.
+VALORES MÍNIMOS - São estabelecidos valores mínimos para o PIS e a COFINS, conforme tipo de produto e da capacidade do recipiente, segundo o Anexo I da Lei nº 13.097/2015 (Decreto nº 8.442/2015, artigo 30). Os valores dos tributos não podem ser inferiores aos valores mínimos, mesmo após a aplicação de qualquer das reduções de alíquotas previstas no Decreto nº 8.442/2015.
+CONCEITO DE VAREJISTA - Considera-se varejista a pessoa jurídica cuja receita decorrente da venda de bens e serviços a consumidor final no ano-calendário imediatamente anterior ao da operação houver sido igual ou superior a 75% de sua receita total de venda de bens e serviços no mesmo período, depois de excluídos os impostos e contribuições incidentes sobre a venda (Decreto nº 8.442/2015, artigo 2º, inciso III, e artigo 3º).
+ALÍQUOTA ZERO - São reduzidas a zero as alíquotas de PIS e COFINS sobre as receitas auferidas por pessoa jurídica varejista, inclusive quando a venda for realizada por empresa optante pelo Simples Nacional (Decreto nº 8.442/2015, artigo 22, caput e § 2º).
+FRETE - Nas operações de venda por pessoa jurídica industrial ou atacadista, o valor do frete integrará a base de cálculo do PIS e da COFINS apurados pela pessoa jurídica vendedora dos citados produtos (Lei nº 13.097/2015, artigo 27; Decreto nº 8.442/2015, artigo 15).
+INDUSTRIALIZAÇÃO POR ENCOMENDA - Na industrialização por encomenda, observados os valores mínimos exigidos, o PIS e a COFINS incidirão sobre a receita auferida pela pessoa jurídica executora da encomenda às alíquotas de 1,65% (PIS) e 7,60% (COFINS), independentemente do regime de apuração a que está submetida a pessoa jurídica (Lei nº 13.097/2015, artigo 25, § 3º e artigo 33; Decreto nº 8.442/2015, artigos 18 e 30; Solução de Consulta Cosit nº 75/2019).
+CRÉDITO PELA AQUISIÇÃO - REGIME NÃO CUMULATIVO - A pessoa jurídica sujeita ao regime de apuração não cumulativa poderá descontar créditos de PIS e COFINS em relação à aquisição no mercado interno ou à importação desse produto, conforme os valores informados na nota fiscal do vendedor.
+Nas aquisições de produtos de pessoa jurídica optante pelo Simples Nacional, os créditos serão calculados mediante a aplicação sobre o valor de aquisição constante do documento fiscal de percentual correspondente a 0,38% (PIS) e 1,60% (COFINS) (Decreto nº 8.442/2015, artigos 24 e 29).
+UTILIZAÇÃO DO CRÉDITO - O crédito para o regime não cumulativo e o crédito presumido somente podem ser utilizados para desconto do valor do PIS e da COFINS devidos pela pessoa jurídica.
+VEDAÇÃO AO CRÉDITO - Fica vedado à pessoa jurídica varejista descontar os créditos do PIS e da COFINS, em relação ao produto revendido com a aplicação da alíquota zero, de acordo com os artigos 22 e 27 do Decreto nº 8.442/2015.
+DARF - As empresas optantes pelo regime cumulativo e não cumulativo recolherão o PIS e a COFINS em DARF, sobre as bebidas frias (Lei nº 13.097/2015, artigos 14 a 36) nos códigos 0691 e 0776, exceto cervejas, que devem ser recolhidos sob os códigos 0679 e 0760 respectivamente, segundo o ADE CODAC nº 21/2015.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
+      <c r="K6" s="1" t="inlineStr"/>
+      <c r="L6" s="1" t="inlineStr"/>
+      <c r="M6" s="1" t="inlineStr"/>
+      <c r="N6" s="1" t="inlineStr"/>
+      <c r="O6" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="P6" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="Q6" s="1" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+      <c r="R6" s="1" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+Com isso, a operação será tributada de acordo com os percentuais específicos aplicáveis às bebidas frias.
+ZONA FRANCA DE MANAUS (ZFM) - Os fabricantes, importadores, comerciantes atacadistas e varejistas estabelecidos fora da Zona Franca de Manaus que vendam bebidas frias para a região incentivada não se sujeitam à alíquota zero na venda, e, em consequência, não estarão sujeitos ao recolhimento na condição de contribuinte substituto do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, § 6º; Lei nº 13.097/2015, artigo 14).
+Com isso, a operação será tributada de acordo com os percentuais específicos aplicáveis às bebidas frias relacionadas na aba anterior.
+ÁREAS DE LIVRE COMÉRCIO - Da mesma forma que nas venda à Zona Franca de Manaus, as vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, não se sujeitam à alíquota zero, devendo ser tributada conforme os percentuais específicos previstos para as operações com bebidas frias relacionadas na aba anterior.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
@@ -759,6 +1125,80 @@
           <t>Cum: Lei nº 9.715/98, artigo 8º, inciso I; Lei nº 9.718/98, artigo 8º | N.Cum: Lei nº 10.637/2002, artigo 2º; Lei nº 10.833/2003, artigo 2º</t>
         </is>
       </c>
+      <c r="J7" s="1" t="inlineStr">
+        <is>
+          <t>REGRA GERAL - O código NCM pesquisado pode enquadrar-se dentre os produtos com benefícios fiscais de PIS e COFINS previstos em legislação. Antes de aplicar as alíquotas correspondentes ao regime tributário da pessoa jurídica é recomendado analisar as outras guias.
+CONDIÇÃO DO ADQUIRENTE - Antes de aplicar a alíquota básica, é importante verificar se a pessoa jurídica adquirente é habilitada em algum regime especial, se está localizada na Zona Franca de Manaus (ZFM) ou em Área de Livre Comércio (ALC), e se a receita é proveniente de exportação de mercadorias.
+NÃO APLICAÇÃO DA INCIDÊNCIA MONOFÁSICA - O Anexo I da Lei nº 10.485/2002 determina a incidência monofásica para a NCM 8481.80.99 Ex 01 e 02 e não se aplica a NCM 8481.80.99 (sem EX). Com a publicação do Decreto nº 5.804/2006, artigo 2º, ficaram suprimidos da tabela do IPI as posições EX 01 a 03 da NCM 8481.80.99 e por conseguinte, a incidência monofásica para as referidas posições NCM da Tipi.
+SIMPLES NACIONAL - A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+DARF - As empresas optantes pelo regime cumulativo recolherão o PIS e a COFINS em DARF, nos códigos 8109 e 2172, respectivamente.
+Para o regime não cumulativo os códigos serão 6912 e 5856.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
+      <c r="K7" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="L7" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="M7" s="1" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+      <c r="N7" s="1" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da suspensão do PIS e da COFINS sobre as receitas de vendas de mercadorias, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+REGIME CUMULATIVO / NÃO CUMULATIVO - Aplica-se a suspensão do PIS e da COFINS à venda realizada para pessoa jurídica beneficiária do Regime Especial de Aquisição de bens de Capital para Empresas Exportadoras (RECAP), para incorporação ao seu ativo imobilizado (Lei nº 11.196/2005, artigo 12; Decreto nº 5.789/2006).</t>
+        </is>
+      </c>
+      <c r="O7" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="P7" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="Q7" s="1" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+      <c r="R7" s="1" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+ZONA FRANCA DE MANAUS (ZFM) - Para os regimes cumulativo e não cumulativo, ficam reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas de vendas de mercadorias destinadas ao consumo (utilizadas diretamente ou para comercialização por atacado ou a varejo) ou à industrialização na Zona Franca de Manaus, por pessoa jurídica estabelecida fora da ZFM (Lei nº 10.996/2004, artigo 2º).
+Nas notas fiscais relativas à venda, deverá constar a expressão "Venda de mercadoria efetuada com alíquota zero da Contribuição para o PIS/Pasep e da COFINS - Lei nº 10.996/2004, artigo 2º".
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, terão a alíquota do PIS e da COFINS reduzidas a zero, exceto nas vendas de mercadorias que tenham como destinatárias pessoas jurídicas atacadistas e varejistas, sujeitas ao regime de apuração não cumulativa do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, §§ 3º e 4º). As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+MATÉRIAS-PRIMAS, PRODUTOS INTERMEDIÁRIOS E MATERIAIS DE EMBALAGEM - São reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas decorrentes da comercialização de matérias-primas, produtos intermediários e materiais de embalagem, produzidos na Zona Franca de Manaus para emprego em processo de industrialização por estabelecimentos industriais dos regimes cumulativo ou não cumulativo ali instalados, consoante projetos aprovados pelo Conselho de Administração da Superintendência da Zona Franca de Manaus (SUFRAMA) (Lei nº 10.637/2002, artigo 5º-A).
+REGIME NÃO CUMULATIVO - As alíquotas especiais para vendas realizadas por pessoa jurídica optante pelo regime não cumulativo estabelecida na Zona Franca de Manaus estão dispostas abaixo do item "Solução de Consulta".</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
@@ -804,6 +1244,87 @@
           <t>Cum: Lei nº 9.715/98, artigo 8º, inciso I; Lei nº 9.718/98, artigo 8º | N.Cum: Lei nº 10.637/2002, artigo 2º; Lei nº 10.833/2003, artigo 2º</t>
         </is>
       </c>
+      <c r="J8" s="1" t="inlineStr">
+        <is>
+          <t>REGRA GERAL - O código NCM pesquisado pode enquadrar-se dentre os produtos com benefícios fiscais de PIS e COFINS previstos em legislação. Antes de aplicar as alíquotas correspondentes ao regime tributário da pessoa jurídica é recomendado analisar as outras guias.
+CONDIÇÃO DO ADQUIRENTE - Antes de aplicar a alíquota básica, é importante verificar se a pessoa jurídica adquirente é habilitada em algum regime especial, se está localizada na Zona Franca de Manaus (ZFM) ou em Área de Livre Comércio (ALC), e se a receita é proveniente de exportação de mercadorias.
+SIMPLES NACIONAL - A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+DARF - As empresas optantes pelo regime cumulativo recolherão o PIS e a COFINS em DARF, nos códigos 8109 e 2172, respectivamente.
+Para o regime não cumulativo os códigos serão 6912 e 5856.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
+      <c r="K8" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="L8" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="M8" s="1" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+      <c r="N8" s="1" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da suspensão do PIS e da COFINS sobre as receitas de vendas de mercadorias, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+REGIME CUMULATIVO / NÃO CUMULATIVO - Aplica-se a suspensão do PIS e da COFINS nos casos de venda realizada a pessoa jurídica inscrita no Regime Especial de Tributação para Desenvolvimento da Atividade de Exibição Cinematográfica (RECINE) (Lei nº 12.599/2012, artigos 12 a 15; Decreto nº 7.729/2012).
+Prazo de vigência do benefício do RECINE: Até 31.12.2029 (Lei nº 13.594/2018).
+A partir de 01.04.2026, os incentivos e benefícios federais de natureza tributária são reduzidos, sendo aqueles de alíquota zero mediante a aplicação de alíquota correspondente a 10% da alíquota do sistema padrão de tributação. Desta forma, tendo em vista que para o PIS e a Cofins existem dois regimes de tributação, as alíquotas devem corresponder a 10% das alíquotas padrão de cada um dos regimes:
+a) Regime cumulativo - PIS: 0,065%; Cofins: 0,3%;
+b) Regime não cumulativo - PIS: 0,165%; Cofins: 0,76%. (Lei Complementar nº 224/2025, artigo 4º, caput e § 4º, inciso I)
+Ressalta-se que o § 1°, do artigo 2°, da IN RFB n° 2.305/2025 limita a redução dos benefícios àqueles discriminados no demonstrativo de gastos tributários anexo à Lei Orçamentária Anual de 2026. O Recine está discriminado, sofrendo redução do benefício.
+Quanto à aplicação da redução dos benefícios, no caso da suspensão, o artigo 6°, da IN RFB n° 2.305/2025 estabelece que a redução não se aplica aos benefícios de suspensão em que se verifique apenas um diferimento temporal no recolhimento do tributo. Logo, tendo em vista que o inciso II, do § 3°, do artigo 14, da Lei n° 12.599/2012 estabelece que a suspensão do PIS/Cofins converte-se em alíquota zero após a incorporação do bem ou material de construção no ativo imobilizado ou sua utilização no complexo de exibição cinematográfica ou cinema itinerante, situação na qual a operação fica sujeita à redução do benefício disposto na Lei Complementar nº 224/2025.
+Preventivamente, a sugestão é de que no cálculo para demonstrar o aumento da carga deve ser aplicado 10% das alíquotas do sistema padrão de PIS/Cofins sobre as vendas ou importação, baseado no artigo 7° da IN RFB 2.305/2025. Tal sugestão é um entendimento que poderá ser confirmado ou reformulado mediante esclarecimento da RFB.
+Visto que essas informações não estão claras na legislação, recomenda-se ao contribuinte buscar o serviço do Receita Soluciona, por meio das Confederações Nacionais de Representação de Categorias Econômicas, às Centrais Sindicais, aos Órgãos de Registro de Classe com atuação nacional e Organizações Associativas Patronais e Empresarias.</t>
+        </is>
+      </c>
+      <c r="O8" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="P8" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="Q8" s="1" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+      <c r="R8" s="1" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+ZONA FRANCA DE MANAUS (ZFM) - Para os regimes cumulativo e não cumulativo, ficam reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas de vendas de mercadorias destinadas ao consumo (utilizadas diretamente ou para comercialização por atacado ou a varejo) ou à industrialização na Zona Franca de Manaus, por pessoa jurídica estabelecida fora da ZFM (Lei nº 10.996/2004, artigo 2º).
+Nas notas fiscais relativas à venda, deverá constar a expressão "Venda de mercadoria efetuada com alíquota zero da Contribuição para o PIS/Pasep e da COFINS - Lei nº 10.996/2004, artigo 2º".
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, terão a alíquota do PIS e da COFINS reduzidas a zero, exceto nas vendas de mercadorias que tenham como destinatárias pessoas jurídicas atacadistas e varejistas, sujeitas ao regime de apuração não cumulativa do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, §§ 3º e 4º). As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+MATÉRIAS-PRIMAS, PRODUTOS INTERMEDIÁRIOS E MATERIAIS DE EMBALAGEM - São reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas decorrentes da comercialização de matérias-primas, produtos intermediários e materiais de embalagem, produzidos na Zona Franca de Manaus para emprego em processo de industrialização por estabelecimentos industriais dos regimes cumulativo ou não cumulativo ali instalados, consoante projetos aprovados pelo Conselho de Administração da Superintendência da Zona Franca de Manaus (SUFRAMA) (Lei nº 10.637/2002, artigo 5º-A).
+REGIME NÃO CUMULATIVO - As alíquotas especiais para vendas realizadas por pessoa jurídica optante pelo regime não cumulativo estabelecida na Zona Franca de Manaus estão dispostas abaixo do item "Solução de Consulta".</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
@@ -849,6 +1370,71 @@
           <t>Cum: Lei nº 10.147/2000, artigo 1º, inciso I, alínea "a" | N.Cum: Lei nº 10.147/2000, artigo 1º, inciso I, alínea "a"</t>
         </is>
       </c>
+      <c r="J9" s="1" t="inlineStr">
+        <is>
+          <t>CONCEITO DE INCIDÊNCIA MONOFÁSICA - O sistema de tributação monofásica é um tratamento tributário próprio e específico, previsto em relação ao PIS e a COFINS incidentes sobre a receita bruta decorrente da venda de determinados produtos, geralmente a fim de concentrar a tributação nas etapas de produção e importação, desonerando as etapas subsequentes de comercialização.
+A concentração da tributação ocorre com a aplicação de alíquotas maiores que as usualmente aplicadas na tributação das demais receitas.
+O álcool e as bebidas frias relacionadas no artigo 14 da Lei nº 13.097/2015 são exceções à regra, visto que o distribuidor também é responsável pelo recolhimento do PIS e da COFINS.
+SIMPLES NACIONAL - As leis que estabelecem a incidência monofásica não trazem dispensa no recolhimento da alíquota concentrada quando se trata de importador ou fabricante optante pelo Simples Nacional. Deste modo, o importador e o fabricante deverão proceder o recolhimento do PIS e da COFINS em DARF separado, mediante a aplicação das alíquotas diferenciadas previstas em legislação própria conforme o produto.
+Deve ser destacada a receita decorrente da venda desse produto, aplicando-se, sobre tal receita, a alíquota efetiva calculada com base no Anexo II da Lei Complementar nº 123/2006, mas sem considerar os percentuais destinados ao PIS e a COFINS.
+Para tanto, o importador e a indústria devem selecionar a atividade de "venda de mercadorias industrializadas, com substituição tributária/tributação monofásica", indicando a opção tributação monofásica em relação ao PIS e a COFINS, a fim de que o aplicativo desconsidere os percentuais desses tributos sobre a receita destacada, ou seja, o recolhimento não será realizado pelo DAS e sim em DARF separado (Lei Complementar nº 123/2006, artigo 18, § 4º-A, inciso I).
+Desde 01.01.2018, a atividade de produção e venda no atacado de bebidas alcoólicas não está vedada ao ingresso ao Simples Nacional, desde que praticada por:
+a) micro e pequenas cervejarias;
+b) micro e pequenas vinícolas;
+c) produtores de licores;
+d) micro e pequenas destilarias.
+As ME e EPP optantes pelo Simples Nacional deverão obrigatoriamente estar registradas no Ministério da Agricultura, Pecuária e Abastecimento e obedecerão também à regulamentação da Agência Nacional de Vigilância Sanitária e da Secretaria da Receita Federal do Brasil quanto à produção e à comercialização de bebidas alcoólicas (Lei Complementar nº 123/2006, artigo 17, § 5º).
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+REGIME CUMULATIVO / NÃO CUMULATIVO (IMPORTADOR OU INDÚSTRIA) - A receita bruta auferida por importador ou por indústria, optantes pelos regimes cumulativo ou não cumulativo, sujeita-se à incidência monofásica do PIS e da COFINS sobre os produtos constantes no artigo 1º da Lei nº 10.147/2000.
+INDUSTRIALIZAÇÃO POR ENCOMENDA - Na industrialização por encomenda, exceto sobre os medicamentos relacionados no artigo 1º, inciso I, alíneas "a" e "b" da Lei nº 10.147/2000, o PIS e a COFINS incidirão sobre a receita auferida pela pessoa jurídica executora da encomenda às alíquotas de 1,65% (PIS) e 7,60% (COFINS), independentemente do regime de apuração a que está submetida a pessoa jurídica. O encomendante deve recolher o PIS e a COFINS mediante as alíquotas monofásicas (Lei nº 11.051/2004, artigo 10, § 2º e Lei nº 10.833/2003, artigo 25, inciso I).
+DARF - As empresas optantes pelo Simples Nacional recolherão o PIS e a COFINS em DARF, nos códigos 8109 e 2172, respectivamente (Lei nº 10.833/2003, artigo 10, inciso III).
+Para as empresas optantes pelo regime cumulativo, o recolhimento será nos códigos 8109 e 2172 e para as optantes pelo regime não cumulativo, será nos códigos 6912 e 5856.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
+      <c r="K9" s="1" t="inlineStr"/>
+      <c r="L9" s="1" t="inlineStr"/>
+      <c r="M9" s="1" t="inlineStr"/>
+      <c r="N9" s="1" t="inlineStr"/>
+      <c r="O9" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="P9" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="Q9" s="1" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+      <c r="R9" s="1" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+ZONA FRANCA DE MANAUS (ZFM) - Para os regimes cumulativo e não cumulativo, ficam reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas de vendas de mercadorias destinadas ao consumo (utilizadas diretamente ou para comercialização por atacado ou a varejo) ou à industrialização na Zona Franca de Manaus, por pessoa jurídica estabelecida fora da ZFM (Lei nº 10.996/2004, artigo 2º).
+Nas notas fiscais relativas à venda, deverá constar a expressão "Venda de mercadoria efetuada com alíquota zero da Contribuição para o PIS/Pasep e da COFINS - Lei nº 10.996/2004, artigo 2º".
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, terão a alíquota do PIS e da COFINS reduzidas a zero, exceto nas vendas de mercadorias que tenham como destinatárias pessoas jurídicas atacadistas e varejistas, sujeitas ao regime de apuração não cumulativa do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, §§ 3º e 4º). As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+MATÉRIAS-PRIMAS, PRODUTOS INTERMEDIÁRIOS E MATERIAIS DE EMBALAGEM - São reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas decorrentes da comercialização de matérias-primas, produtos intermediários e materiais de embalagem, produzidos na Zona Franca de Manaus para emprego em processo de industrialização por estabelecimentos industriais dos regimes cumulativo ou não cumulativo ali instalados, consoante projetos aprovados pelo Conselho de Administração da Superintendência da Zona Franca de Manaus (SUFRAMA) (Lei nº 10.637/2002, artigo 5º-A).
+REGIME NÃO CUMULATIVO - As alíquotas especiais para vendas realizadas por pessoa jurídica optante pelo regime não cumulativo estabelecida na Zona Franca de Manaus estão dispostas abaixo do item "Solução de Consulta".</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
@@ -894,6 +1480,60 @@
           <t>Cum: Lei nº 9.715/98, artigo 8º, inciso I; Lei nº 9.718/98, artigo 8º | N.Cum: Lei nº 10.637/2002, artigo 2º; Lei nº 10.833/2003, artigo 2º</t>
         </is>
       </c>
+      <c r="J10" s="1" t="inlineStr">
+        <is>
+          <t>REGRA GERAL - O código NCM pesquisado não se encontra dentre os produtos com benefícios fiscais de PIS e COFINS previstos em legislação. Antes de aplicar as alíquotas correspondentes ao regime tributário da pessoa jurídica é recomendado analisar as outras guias.
+CONDIÇÃO DO ADQUIRENTE - Antes de aplicar a alíquota básica, é importante verificar se a pessoa jurídica adquirente é habilitada em algum regime especial, se está localizada na Zona Franca de Manaus (ZFM) ou em Área de Livre Comércio (ALC), e se a receita é proveniente de exportação de mercadorias.
+SIMPLES NACIONAL - A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+DARF - As empresas optantes pelo regime cumulativo recolherão o PIS e a COFINS em DARF, nos códigos 8109 e 2172, respectivamente.
+Para o regime não cumulativo os códigos serão 6912 e 5856.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
+      <c r="K10" s="1" t="inlineStr"/>
+      <c r="L10" s="1" t="inlineStr"/>
+      <c r="M10" s="1" t="inlineStr"/>
+      <c r="N10" s="1" t="inlineStr"/>
+      <c r="O10" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="P10" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="Q10" s="1" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+      <c r="R10" s="1" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+ZONA FRANCA DE MANAUS (ZFM) - Para os regimes cumulativo e não cumulativo, ficam reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas de vendas de mercadorias destinadas ao consumo (utilizadas diretamente ou para comercialização por atacado ou a varejo) ou à industrialização na Zona Franca de Manaus, por pessoa jurídica estabelecida fora da ZFM (Lei nº 10.996/2004, artigo 2º).
+Nas notas fiscais relativas à venda, deverá constar a expressão "Venda de mercadoria efetuada com alíquota zero da Contribuição para o PIS/Pasep e da COFINS - Lei nº 10.996/2004, artigo 2º".
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, terão a alíquota do PIS e da COFINS reduzidas a zero, exceto nas vendas de mercadorias que tenham como destinatárias pessoas jurídicas atacadistas e varejistas, sujeitas ao regime de apuração não cumulativa do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, §§ 3º e 4º). As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+MATÉRIAS-PRIMAS, PRODUTOS INTERMEDIÁRIOS E MATERIAIS DE EMBALAGEM - São reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas decorrentes da comercialização de matérias-primas, produtos intermediários e materiais de embalagem, produzidos na Zona Franca de Manaus para emprego em processo de industrialização por estabelecimentos industriais dos regimes cumulativo ou não cumulativo ali instalados, consoante projetos aprovados pelo Conselho de Administração da Superintendência da Zona Franca de Manaus (SUFRAMA) (Lei nº 10.637/2002, artigo 5º-A).
+REGIME NÃO CUMULATIVO - As alíquotas especiais para vendas realizadas por pessoa jurídica optante pelo regime não cumulativo estabelecida na Zona Franca de Manaus estão dispostas abaixo do item "Solução de Consulta".</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -939,6 +1579,57 @@
           <t>Cum: Lei nº 10.925/2004, artigo 1º, inciso V | N.Cum: Lei nº 10.925/2004, artigo 1º, inciso V</t>
         </is>
       </c>
+      <c r="J11" s="1" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+REGIME CUMULATIVO / NÃO CUMULATIVO - Aplica-se à alíquota zero do PIS e da COFINS à receita bruta de venda no mercado interno (Lei nº 10.925/2004, artigo 1º, inciso V).</t>
+        </is>
+      </c>
+      <c r="K11" s="1" t="inlineStr"/>
+      <c r="L11" s="1" t="inlineStr"/>
+      <c r="M11" s="1" t="inlineStr"/>
+      <c r="N11" s="1" t="inlineStr"/>
+      <c r="O11" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="P11" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="Q11" s="1" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+      <c r="R11" s="1" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+ZONA FRANCA DE MANAUS (ZFM) - Para os regimes cumulativo e não cumulativo, ficam reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas de vendas de mercadorias destinadas ao consumo (utilizadas diretamente ou para comercialização por atacado ou a varejo) ou à industrialização na Zona Franca de Manaus, por pessoa jurídica estabelecida fora da ZFM (Lei nº 10.996/2004, artigo 2º).
+Nas notas fiscais relativas à venda, deverá constar a expressão "Venda de mercadoria efetuada com alíquota zero da Contribuição para o PIS/Pasep e da COFINS - Lei nº 10.996/2004, artigo 2º".
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, terão a alíquota do PIS e da COFINS reduzidas a zero, exceto nas vendas de mercadorias que tenham como destinatárias pessoas jurídicas atacadistas e varejistas, sujeitas ao regime de apuração não cumulativa do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, §§ 3º e 4º). As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+MATÉRIAS-PRIMAS, PRODUTOS INTERMEDIÁRIOS E MATERIAIS DE EMBALAGEM - São reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas decorrentes da comercialização de matérias-primas, produtos intermediários e materiais de embalagem, produzidos na Zona Franca de Manaus para emprego em processo de industrialização por estabelecimentos industriais dos regimes cumulativo ou não cumulativo ali instalados, consoante projetos aprovados pelo Conselho de Administração da Superintendência da Zona Franca de Manaus (SUFRAMA) (Lei nº 10.637/2002, artigo 5º-A).
+REGIME NÃO CUMULATIVO - As alíquotas especiais para vendas realizadas por pessoa jurídica optante pelo regime não cumulativo estabelecida na Zona Franca de Manaus estão dispostas abaixo do item "Solução de Consulta".</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
@@ -984,6 +1675,67 @@
           <t>Cum: Lei nº 9.715/98, artigo 8º, inciso I; Lei nº 9.718/98, artigo 8º | N.Cum: Lei nº 10.637/2002, artigo 2º; Lei nº 10.833/2003, artigo 2º</t>
         </is>
       </c>
+      <c r="J12" s="1" t="inlineStr">
+        <is>
+          <t>REGRA GERAL - O código NCM pesquisado não se encontra dentre os produtos com benefícios fiscais de PIS e COFINS previstos em legislação. Antes de aplicar as alíquotas correspondentes ao regime tributário da pessoa jurídica é recomendado analisar as outras guias.
+INCIDÊNCIA MONOFÁSICA - Caberá a aplicação da incidência monofásica para os produtos constantes dos Anexos I e II da Lei nº 10.485/2002, caso o produto seja destinado ao setor automotivo, conforme previsto Solução de Consulta Cosit nº 55/2018.
+O item 27 da referida solução de consulta, prevê que: Se pelas suas características, dimensões, finalidades, for possível evidenciar não ter aplicação no setor automotivo, deverão ser aplicadas as alíquotas gerais de acordo com a sistemática de tributação do vendedor, Lucro Real, Lucro Presumido ou Simples Nacional, haja vista não se subsumir às previsões da Lei nº 10.485/2002.
+Nesta concepção o setor automotivo engloba os veículos automotores terrestres (tais como carros, ônibus, caminhões, tratores, entre outros), motocicletas e as máquinas agrícolas autopropulsadas, não compreendendo na incidência monofásica, portanto, as autopeças constantes nos Anexos I e II destinadas à embarcações e aeronaves (Solução de Consulta Interna Cosit nº 01/2019; Solução de Consulta nº 4.005/2020, da 4ª Região Fiscal; Solução de Consulta COSIT nº 149/2018).
+O entendimento expresso na Solução de Consulta Cosit nº 55/2018 também é reforçado com a previsão do § 4º, do artigo 427 da IN nº 2.121/2022, incluído pela Instrução Normativa RFB nº 2.152/2023, que indica a aplicação das alíquotas de regra geral, em caso que os produtos dos Anexos I e II não sejam partes ou componentes das máquinas, dos veículos e dos implementos citados no artigo 1º da Lei nº 10.485/2002.
+Adicionalmente informamos que a Solução de Consulta Cosit e a Solução de Divergência, a partir da data de sua publicação, têm efeito vinculante no âmbito da RFB, respaldam o sujeito passivo que as aplicar, independentemente de ser o consulente, desde que se enquadre na hipótese por elas abrangida, sem prejuízo de que a autoridade fiscal, em procedimento de fiscalização, verifique seu efetivo enquadramento (IN RFB nº 2.058/2021, artigo 33, e artigo 39, § 2º).
+PRODUTOS USADOS - Os produtos usados não estão sujeitos a incidência monofásica do PIS e da COFINS (Lei nº 10.485/2002, artigo 6º).
+CONDIÇÃO DO ADQUIRENTE - Antes de aplicar a alíquota básica, é importante verificar se a pessoa jurídica adquirente é habilitada em algum regime especial, se está localizada na Zona Franca de Manaus (ZFM) ou em Área de Livre Comércio (ALC), e se a receita é proveniente de exportação de mercadorias.
+SIMPLES NACIONAL - A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+DARF - As empresas optantes pelo regime cumulativo recolherão o PIS e a COFINS em DARF, nos códigos 8109 e 2172, respectivamente.
+Para o regime não cumulativo os códigos serão 6912 e 5856.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
+      <c r="K12" s="1" t="inlineStr"/>
+      <c r="L12" s="1" t="inlineStr"/>
+      <c r="M12" s="1" t="inlineStr"/>
+      <c r="N12" s="1" t="inlineStr"/>
+      <c r="O12" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="P12" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="Q12" s="1" t="inlineStr">
+        <is>
+          <t>Lei nº 10.485/2002, artigos 1º e 3º</t>
+        </is>
+      </c>
+      <c r="R12" s="1" t="inlineStr">
+        <is>
+          <t>VENDA A MONTADORAS DE VEÍCULOS - Não se aplica a substituição tributária na venda de autopeças, pneus novos e câmaras de ar para montadoras de veículos. (Lei nº 11.196/2005, artigo 65, § 6º).
+Não haverá crédito de PIS e COFINS nas aquisições feitas pelas montadoras de veículos estabelecidas na ZFM, pela compra dos referidos produtos, mesmo sendo a título de insumo ou imobilizado (Lei nº 11.196/2005, artigo 65, § 6º).
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica estabelecida fora dessas áreas, terão o mesmo tratamento da substituição tributária prevista para fabricante ou importador estabelecido fora da Zona Franca de Manaus. Porém, a redução a zero e a respectiva substituição tributária não se aplicam às vendas para adquirente atacadista ou varejista sujeito ao regime não cumulativo situado nas ALC (Lei nº 11.196/2005, artigos 2º, § 4º.
+As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+TRIBUTAÇÃO - A tributação de produtos monofásicos destinados ao consumo ou industrialização a Pessoas Jurídicas localizadas na ZFM possuirá dois momentos: a contribuição própria do vendedor localizado fora da área incentivada (redução a zero conforme prevê a Lei nº 10.996/2004, artigo 2º) e a contribuição como sujeito passivo por substituição tributária (responsável tributário), recolhendo antecipadamente o PIS e a COFINS do contribuinte situado na ZFM onde aplicará alíquotas de acordo com a legislação pertinente ao produto (Lei nº 11.196/2005, artigos 64 e 65; ADI nº 4.254).
+PRODUTOS USADOS - Os produtos usados não estão sujeitos a incidência monofásica do PIS e da COFINS (Lei nº 10.485/2002, artigo 6º).
+ALÍQUOTAS - O fabricante ou importador dos produtos monofásicos citados no artigo 65 da Lei nº 11.196/2005 estabelecido fora da ZFM, fica obrigado a cobrar e recolher como substituto tributário o PIS e a COFINS devidos pela pessoa jurídica estabelecida na ZFM.
+Até 24.09.2020, as alíquotas eram de 2,30% (PIS) e de 10,80% (COFINS) nas vendas para comerciantes atacadistas, varejistas ou consumidores, ou de 1,65% (PIS) e 7,6% (COFINS) nas vendas a fabricantes de veículos e máquinas do artigo 1º da Lei nº 10.485/2002 ou para fabricantes de autopeças dos Anexos I e II da mesma lei. (Lei nº 11.196/2005, artigo 65, § 1º, inciso V e Lei nº 10.485/2002, artigo 3º, inciso II).
+A partir da vinculação da ADI nº 4.254, em 25.09.2020, o Supremo Tribunal Federal (STF) declarou a inconstitucionalidade das alíquotas majoradas citadas no artigo 65 da Lei nº 11.196/2005 e, em decorrência desse julgamento, o Ministro proferiu decisão determinando a aplicação das alíquotas gerais de 1,65% (PIS) e 7,6% (COFINS) para suprir a lacuna legislativa.
+Posteriormente, emitiu-se o Parecer SEI nº 298/2023 com vigência a partir de 30.03.2023, que concluiu pela inaplicabilidade legal das alíquotas estabelecidas pelo Ministro do STF e, determinou não ser possível a tributação sobre a revenda realizada pelas empresas situadas na ZFM, e consequentemente a substituição tributária pelo fabricante/importador, até que nova legislação fosse promulgada para fixar tais percentuais.
+Embora tenha sido publicada no DOU de 18.07.2023, a Instrução Normativa RFB nº 2.152/2023 consolidando no § 2º do artigo 545 e § 2º do artigo 551 da Instrução Normativa RFB nº 2.121/2022 a utilização das alíquotas de 1,65% (PIS) e 7,6% (COFINS), no mesmo sentido da ADI. Contudo, pela leitura do relatório complementar das Soluções de Consulta Cosit n° 271/2023 (item 20 do relatório) e nº 176/2024 (item 18 do relatório), a autoridade fiscal reconhece a necessidade de atualização do texto da Instrução Normativa para que ela seja adequada à redação do Parecer SEI nº 298/2023.
+Assim, interpreta-se que as alíquotas para o fabricante/importador na substituição tributária são:
+a) até 24.09.2020: 2,30% (PIS) e de 10,80% (COFINS) - nas vendas para comerciantes atacadistas, varejistas ou consumidores, ou de 1,65% (PIS) e 7,6% (COFINS) nas vendas a fabricantes de veículos e máquinas do artigo 1º da Lei nº 10.485/2002 ou para fabricantes de autopeças dos Anexos I e II da mesma lei. (Lei nº 11.196/2005, artigo 65, § 1º, inciso V);
+b) de 25.09.2020 em diante: inexistência de alíquotas para o importador/fabricante em decorrência de lacuna normativa, essa a ensejar, atualmente, a ausência de tributação na operação de revenda pela pessoa jurídica localizada na ZFM. ADI nº 4.254; Parecer SEI nº 298/2023; SC Cosit n° 271/2023 e nº 176/2024.
+DARF - As empresas optantes pelo regime cumulativo e não cumulativo recolherão o PIS e a COFINS em DARF, sobre as receitas de vendas à Zona Franca de Manaus (Substituição Tributária), nos códigos 1921 e 1840, respectivamente.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="30.75" customHeight="1">
       <c r="A13" s="1" t="n">
@@ -1029,6 +1781,58 @@
           <t>Cum: Lei nº 10.925/2004, artigo 1º, inciso XIX e § 4º | N.Cum: Lei nº 10.925/2004, artigo 1º, inciso XIX e § 4º</t>
         </is>
       </c>
+      <c r="J13" s="1" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+REGIME CUMULATIVO / NÃO CUMULATIVO - O produto está sujeito à alíquota zero do PIS e da COFINS sobre a receita decorrente da venda no mercado interno (Lei nº 10.925/2004, artigo 1º, inciso XIX e § 4º) .
+Também aplica-se a alíquota zero e sobre a receita bruta decorrente das saídas do estabelecimento industrial, na industrialização por conta e ordem de terceiros, dos bens e produtos classificados nas posições NCM 0103, 0105, 0203, 02.06.30.00, 0206.4, 0207 e 0210.1 (Lei nº 10.925/2004, artigo 1º, § 4º).</t>
+        </is>
+      </c>
+      <c r="K13" s="1" t="inlineStr"/>
+      <c r="L13" s="1" t="inlineStr"/>
+      <c r="M13" s="1" t="inlineStr"/>
+      <c r="N13" s="1" t="inlineStr"/>
+      <c r="O13" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="P13" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="Q13" s="1" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+      <c r="R13" s="1" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+ZONA FRANCA DE MANAUS (ZFM) - Para os regimes cumulativo e não cumulativo, ficam reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas de vendas de mercadorias destinadas ao consumo (utilizadas diretamente ou para comercialização por atacado ou a varejo) ou à industrialização na Zona Franca de Manaus, por pessoa jurídica estabelecida fora da ZFM (Lei nº 10.996/2004, artigo 2º).
+Nas notas fiscais relativas à venda, deverá constar a expressão "Venda de mercadoria efetuada com alíquota zero da Contribuição para o PIS/Pasep e da COFINS - Lei nº 10.996/2004, artigo 2º".
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, terão a alíquota do PIS e da COFINS reduzidas a zero, exceto nas vendas de mercadorias que tenham como destinatárias pessoas jurídicas atacadistas e varejistas, sujeitas ao regime de apuração não cumulativa do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, §§ 3º e 4º). As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+MATÉRIAS-PRIMAS, PRODUTOS INTERMEDIÁRIOS E MATERIAIS DE EMBALAGEM - São reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas decorrentes da comercialização de matérias-primas, produtos intermediários e materiais de embalagem, produzidos na Zona Franca de Manaus para emprego em processo de industrialização por estabelecimentos industriais dos regimes cumulativo ou não cumulativo ali instalados, consoante projetos aprovados pelo Conselho de Administração da Superintendência da Zona Franca de Manaus (SUFRAMA) (Lei nº 10.637/2002, artigo 5º-A).
+REGIME NÃO CUMULATIVO - As alíquotas especiais para vendas realizadas por pessoa jurídica optante pelo regime não cumulativo estabelecida na Zona Franca de Manaus estão dispostas abaixo do item "Solução de Consulta".</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
@@ -1074,6 +1878,60 @@
           <t>Cum: Lei nº 9.715/98, artigo 8º, inciso I; Lei nº 9.718/98, artigo 8º | N.Cum: Lei nº 10.637/2002, artigo 2º; Lei nº 10.833/2003, artigo 2º</t>
         </is>
       </c>
+      <c r="J14" s="1" t="inlineStr">
+        <is>
+          <t>REGRA GERAL - O código NCM pesquisado pode enquadrar-se dentre os produtos com benefícios fiscais de PIS e COFINS previstos em legislação. Antes de aplicar as alíquotas correspondentes ao regime tributário da pessoa jurídica é recomendado analisar as outras guias.
+CONDIÇÃO DO ADQUIRENTE - Antes de aplicar a alíquota básica, é importante verificar se a pessoa jurídica adquirente é habilitada em algum regime especial, se está localizada na Zona Franca de Manaus (ZFM) ou em Área de Livre Comércio (ALC), e se a receita é proveniente de exportação de mercadorias.
+SIMPLES NACIONAL - A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+DARF - As empresas optantes pelo regime cumulativo recolherão o PIS e a COFINS em DARF, nos códigos 8109 e 2172, respectivamente.
+Para o regime não cumulativo os códigos serão 6912 e 5856.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
+      <c r="K14" s="1" t="inlineStr"/>
+      <c r="L14" s="1" t="inlineStr"/>
+      <c r="M14" s="1" t="inlineStr"/>
+      <c r="N14" s="1" t="inlineStr"/>
+      <c r="O14" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="P14" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="Q14" s="1" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+      <c r="R14" s="1" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+ZONA FRANCA DE MANAUS (ZFM) - Para os regimes cumulativo e não cumulativo, ficam reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas de vendas de mercadorias destinadas ao consumo (utilizadas diretamente ou para comercialização por atacado ou a varejo) ou à industrialização na Zona Franca de Manaus, por pessoa jurídica estabelecida fora da ZFM (Lei nº 10.996/2004, artigo 2º).
+Nas notas fiscais relativas à venda, deverá constar a expressão "Venda de mercadoria efetuada com alíquota zero da Contribuição para o PIS/Pasep e da COFINS - Lei nº 10.996/2004, artigo 2º".
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, terão a alíquota do PIS e da COFINS reduzidas a zero, exceto nas vendas de mercadorias que tenham como destinatárias pessoas jurídicas atacadistas e varejistas, sujeitas ao regime de apuração não cumulativa do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, §§ 3º e 4º). As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+MATÉRIAS-PRIMAS, PRODUTOS INTERMEDIÁRIOS E MATERIAIS DE EMBALAGEM - São reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas decorrentes da comercialização de matérias-primas, produtos intermediários e materiais de embalagem, produzidos na Zona Franca de Manaus para emprego em processo de industrialização por estabelecimentos industriais dos regimes cumulativo ou não cumulativo ali instalados, consoante projetos aprovados pelo Conselho de Administração da Superintendência da Zona Franca de Manaus (SUFRAMA) (Lei nº 10.637/2002, artigo 5º-A).
+REGIME NÃO CUMULATIVO - As alíquotas especiais para vendas realizadas por pessoa jurídica optante pelo regime não cumulativo estabelecida na Zona Franca de Manaus estão dispostas abaixo do item "Solução de Consulta".</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -1119,6 +1977,60 @@
           <t>Cum: Lei nº 9.715/98, artigo 8º, inciso I; Lei nº 9.718/98, artigo 8º | N.Cum: Lei nº 10.637/2002, artigo 2º; Lei nº 10.833/2003, artigo 2º</t>
         </is>
       </c>
+      <c r="J15" s="1" t="inlineStr">
+        <is>
+          <t>REGRA GERAL - O código NCM pesquisado não se encontra dentre os produtos com benefícios fiscais de PIS e COFINS previstos em legislação. Antes de aplicar as alíquotas correspondentes ao regime tributário da pessoa jurídica é recomendado analisar as outras guias.
+CONDIÇÃO DO ADQUIRENTE - Antes de aplicar a alíquota básica, é importante verificar se a pessoa jurídica adquirente é habilitada em algum regime especial, se está localizada na Zona Franca de Manaus (ZFM) ou em Área de Livre Comércio (ALC), e se a receita é proveniente de exportação de mercadorias.
+SIMPLES NACIONAL - A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+DARF - As empresas optantes pelo regime cumulativo recolherão o PIS e a COFINS em DARF, nos códigos 8109 e 2172, respectivamente.
+Para o regime não cumulativo os códigos serão 6912 e 5856.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
+      <c r="K15" s="1" t="inlineStr"/>
+      <c r="L15" s="1" t="inlineStr"/>
+      <c r="M15" s="1" t="inlineStr"/>
+      <c r="N15" s="1" t="inlineStr"/>
+      <c r="O15" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="P15" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="Q15" s="1" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+      <c r="R15" s="1" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+ZONA FRANCA DE MANAUS (ZFM) - Para os regimes cumulativo e não cumulativo, ficam reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas de vendas de mercadorias destinadas ao consumo (utilizadas diretamente ou para comercialização por atacado ou a varejo) ou à industrialização na Zona Franca de Manaus, por pessoa jurídica estabelecida fora da ZFM (Lei nº 10.996/2004, artigo 2º).
+Nas notas fiscais relativas à venda, deverá constar a expressão "Venda de mercadoria efetuada com alíquota zero da Contribuição para o PIS/Pasep e da COFINS - Lei nº 10.996/2004, artigo 2º".
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, terão a alíquota do PIS e da COFINS reduzidas a zero, exceto nas vendas de mercadorias que tenham como destinatárias pessoas jurídicas atacadistas e varejistas, sujeitas ao regime de apuração não cumulativa do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, §§ 3º e 4º). As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+MATÉRIAS-PRIMAS, PRODUTOS INTERMEDIÁRIOS E MATERIAIS DE EMBALAGEM - São reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas decorrentes da comercialização de matérias-primas, produtos intermediários e materiais de embalagem, produzidos na Zona Franca de Manaus para emprego em processo de industrialização por estabelecimentos industriais dos regimes cumulativo ou não cumulativo ali instalados, consoante projetos aprovados pelo Conselho de Administração da Superintendência da Zona Franca de Manaus (SUFRAMA) (Lei nº 10.637/2002, artigo 5º-A).
+REGIME NÃO CUMULATIVO - As alíquotas especiais para vendas realizadas por pessoa jurídica optante pelo regime não cumulativo estabelecida na Zona Franca de Manaus estão dispostas abaixo do item "Solução de Consulta".</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
@@ -1164,6 +2076,60 @@
           <t>Cum: Lei nº 9.715/98, artigo 8º, inciso I; Lei nº 9.718/98, artigo 8º | N.Cum: Lei nº 10.637/2002, artigo 2º; Lei nº 10.833/2003, artigo 2º</t>
         </is>
       </c>
+      <c r="J16" s="1" t="inlineStr">
+        <is>
+          <t>REGRA GERAL - O código NCM pesquisado pode enquadrar-se dentre os produtos com benefícios fiscais de PIS e COFINS previstos em legislação. Antes de aplicar as alíquotas correspondentes ao regime tributário da pessoa jurídica é recomendado analisar as outras guias.
+CONDIÇÃO DO ADQUIRENTE - Antes de aplicar a alíquota básica, é importante verificar se a pessoa jurídica adquirente é habilitada em algum regime especial, se está localizada na Zona Franca de Manaus (ZFM) ou em Área de Livre Comércio (ALC), e se a receita é proveniente de exportação de mercadorias.
+SIMPLES NACIONAL - A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+DARF - As empresas optantes pelo regime cumulativo recolherão o PIS e a COFINS em DARF, nos códigos 8109 e 2172, respectivamente.
+Para o regime não cumulativo os códigos serão 6912 e 5856.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
+      <c r="K16" s="1" t="inlineStr"/>
+      <c r="L16" s="1" t="inlineStr"/>
+      <c r="M16" s="1" t="inlineStr"/>
+      <c r="N16" s="1" t="inlineStr"/>
+      <c r="O16" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="P16" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="Q16" s="1" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+      <c r="R16" s="1" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+ZONA FRANCA DE MANAUS (ZFM) - Para os regimes cumulativo e não cumulativo, ficam reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas de vendas de mercadorias destinadas ao consumo (utilizadas diretamente ou para comercialização por atacado ou a varejo) ou à industrialização na Zona Franca de Manaus, por pessoa jurídica estabelecida fora da ZFM (Lei nº 10.996/2004, artigo 2º).
+Nas notas fiscais relativas à venda, deverá constar a expressão "Venda de mercadoria efetuada com alíquota zero da Contribuição para o PIS/Pasep e da COFINS - Lei nº 10.996/2004, artigo 2º".
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, terão a alíquota do PIS e da COFINS reduzidas a zero, exceto nas vendas de mercadorias que tenham como destinatárias pessoas jurídicas atacadistas e varejistas, sujeitas ao regime de apuração não cumulativa do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, §§ 3º e 4º). As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+MATÉRIAS-PRIMAS, PRODUTOS INTERMEDIÁRIOS E MATERIAIS DE EMBALAGEM - São reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas decorrentes da comercialização de matérias-primas, produtos intermediários e materiais de embalagem, produzidos na Zona Franca de Manaus para emprego em processo de industrialização por estabelecimentos industriais dos regimes cumulativo ou não cumulativo ali instalados, consoante projetos aprovados pelo Conselho de Administração da Superintendência da Zona Franca de Manaus (SUFRAMA) (Lei nº 10.637/2002, artigo 5º-A).
+REGIME NÃO CUMULATIVO - As alíquotas especiais para vendas realizadas por pessoa jurídica optante pelo regime não cumulativo estabelecida na Zona Franca de Manaus estão dispostas abaixo do item "Solução de Consulta".</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
@@ -1209,6 +2175,87 @@
           <t>Cum: Lei nº 9.715/98, artigo 8º, inciso I; Lei nº 9.718/98, artigo 8º | N.Cum: Lei nº 10.637/2002, artigo 2º; Lei nº 10.833/2003, artigo 2º</t>
         </is>
       </c>
+      <c r="J17" s="1" t="inlineStr">
+        <is>
+          <t>REGRA GERAL - O código NCM pesquisado pode enquadrar-se dentre os produtos com benefícios fiscais de PIS e COFINS previstos em legislação. Antes de aplicar as alíquotas correspondentes ao regime tributário da pessoa jurídica é recomendado analisar as outras guias.
+CONDIÇÃO DO ADQUIRENTE - Antes de aplicar a alíquota básica, é importante verificar se a pessoa jurídica adquirente é habilitada em algum regime especial, se está localizada na Zona Franca de Manaus (ZFM) ou em Área de Livre Comércio (ALC), e se a receita é proveniente de exportação de mercadorias.
+SIMPLES NACIONAL - A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+DARF - As empresas optantes pelo regime cumulativo recolherão o PIS e a COFINS em DARF, nos códigos 8109 e 2172, respectivamente.
+Para o regime não cumulativo os códigos serão 6912 e 5856.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
+      <c r="K17" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="L17" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="M17" s="1" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+      <c r="N17" s="1" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da suspensão do PIS e da COFINS sobre as receitas de vendas de mercadorias, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+REGIME CUMULATIVO / NÃO CUMULATIVO - Aplica-se a suspensão do PIS e da COFINS nos casos de venda realizada a pessoa jurídica inscrita no Regime Especial de Tributação para Desenvolvimento da Atividade de Exibição Cinematográfica (RECINE) (Lei nº 12.599/2012, artigos 12 a 15; Decreto nº 7.729/2012).
+Prazo de vigência do benefício do RECINE: Até 31.12.2029 (Lei nº 13.594/2018).
+A partir de 01.04.2026, os incentivos e benefícios federais de natureza tributária são reduzidos, sendo aqueles de alíquota zero mediante a aplicação de alíquota correspondente a 10% da alíquota do sistema padrão de tributação. Desta forma, tendo em vista que para o PIS e a Cofins existem dois regimes de tributação, as alíquotas devem corresponder a 10% das alíquotas padrão de cada um dos regimes:
+a) Regime cumulativo - PIS: 0,065%; Cofins: 0,3%;
+b) Regime não cumulativo - PIS: 0,165%; Cofins: 0,76%. (Lei Complementar nº 224/2025, artigo 4º, caput e § 4º, inciso I)
+Ressalta-se que o § 1°, do artigo 2°, da IN RFB n° 2.305/2025 limita a redução dos benefícios àqueles discriminados no demonstrativo de gastos tributários anexo à Lei Orçamentária Anual de 2026. O Recine está discriminado, sofrendo redução do benefício.
+Quanto à aplicação da redução dos benefícios, no caso da suspensão, o artigo 6°, da IN RFB n° 2.305/2025 estabelece que a redução não se aplica aos benefícios de suspensão em que se verifique apenas um diferimento temporal no recolhimento do tributo. Logo, tendo em vista que o inciso II, do § 3°, do artigo 14, da Lei n° 12.599/2012 estabelece que a suspensão do PIS/Cofins converte-se em alíquota zero após a incorporação do bem ou material de construção no ativo imobilizado ou sua utilização no complexo de exibição cinematográfica ou cinema itinerante, situação na qual a operação fica sujeita à redução do benefício disposto na Lei Complementar nº 224/2025.
+Preventivamente, a sugestão é de que no cálculo para demonstrar o aumento da carga deve ser aplicado 10% das alíquotas do sistema padrão de PIS/Cofins sobre as vendas ou importação, baseado no artigo 7° da IN RFB 2.305/2025. Tal sugestão é um entendimento que poderá ser confirmado ou reformulado mediante esclarecimento da RFB.
+Visto que essas informações não estão claras na legislação, recomenda-se ao contribuinte buscar o serviço do Receita Soluciona, por meio das Confederações Nacionais de Representação de Categorias Econômicas, às Centrais Sindicais, aos Órgãos de Registro de Classe com atuação nacional e Organizações Associativas Patronais e Empresarias.</t>
+        </is>
+      </c>
+      <c r="O17" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="P17" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="Q17" s="1" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+      <c r="R17" s="1" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+ZONA FRANCA DE MANAUS (ZFM) - Para os regimes cumulativo e não cumulativo, ficam reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas de vendas de mercadorias destinadas ao consumo (utilizadas diretamente ou para comercialização por atacado ou a varejo) ou à industrialização na Zona Franca de Manaus, por pessoa jurídica estabelecida fora da ZFM (Lei nº 10.996/2004, artigo 2º).
+Nas notas fiscais relativas à venda, deverá constar a expressão "Venda de mercadoria efetuada com alíquota zero da Contribuição para o PIS/Pasep e da COFINS - Lei nº 10.996/2004, artigo 2º".
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, terão a alíquota do PIS e da COFINS reduzidas a zero, exceto nas vendas de mercadorias que tenham como destinatárias pessoas jurídicas atacadistas e varejistas, sujeitas ao regime de apuração não cumulativa do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, §§ 3º e 4º). As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+MATÉRIAS-PRIMAS, PRODUTOS INTERMEDIÁRIOS E MATERIAIS DE EMBALAGEM - São reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas decorrentes da comercialização de matérias-primas, produtos intermediários e materiais de embalagem, produzidos na Zona Franca de Manaus para emprego em processo de industrialização por estabelecimentos industriais dos regimes cumulativo ou não cumulativo ali instalados, consoante projetos aprovados pelo Conselho de Administração da Superintendência da Zona Franca de Manaus (SUFRAMA) (Lei nº 10.637/2002, artigo 5º-A).
+REGIME NÃO CUMULATIVO - As alíquotas especiais para vendas realizadas por pessoa jurídica optante pelo regime não cumulativo estabelecida na Zona Franca de Manaus estão dispostas abaixo do item "Solução de Consulta".</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
@@ -1254,6 +2301,89 @@
           <t>Cum: Lei nº 9.715/98, artigo 8º, inciso I; Lei nº 9.718/98, artigo 8º | N.Cum: Lei nº 10.637/2002, artigo 2º; Lei nº 10.833/2003, artigo 2º</t>
         </is>
       </c>
+      <c r="J18" s="1" t="inlineStr">
+        <is>
+          <t>REGRA GERAL - O código NCM pesquisado pode enquadrar-se dentre os produtos com benefícios fiscais de PIS e COFINS previstos em legislação. Antes de aplicar as alíquotas correspondentes ao regime tributário da pessoa jurídica é recomendado analisar as outras guias.
+CONDIÇÃO DO ADQUIRENTE - Antes de aplicar a alíquota básica, é importante verificar se a pessoa jurídica adquirente é habilitada em algum regime especial, se está localizada na Zona Franca de Manaus (ZFM) ou em Área de Livre Comércio (ALC), e se a receita é proveniente de exportação de mercadorias.
+SIMPLES NACIONAL - A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+DARF - As empresas optantes pelo regime cumulativo recolherão o PIS e a COFINS em DARF, nos códigos 8109 e 2172, respectivamente.
+Para o regime não cumulativo os códigos serão 6912 e 5856.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
+      <c r="K18" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="L18" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="M18" s="1" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+      <c r="N18" s="1" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da suspensão do PIS e da COFINS sobre as receitas de vendas de mercadorias, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+REGIME CUMULATIVO / NÃO CUMULATIVO - Aplica-se a suspensão do PIS e da COFINS nos casos de venda realizada a pessoa jurídica inscrita no Regime Especial de Tributação para Desenvolvimento da Atividade de Exibição Cinematográfica (RECINE) (Lei nº 12.599/2012, artigos 12 a 15; Decreto nº 7.729/2012).
+Prazo de vigência do benefício do RECINE: Até 31.12.2029 (Lei nº 13.594/2018).
+Também se aplica a suspensão no caso de venda de bens novos, destinados ao desenvolvimento, no País, de software e de serviços de tecnologia da informação, quando os referidos bens forem adquiridos por pessoa jurídica beneficiária do Regime Especial de Tributação para a Plataforma de Exportação de Serviços de Tecnologia da Informação (REPES) para incorporação ao seu ativo imobilizado (Lei nº 11.196/2005, artigos 4º e 11; Decreto nº 5.713/2006, artigo 1º).
+A partir de 01.04.2026, os incentivos e benefícios federais de natureza tributária são reduzidos, sendo aqueles de alíquota zero mediante a aplicação de alíquota correspondente a 10% da alíquota do sistema padrão de tributação. Desta forma, tendo em vista que para o PIS e a Cofins existem dois regimes de tributação, as alíquotas devem corresponder a 10% das alíquotas padrão de cada um dos regimes:
+a) Regime cumulativo - PIS: 0,065%; Cofins: 0,3%;
+b) Regime não cumulativo - PIS: 0,165%; Cofins: 0,76%. (Lei Complementar nº 224/2025, artigo 4º, caput e § 4º, inciso I)
+Ressalta-se que o § 1°, do artigo 2°, da IN RFB n° 2.305/2025 limita a redução dos benefícios àqueles discriminados no demonstrativo de gastos tributários anexo à Lei Orçamentária Anual de 2026. O Recine está discriminado, sofrendo redução do benefício.
+O Repes não está discriminado no demonstrativo de gastos tributários, não se sujeitando à redução estabelecida na Lei Complementar nº 224/2025.
+Quanto à aplicação da redução dos benefícios, no caso da suspensão, o artigo 6°, da IN RFB n° 2.305/2025 estabelece que a redução não se aplica aos benefícios de suspensão em que se verifique apenas um diferimento temporal no recolhimento do tributo. Logo, tendo em vista que o inciso II, do § 3°, do artigo 14, da Lei n° 12.599/2012 estabelece que a suspensão do PIS/Cofins converte-se em alíquota zero após a incorporação do bem ou material de construção no ativo imobilizado ou sua utilização no complexo de exibição cinematográfica ou cinema itinerante, situação na qual a operação fica sujeita à redução do benefício disposto na Lei Complementar nº 224/2025.
+Preventivamente, a sugestão é de que no cálculo para demonstrar o aumento da carga deve ser aplicado 10% das alíquotas do sistema padrão de PIS/Cofins sobre as vendas ou importação, baseado no artigo 7° da IN RFB 2.305/2025. Tal sugestão é um entendimento que poderá ser confirmado ou reformulado mediante esclarecimento da RFB.
+Visto que essas informações não estão claras na legislação, recomenda-se ao contribuinte buscar o serviço do Receita Soluciona, por meio das Confederações Nacionais de Representação de Categorias Econômicas, às Centrais Sindicais, aos Órgãos de Registro de Classe com atuação nacional e Organizações Associativas Patronais e Empresarias.</t>
+        </is>
+      </c>
+      <c r="O18" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="P18" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="Q18" s="1" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+      <c r="R18" s="1" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+ZONA FRANCA DE MANAUS (ZFM) - Para os regimes cumulativo e não cumulativo, ficam reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas de vendas de mercadorias destinadas ao consumo (utilizadas diretamente ou para comercialização por atacado ou a varejo) ou à industrialização na Zona Franca de Manaus, por pessoa jurídica estabelecida fora da ZFM (Lei nº 10.996/2004, artigo 2º).
+Nas notas fiscais relativas à venda, deverá constar a expressão "Venda de mercadoria efetuada com alíquota zero da Contribuição para o PIS/Pasep e da COFINS - Lei nº 10.996/2004, artigo 2º".
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, terão a alíquota do PIS e da COFINS reduzidas a zero, exceto nas vendas de mercadorias que tenham como destinatárias pessoas jurídicas atacadistas e varejistas, sujeitas ao regime de apuração não cumulativa do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, §§ 3º e 4º). As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+MATÉRIAS-PRIMAS, PRODUTOS INTERMEDIÁRIOS E MATERIAIS DE EMBALAGEM - São reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas decorrentes da comercialização de matérias-primas, produtos intermediários e materiais de embalagem, produzidos na Zona Franca de Manaus para emprego em processo de industrialização por estabelecimentos industriais dos regimes cumulativo ou não cumulativo ali instalados, consoante projetos aprovados pelo Conselho de Administração da Superintendência da Zona Franca de Manaus (SUFRAMA) (Lei nº 10.637/2002, artigo 5º-A).
+REGIME NÃO CUMULATIVO - As alíquotas especiais para vendas realizadas por pessoa jurídica optante pelo regime não cumulativo estabelecida na Zona Franca de Manaus estão dispostas abaixo do item "Solução de Consulta".</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
@@ -1297,6 +2427,67 @@
       <c r="I19" s="1" t="inlineStr">
         <is>
           <t>Cum: Lei nº 10.925/2004, artigo 1º, inciso XI | N.Cum: Lei nº 10.925/2004, artigo 1º, inciso XI</t>
+        </is>
+      </c>
+      <c r="J19" s="1" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+REGIME CUMULATIVO / NÃO CUMULATIVO - Aplica-se a alíquota zero do PIS e da COFINS à venda, no mercado interno, de (Lei nº 10.925/2004, artigo 1º, inciso XI):
+a) leite fluido pasteurizado ou industrializado, na forma de ultrapasteurizado, destinados ao consumo humano ou utilizados na industrialização de produtos que se destinam ao consumo humano;
+b) leite em pó, integral, semidesnatado ou desnatado, destinados ao consumo humano ou utilizados na industrialização de produtos que se destinam ao consumo humano;
+c) leite fermentado, bebidas e compostos lácteos e fórmulas infantis, assim definidas conforme previsão legal específica das instruções normativas do Ministério da Agricultura, Pecuária e Abastecimento, destinados ao consumo humano ou utilizados na industrialização de produtos que se destinam ao consumo humano.
+O benefício é aplicável apenas ao leite extraído de vacas. Portanto, não se aplica o benefício ao leite de cabra e seus derivados. (Soluções de Consulta Cosit n° 265/2023 e n° 44/2025)
+As definições de leite fermentado, bebidas e compostos lácteos e fórmulas infantis estão contidas nos seguintes dispositivos legais:
+- Leite Fermentado (Instrução Normativa MAPA nº 46/2007, Anexo, item 2.1);
+- Bebidas Lácteas (Instrução Normativa MAPA nº 16/2005, Anexo, item 2.1.1);
+- Compostos Lácteos (Instrução Normativa MAPA nº 28/2007, Anexo, item 2.1.1);
+- Fórmulas Infantis (Lei nº 11.265/2006, artigo 3º, incisos XVIII a XXI).
+Conforme o Acórdão DRJ/SPO (Delegacia da Receita Federal do Brasil de Julgamento em São Paulo) nº 1664862, de 22.01.2015, a venda de leite condensado e creme de leite não se enquadra na hipótese de alíquota zero prevista no artigo 1º, inciso XI, da Lei nº 10.925/2004).</t>
+        </is>
+      </c>
+      <c r="K19" s="1" t="inlineStr"/>
+      <c r="L19" s="1" t="inlineStr"/>
+      <c r="M19" s="1" t="inlineStr"/>
+      <c r="N19" s="1" t="inlineStr"/>
+      <c r="O19" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="P19" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="Q19" s="1" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+      <c r="R19" s="1" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+ZONA FRANCA DE MANAUS (ZFM) - Para os regimes cumulativo e não cumulativo, ficam reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas de vendas de mercadorias destinadas ao consumo (utilizadas diretamente ou para comercialização por atacado ou a varejo) ou à industrialização na Zona Franca de Manaus, por pessoa jurídica estabelecida fora da ZFM (Lei nº 10.996/2004, artigo 2º).
+Nas notas fiscais relativas à venda, deverá constar a expressão "Venda de mercadoria efetuada com alíquota zero da Contribuição para o PIS/Pasep e da COFINS - Lei nº 10.996/2004, artigo 2º".
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, terão a alíquota do PIS e da COFINS reduzidas a zero, exceto nas vendas de mercadorias que tenham como destinatárias pessoas jurídicas atacadistas e varejistas, sujeitas ao regime de apuração não cumulativa do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, §§ 3º e 4º). As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+MATÉRIAS-PRIMAS, PRODUTOS INTERMEDIÁRIOS E MATERIAIS DE EMBALAGEM - São reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas decorrentes da comercialização de matérias-primas, produtos intermediários e materiais de embalagem, produzidos na Zona Franca de Manaus para emprego em processo de industrialização por estabelecimentos industriais dos regimes cumulativo ou não cumulativo ali instalados, consoante projetos aprovados pelo Conselho de Administração da Superintendência da Zona Franca de Manaus (SUFRAMA) (Lei nº 10.637/2002, artigo 5º-A).
+REGIME NÃO CUMULATIVO - As alíquotas especiais para vendas realizadas por pessoa jurídica optante pelo regime não cumulativo estabelecida na Zona Franca de Manaus estão dispostas abaixo do item "Solução de Consulta".</t>
         </is>
       </c>
     </row>
@@ -1314,7 +2505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2420,6 +3611,3621 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>8471.41.90</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Observações (Regra Geral)</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>ALTERAÇÃO NA NCM - A reclassificação dos códigos NCM promovida pelo Decreto nº 11.158/2022 não faz com que o produto sofra alteração de tributação prevista na legislação mencionada anteriormente.
+Desta forma, a definição da NCM deverá seguir o disposto no artigo 16 do RIPI (Decreto nº 7.212/2010). Para verificar se houve reclassificação utilize a ferramenta Correlação da NCM.
+REGRA GERAL - O código NCM pesquisado não se encontra dentre os produtos com benefícios fiscais de PIS e COFINS previstos em legislação. Antes de aplicar as alíquotas correspondentes ao regime tributário da pessoa jurídica é recomendado analisar as outras guias.
+CONDIÇÃO DO ADQUIRENTE - Antes de aplicar a alíquota básica, é importante verificar se a pessoa jurídica adquirente é habilitada em algum regime especial, se está localizada na Zona Franca de Manaus (ZFM) ou em Área de Livre Comércio (ALC), e se a receita é proveniente de exportação de mercadorias.
+SIMPLES NACIONAL - A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+DARF - As empresas optantes pelo regime cumulativo recolherão o PIS e a COFINS em DARF, nos códigos 8109 e 2172, respectivamente.
+Para o regime não cumulativo os códigos serão 6912 e 5856.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>8471.41.90</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Suspensão - PIS</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>8471.41.90</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Suspensão - COFINS</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>8471.41.90</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Suspensão - Legislação</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>8471.41.90</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Suspensão - Observações</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>ALTERAÇÃO NA NCM - A reclassificação dos códigos NCM promovida pelo Decreto nº 11.158/2022 não faz com que o produto sofra alteração de tributação prevista na legislação mencionada anteriormente.
+Desta forma, a definição da NCM deverá seguir o disposto no artigo 16 do RIPI (Decreto nº 7.212/2010). Para verificar se houve reclassificação utilize a ferramenta Correlação da NCM.
+SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da suspensão do PIS e da COFINS sobre as receitas de vendas de mercadorias, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+REGIME CUMULATIVO / NÃO CUMULATIVO - Aplica-se a suspensão do PIS e da COFINS:
+a) na venda realizada para pessoa jurídica beneficiária do Regime Especial de Aquisição de bens de Capital para Empresas Exportadoras (RECAP), para incorporação ao seu ativo imobilizado (Lei nº 11.196/2005, artigo 12; Decreto nº 5.789/2006);
+b) na venda para pessoa jurídica beneficiária do RECAP, sobre os bens adquiridos ou importados por estaleiro naval brasileiro (Lei nº 11.196/2005, artigo 13, § 3º, inciso II; Decreto nº 5.788/2006). Essa suspensão aplica-se somente quando os referidos bens forem destinados às atividades de construção, conservação, modernização, conversão e reparo de embarcações pré-registradas ou registradas no Registro Especial Brasileiro (REB), instituído pela Lei nº 9.432/97;
+c) na venda realizada a pessoa jurídica inscrita no Regime Especial de Tributação para Desenvolvimento da Atividade de Exibição Cinematográfica (RECINE) (Lei nº 12.599/2012, artigos 12 a 15; Decreto nº 7.729/2012).
+Prazo de vigência do benefício do RECINE: Até 31.12.2029 (Lei nº 13.594/2018);
+d) na venda de bens novos, destinados ao desenvolvimento, no País, de software e de serviços de tecnologia da informação, quando os referidos bens forem adquiridos por pessoa jurídica beneficiária do Regime Especial de Tributação para a Plataforma de Exportação de Serviços de Tecnologia da Informação (REPES) para incorporação ao seu ativo imobilizado (Lei nº 11.196/2005, artigos 4º e 11; Decreto nº 5.713/2006, artigo 1º).
+A partir de 01.04.2026, os incentivos e benefícios federais de natureza tributária são reduzidos, sendo aqueles de alíquota zero mediante a aplicação de alíquota correspondente a 10% da alíquota do sistema padrão de tributação. Desta forma, tendo em vista que para o PIS e a Cofins existem dois regimes de tributação, as alíquotas devem corresponder a 10% das alíquotas padrão de cada um dos regimes:
+a) Regime cumulativo - PIS: 0,065%; Cofins: 0,3%;
+b) Regime não cumulativo - PIS: 0,165%; Cofins: 0,76%. (Lei Complementar nº 224/2025, artigo 4º, caput e § 4º, inciso I)
+Ressalta-se que o § 1°, do artigo 2°, da IN RFB n° 2.305/2025 limita a redução dos benefícios àqueles discriminados no demonstrativo de gastos tributários anexo à Lei Orçamentária Anual de 2026. O Recine está discriminado, sofrendo redução do benefício.
+O Recap e o Repes não estão discriminados no demonstrativo de gastos tributários, não se sujeitando à redução estabelecida na Lei Complementar nº 224/2025.
+Quanto à aplicação da redução dos benefícios, no caso da suspensão, o artigo 6°, da IN RFB n° 2.305/2025 estabelece que a redução não se aplica aos benefícios de suspensão em que se verifique apenas um diferimento temporal no recolhimento do tributo. Logo, tendo em vista que o inciso II, do § 3°, do artigo 14, da Lei n° 12.599/2012 estabelece que a suspensão do PIS/Cofins converte-se em alíquota zero após a incorporação do bem ou material de construção no ativo imobilizado ou sua utilização no complexo de exibição cinematográfica ou cinema itinerante, situação na qual a operação fica sujeita à redução do benefício disposto na Lei Complementar nº 224/2025.
+Preventivamente, a sugestão é de que no cálculo para demonstrar o aumento da carga deve ser aplicado 10% das alíquotas do sistema padrão de PIS/Cofins sobre as vendas ou importação, baseado no artigo 7° da IN RFB 2.305/2025. Tal sugestão é um entendimento que poderá ser confirmado ou reformulado mediante esclarecimento da RFB.
+Visto que essas informações não estão claras na legislação, recomenda-se ao contribuinte buscar o serviço do Receita Soluciona, por meio das Confederações Nacionais de Representação de Categorias Econômicas, às Centrais Sindicais, aos Órgãos de Registro de Classe com atuação nacional e Organizações Associativas Patronais e Empresarias.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>8471.41.90</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>ZFM - PIS</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>8471.41.90</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>8471.41.90</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>ZFM - Legislação</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>8471.41.90</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>ZFM - Observações</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+ZONA FRANCA DE MANAUS (ZFM) - Para os regimes cumulativo e não cumulativo, ficam reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas de vendas de mercadorias destinadas ao consumo (utilizadas diretamente ou para comercialização por atacado ou a varejo) ou à industrialização na Zona Franca de Manaus, por pessoa jurídica estabelecida fora da ZFM (Lei nº 10.996/2004, artigo 2º).
+Nas notas fiscais relativas à venda, deverá constar a expressão "Venda de mercadoria efetuada com alíquota zero da Contribuição para o PIS/Pasep e da COFINS - Lei nº 10.996/2004, artigo 2º".
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, terão a alíquota do PIS e da COFINS reduzidas a zero, exceto nas vendas de mercadorias que tenham como destinatárias pessoas jurídicas atacadistas e varejistas, sujeitas ao regime de apuração não cumulativa do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, §§ 3º e 4º). As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+MATÉRIAS-PRIMAS, PRODUTOS INTERMEDIÁRIOS E MATERIAIS DE EMBALAGEM - São reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas decorrentes da comercialização de matérias-primas, produtos intermediários e materiais de embalagem, produzidos na Zona Franca de Manaus para emprego em processo de industrialização por estabelecimentos industriais dos regimes cumulativo ou não cumulativo ali instalados, consoante projetos aprovados pelo Conselho de Administração da Superintendência da Zona Franca de Manaus (SUFRAMA) (Lei nº 10.637/2002, artigo 5º-A).
+REGIME NÃO CUMULATIVO - As alíquotas especiais para vendas realizadas por pessoa jurídica optante pelo regime não cumulativo estabelecida na Zona Franca de Manaus estão dispostas abaixo do item "Solução de Consulta".</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>3926.90.90</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Observações (Regra Geral)</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>REGRA GERAL - O código NCM pesquisado pode enquadrar-se dentre os produtos com benefícios fiscais de PIS e COFINS previstos em legislação. Antes de aplicar as alíquotas correspondentes ao regime tributário da pessoa jurídica é recomendado analisar as outras guias.
+CONDIÇÃO DO ADQUIRENTE - Antes de aplicar a alíquota básica, é importante verificar se a pessoa jurídica adquirente é habilitada em algum regime especial, se está localizada na Zona Franca de Manaus (ZFM) ou em Área de Livre Comércio (ALC), e se a receita é proveniente de exportação de mercadorias.
+SIMPLES NACIONAL - A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+DARF - As empresas optantes pelo regime cumulativo recolherão o PIS e a COFINS em DARF, nos códigos 8109 e 2172, respectivamente.
+Para o regime não cumulativo os códigos serão 6912 e 5856.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>3926.90.90</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>ZFM - PIS</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>3926.90.90</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>3926.90.90</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>ZFM - Legislação</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>3926.90.90</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>ZFM - Observações</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+ZONA FRANCA DE MANAUS (ZFM) - Para os regimes cumulativo e não cumulativo, ficam reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas de vendas de mercadorias destinadas ao consumo (utilizadas diretamente ou para comercialização por atacado ou a varejo) ou à industrialização na Zona Franca de Manaus, por pessoa jurídica estabelecida fora da ZFM (Lei nº 10.996/2004, artigo 2º).
+Nas notas fiscais relativas à venda, deverá constar a expressão "Venda de mercadoria efetuada com alíquota zero da Contribuição para o PIS/Pasep e da COFINS - Lei nº 10.996/2004, artigo 2º".
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, terão a alíquota do PIS e da COFINS reduzidas a zero, exceto nas vendas de mercadorias que tenham como destinatárias pessoas jurídicas atacadistas e varejistas, sujeitas ao regime de apuração não cumulativa do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, §§ 3º e 4º). As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+MATÉRIAS-PRIMAS, PRODUTOS INTERMEDIÁRIOS E MATERIAIS DE EMBALAGEM - São reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas decorrentes da comercialização de matérias-primas, produtos intermediários e materiais de embalagem, produzidos na Zona Franca de Manaus para emprego em processo de industrialização por estabelecimentos industriais dos regimes cumulativo ou não cumulativo ali instalados, consoante projetos aprovados pelo Conselho de Administração da Superintendência da Zona Franca de Manaus (SUFRAMA) (Lei nº 10.637/2002, artigo 5º-A).
+REGIME NÃO CUMULATIVO - As alíquotas especiais para vendas realizadas por pessoa jurídica optante pelo regime não cumulativo estabelecida na Zona Franca de Manaus estão dispostas abaixo do item "Solução de Consulta".</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>6109.10.00</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Observações (Regra Geral)</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>REGRA GERAL - O código NCM pesquisado não se encontra dentre os produtos com benefícios fiscais de PIS e COFINS previstos em legislação. Antes de aplicar as alíquotas correspondentes ao regime tributário da pessoa jurídica é recomendado analisar as outras guias.
+CONDIÇÃO DO ADQUIRENTE - Antes de aplicar a alíquota básica, é importante verificar se a pessoa jurídica adquirente é habilitada em algum regime especial, se está localizada na Zona Franca de Manaus (ZFM) ou em Área de Livre Comércio (ALC), e se a receita é proveniente de exportação de mercadorias.
+SIMPLES NACIONAL - A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+DARF - As empresas optantes pelo regime cumulativo recolherão o PIS e a COFINS em DARF, nos códigos 8109 e 2172, respectivamente.
+Para o regime não cumulativo os códigos serão 6912 e 5856.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>6109.10.00</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>ZFM - PIS</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>6109.10.00</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>6109.10.00</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>ZFM - Legislação</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>6109.10.00</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>ZFM - Observações</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+ZONA FRANCA DE MANAUS (ZFM) - Para os regimes cumulativo e não cumulativo, ficam reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas de vendas de mercadorias destinadas ao consumo (utilizadas diretamente ou para comercialização por atacado ou a varejo) ou à industrialização na Zona Franca de Manaus, por pessoa jurídica estabelecida fora da ZFM (Lei nº 10.996/2004, artigo 2º).
+Nas notas fiscais relativas à venda, deverá constar a expressão "Venda de mercadoria efetuada com alíquota zero da Contribuição para o PIS/Pasep e da COFINS - Lei nº 10.996/2004, artigo 2º".
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, terão a alíquota do PIS e da COFINS reduzidas a zero, exceto nas vendas de mercadorias que tenham como destinatárias pessoas jurídicas atacadistas e varejistas, sujeitas ao regime de apuração não cumulativa do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, §§ 3º e 4º). As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+MATÉRIAS-PRIMAS, PRODUTOS INTERMEDIÁRIOS E MATERIAIS DE EMBALAGEM - São reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas decorrentes da comercialização de matérias-primas, produtos intermediários e materiais de embalagem, produzidos na Zona Franca de Manaus para emprego em processo de industrialização por estabelecimentos industriais dos regimes cumulativo ou não cumulativo ali instalados, consoante projetos aprovados pelo Conselho de Administração da Superintendência da Zona Franca de Manaus (SUFRAMA) (Lei nº 10.637/2002, artigo 5º-A).
+REGIME NÃO CUMULATIVO - As alíquotas especiais para vendas realizadas por pessoa jurídica optante pelo regime não cumulativo estabelecida na Zona Franca de Manaus estão dispostas abaixo do item "Solução de Consulta".</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>8703.21.10</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Observações (Regra Geral)</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>CONCEITO DE INCIDÊNCIA MONOFÁSICA - O sistema de tributação monofásica é um tratamento tributário próprio e específico, previsto em relação ao PIS e a COFINS incidentes sobre a receita bruta decorrente da venda de determinados produtos, geralmente a fim de concentrar a tributação nas etapas de produção e importação, desonerando as etapas subsequentes de comercialização.
+A concentração da tributação ocorre com a aplicação de alíquotas maiores que as usualmente aplicadas na tributação das demais receitas.
+O álcool e as bebidas frias relacionadas no artigo 14 da Lei nº 13.097/2015 são exceções à regra, visto que o distribuidor também é responsável pelo recolhimento do PIS e da COFINS.
+SIMPLES NACIONAL - As leis que estabelecem a incidência monofásica não trazem dispensa no recolhimento da alíquota concentrada quando se trata de importador ou fabricante optante pelo Simples Nacional. Deste modo, o importador e o fabricante deverão proceder o recolhimento do PIS e da COFINS em DARF separado, mediante a aplicação das alíquotas diferenciadas previstas em legislação própria conforme o produto.
+Deve ser destacada a receita decorrente da venda desse produto, aplicando-se, sobre tal receita, a alíquota efetiva calculada com base no Anexo II da Lei Complementar nº 123/2006, mas sem considerar os percentuais destinados ao PIS e a COFINS.
+Para tanto, o importador e a indústria devem selecionar a atividade de "venda de mercadorias industrializadas, com substituição tributária/tributação monofásica", indicando a opção tributação monofásica em relação ao PIS e a COFINS, a fim de que o aplicativo desconsidere os percentuais desses tributos sobre a receita destacada, ou seja, o recolhimento não será realizado pelo DAS e sim em DARF separado (Lei Complementar nº 123/2006, artigo 18, § 4º-A, inciso I).
+Desde 01.01.2018, a atividade de produção e venda no atacado de bebidas alcoólicas não está vedada ao ingresso ao Simples Nacional, desde que praticada por:
+a) micro e pequenas cervejarias;
+b) micro e pequenas vinícolas;
+c) produtores de licores;
+d) micro e pequenas destilarias.
+As ME e EPP optantes pelo Simples Nacional deverão obrigatoriamente estar registradas no Ministério da Agricultura, Pecuária e Abastecimento e obedecerão também à regulamentação da Agência Nacional de Vigilância Sanitária e da Secretaria da Receita Federal do Brasil quanto à produção e à comercialização de bebidas alcoólicas (Lei Complementar nº 123/2006, artigo 17, § 5º).
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+REGIME CUMULATIVO / NÃO CUMULATIVO (IMPORTADOR OU INDÚSTRIA) - A receita bruta auferida por importador ou por indústria, optantes pelos regimes cumulativo ou não cumulativo, sujeita-se à incidência monofásica do PIS e da COFINS sobre os produtos constantes nos artigos 1º e 3º da Lei nº 10.485/2002.
+PRODUTOS USADOS - Os produtos usados não estão sujeitos a incidência monofásica do PIS e da COFINS (Lei nº 10.485/2002, artigo 6º).
+INDUSTRIALIZAÇÃO POR ENCOMENDA - Na industrialização por encomenda, exceto sobre os medicamentos relacionados no artigo 1º, inciso I, alíneas "a" e "b" da Lei nº 10.147/2000, o PIS e a COFINS incidirão sobre a receita auferida pela pessoa jurídica executora da encomenda às alíquotas de 1,65% (PIS) e 7,60% (COFINS), independentemente do regime de apuração a que está submetida a pessoa jurídica. O encomendante deve recolher o PIS e a COFINS mediante as alíquotas monofásicas (Lei nº 11.051/2004, artigo 10, § 2º e Lei nº 10.833/2003, artigo 25, inciso I).
+DARF - As empresas optantes pelo Simples Nacional recolherão o PIS e a COFINS em DARF, nos códigos 8109 e 2172, respectivamente (Lei nº 10.833/2003, artigo 10, inciso III).
+Para as empresas optantes pelo regime cumulativo, o recolhimento será nos códigos 8109 e 2172 e para as optantes pelo regime não cumulativo, será nos códigos 6912 e 5856.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>8703.21.10</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>ZFM - PIS</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>8703.21.10</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>8703.21.10</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>ZFM - Legislação</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Lei nº 10.485/2002, artigo 1º; Lei nº 11.196/2005, artigo 65</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>8703.21.10</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>ZFM - Observações</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>ALÍQUOTA - O fabricante ou importador dos produtos monofásicos citados no artigo 65 da Lei nº 11.196/2005 estabelecido fora da ZFM, fica obrigado a cobrar e recolher como substituto tributário o PIS e a COFINS devidos pela pessoa jurídica estabelecida na ZFM.
+Até 24.09.2020, as alíquotas eram de 2% (PIS) e de 9,6% (COFINS) (Lei nº 11.196/2005, artigo 65, § 1º, inciso III e Lei nº 10.485/2002, artigo 1º).
+A partir da vinculação da ADI nº 4.254, em 25.09.2020, o Supremo Tribunal Federal (STF) declarou a inconstitucionalidade das alíquotas majoradas citadas no artigo 65 da Lei nº 11.196/2005 e, em decorrência desse julgamento, o Ministro proferiu decisão determinando a aplicação das alíquotas gerais de 1,65% (PIS) e 7,6% (COFINS) para suprir a lacuna legislativa.
+Posteriormente, emitiu-se o Parecer SEI nº 298/2023 com vigência a partir de 30.03.2023, que concluiu pela inaplicabilidade legal das alíquotas estabelecidas pelo Ministro do STF e, determinou não ser possível a tributação sobre a revenda realizada pelas empresas situadas na ZFM, e consequentemente a substituição tributária pelo fabricante/importador, até que nova legislação fosse promulgada para fixar tais percentuais.
+Embora tenha sido publicada no DOU de 18.07.2023, a Instrução Normativa RFB nº 2.152/2023 consolidando no § 2º do artigo 545 e § 2º do artigo 551 da Instrução Normativa RFB nº 2.121/2022 a utilização das alíquotas de 1,65% (PIS) e 7,6% (COFINS), no mesmo sentido da ADI. Contudo, pela leitura do relatório complementar das Soluções de Consulta Cosit nº 271/2023 (item 20 do relatório) e nº 176/2024 (item 18 do relatório), a autoridade fiscal reconhece a necessidade de atualização do texto da Instrução Normativa para que ela seja adequada à redação do Parecer SEI nº 298/2023.
+Assim, interpreta-se que as alíquotas para o fabricante/importador na substituição tributária são:
+a) até 24.09.2020: 2% (PIS) e de 9,6% (COFINS) - Lei nº 11.196/2005, artigo 65, § 1º, inciso III;
+b) de 25.09.2020 em diante: inexistência de alíquotas para o importador/fabricante em decorrência de lacuna normativa, essa a ensejar, atualmente, a ausência de tributação na operação de revenda pela pessoa jurídica localizada na ZFM. - ADI nº 4.254; Parecer SEI nº 298/2023; SC Cosit nº 271/2023 e nº 176/2024.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica estabelecida fora dessas áreas, terão o mesmo tratamento da substituição tributária prevista para fabricante ou importador estabelecido fora da Zona Franca de Manaus. Porém, a redução a zero e a respectiva substituição tributária não se aplicam às vendas para adquirente atacadista ou varejista sujeito ao regime não cumulativo situado nas ALC (Lei nº 11.196/2005, artigos 2º, § 4º.
+As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+TRIBUTAÇÃO - A tributação de produtos monofásicos destinados ao consumo ou industrialização a Pessoas Jurídicas localizadas na ZFM possuirá dois momentos: a contribuição própria do vendedor localizado fora da área incentivada (redução a zero conforme prevê a Lei nº 10.996/2004, artigo 2º) e a contribuição como sujeito passivo por substituição tributária (responsável tributário), recolhendo antecipadamente o PIS e a COFINS do contribuinte situado na ZFM onde aplicará alíquotas de acordo com a legislação pertinente ao produto (Lei nº 11.196/2005, artigos 64 e 65; ADI nº 4.254).
+VENDA A MONTADORAS DE VEÍCULOS - Não haverá recolhimento da substituição tributária de PIS e COFINS nas vendas para montadoras de veículos situadas na ZFM, em relação as vendas das autopeças relacionadas nos Anexos I e II da Lei nº 10.485/2002 (Lei nº 11.196/2005, artigo 65, § 6º).
+DARF - As empresas optantes pelo regime cumulativo e não cumulativo recolherão o PIS e a COFINS em DARF, sobre as receitas de vendas à Zona Franca de Manaus (Substituição Tributária), nos códigos 1921 e 1840, respectivamente.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>2202.10.00</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Observações (Regra Geral)</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>CONCEITO DE INCIDÊNCIA MONOFÁSICA - As bebidas frias listadas no artigo 14 da Lei nº 13.097/2015 estão sujeitas a incidência monofásica, conforme prevê o artigo 25 da referida Lei. O sistema de tributação monofásica é um tratamento tributário próprio e específico, previsto em relação ao PIS e a COFINS incidentes sobre a receita bruta decorrente da venda de determinados produtos, onde usualmente a tributação ocorre de forma concentrada no produtor e importador, e no caso das bebidas frias ocorrerá também no atacadista, desonerando as etapas subsequentes de comercialização. A concentração da tributação ocorre com a aplicação de alíquotas maiores que as usualmente aplicadas na tributação das demais receitas.
+Em relação aos produtos classificados nas posições 22.01 e 22.02 da Tipi, o alcance da incidência monofásica é exclusivamente para água e refrigerantes, refrescos, cerveja sem álcool, repositores hidroeletrolíticos, bebidas energéticas e compostos líquidos prontos para o consumo que contenham como ingrediente principal inositol, glucoronolactona, taurina ou cafeína, segundo o parágrafo único do artigo 1º do Decreto nº 8.442/2015.
+SIMPLES NACIONAL - Para os fabricantes, importadores e distribuidores, a tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento, pois neste regime tributário não caberá a aplicação das alíquotas correspondentes à incidência monofásica em função do disposto no artigo 25, § 2º da Lei nº 13.097/2015.
+Cabe destacar que a atividade de produção e venda no atacado de bebidas alcoólicas estava terminantemente vedada ao Simples Nacional até 31/12/2017, passando a ser autorizada nos casos excepcionais de produção ou venda no atacado por micro e pequenos produtores. A atividade de produção e venda no atacado de cervejas sem álcool permanecerá vedada mesmo após 31/12/2017 (Lei Complementar nº 123/2006, artigo 17, inciso X, alíneas "b" e "c").
+Já na venda a varejo (nos moldes do conceito de varejista abaixo), ficam reduzidas a zero as alíquotas do PIS e da COFINS, de modo que estes contribuintes poderão segregar a receita e desonerar os percentuais efetivos das contribuições. (Lei nº 13.097/2015, artigo 28, § 2º).
+RECOLHIMENTO - São responsáveis pelo recolhimento do PIS e da COFINS, os importadores, fabricantes e atacadistas dos produtos relacionados no artigo 14 da Lei nº 13.097/2015.
+VALORES MÍNIMOS - São estabelecidos valores mínimos para o PIS e a COFINS, conforme tipo de produto e da capacidade do recipiente, segundo o Anexo I da Lei nº 13.097/2015 (Decreto nº 8.442/2015, artigo 30). Os valores dos tributos não podem ser inferiores aos valores mínimos, mesmo após a aplicação de qualquer das reduções de alíquotas previstas no Decreto nº 8.442/2015.
+CONCEITO DE VAREJISTA - Considera-se varejista a pessoa jurídica cuja receita decorrente da venda de bens e serviços a consumidor final no ano-calendário imediatamente anterior ao da operação houver sido igual ou superior a 75% de sua receita total de venda de bens e serviços no mesmo período, depois de excluídos os impostos e contribuições incidentes sobre a venda (Decreto nº 8.442/2015, artigo 2º, inciso III, e artigo 3º).
+ALÍQUOTA ZERO - São reduzidas a zero as alíquotas de PIS e COFINS sobre as receitas auferidas por pessoa jurídica varejista, inclusive quando a venda for realizada por empresa optante pelo Simples Nacional (Decreto nº 8.442/2015, artigo 22, caput e § 2º).
+FRETE - Nas operações de venda por pessoa jurídica industrial ou atacadista, o valor do frete integrará a base de cálculo do PIS e da COFINS apurados pela pessoa jurídica vendedora dos citados produtos (Lei nº 13.097/2015, artigo 27; Decreto nº 8.442/2015, artigo 15).
+INDUSTRIALIZAÇÃO POR ENCOMENDA - Na industrialização por encomenda, observados os valores mínimos exigidos, o PIS e a COFINS incidirão sobre a receita auferida pela pessoa jurídica executora da encomenda às alíquotas de 1,65% (PIS) e 7,60% (COFINS), independentemente do regime de apuração a que está submetida a pessoa jurídica (Lei nº 13.097/2015, artigo 25, § 3º e artigo 33; Decreto nº 8.442/2015, artigos 18 e 30; Solução de Consulta Cosit nº 75/2019).
+CRÉDITO PELA AQUISIÇÃO - REGIME NÃO CUMULATIVO - A pessoa jurídica sujeita ao regime de apuração não cumulativa poderá descontar créditos de PIS e COFINS em relação à aquisição no mercado interno ou à importação desse produto, conforme os valores informados na nota fiscal do vendedor.
+Nas aquisições de produtos de pessoa jurídica optante pelo Simples Nacional, os créditos serão calculados mediante a aplicação sobre o valor de aquisição constante do documento fiscal de percentual correspondente a 0,38% (PIS) e 1,60% (COFINS) (Decreto nº 8.442/2015, artigos 24 e 29).
+UTILIZAÇÃO DO CRÉDITO - O crédito para o regime não cumulativo e o crédito presumido somente podem ser utilizados para desconto do valor do PIS e da COFINS devidos pela pessoa jurídica.
+VEDAÇÃO AO CRÉDITO - Fica vedado à pessoa jurídica varejista descontar os créditos do PIS e da COFINS, em relação ao produto revendido com a aplicação da alíquota zero, de acordo com os artigos 22 e 27 do Decreto nº 8.442/2015.
+DARF - As empresas optantes pelo regime cumulativo e não cumulativo recolherão o PIS e a COFINS em DARF, sobre as bebidas frias (Lei nº 13.097/2015, artigos 14 a 36) nos códigos 0691 e 0776, exceto cervejas, que devem ser recolhidos sob os códigos 0679 e 0760 respectivamente, segundo o ADE CODAC nº 21/2015.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>2202.10.00</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>ZFM - PIS</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>2202.10.00</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>2202.10.00</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>ZFM - Legislação</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr"/>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>2202.10.00</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>ZFM - Observações</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+Com isso, a operação será tributada de acordo com os percentuais específicos aplicáveis às bebidas frias.
+ZONA FRANCA DE MANAUS (ZFM) - Os fabricantes, importadores, comerciantes atacadistas e varejistas estabelecidos fora da Zona Franca de Manaus que vendam bebidas frias para a região incentivada não se sujeitam à alíquota zero na venda, e, em consequência, não estarão sujeitos ao recolhimento na condição de contribuinte substituto do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, § 6º; Lei nº 13.097/2015, artigo 14).
+Com isso, a operação será tributada de acordo com os percentuais específicos aplicáveis às bebidas frias relacionadas na aba anterior.
+ÁREAS DE LIVRE COMÉRCIO - Da mesma forma que nas venda à Zona Franca de Manaus, as vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, não se sujeitam à alíquota zero, devendo ser tributada conforme os percentuais específicos previstos para as operações com bebidas frias relacionadas na aba anterior.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>8481.80.99</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Observações (Regra Geral)</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>REGRA GERAL - O código NCM pesquisado pode enquadrar-se dentre os produtos com benefícios fiscais de PIS e COFINS previstos em legislação. Antes de aplicar as alíquotas correspondentes ao regime tributário da pessoa jurídica é recomendado analisar as outras guias.
+CONDIÇÃO DO ADQUIRENTE - Antes de aplicar a alíquota básica, é importante verificar se a pessoa jurídica adquirente é habilitada em algum regime especial, se está localizada na Zona Franca de Manaus (ZFM) ou em Área de Livre Comércio (ALC), e se a receita é proveniente de exportação de mercadorias.
+NÃO APLICAÇÃO DA INCIDÊNCIA MONOFÁSICA - O Anexo I da Lei nº 10.485/2002 determina a incidência monofásica para a NCM 8481.80.99 Ex 01 e 02 e não se aplica a NCM 8481.80.99 (sem EX). Com a publicação do Decreto nº 5.804/2006, artigo 2º, ficaram suprimidos da tabela do IPI as posições EX 01 a 03 da NCM 8481.80.99 e por conseguinte, a incidência monofásica para as referidas posições NCM da Tipi.
+SIMPLES NACIONAL - A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+DARF - As empresas optantes pelo regime cumulativo recolherão o PIS e a COFINS em DARF, nos códigos 8109 e 2172, respectivamente.
+Para o regime não cumulativo os códigos serão 6912 e 5856.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>8481.80.99</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Suspensão - PIS</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>8481.80.99</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Suspensão - COFINS</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>8481.80.99</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Suspensão - Legislação</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>8481.80.99</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Suspensão - Observações</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr"/>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da suspensão do PIS e da COFINS sobre as receitas de vendas de mercadorias, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+REGIME CUMULATIVO / NÃO CUMULATIVO - Aplica-se a suspensão do PIS e da COFINS à venda realizada para pessoa jurídica beneficiária do Regime Especial de Aquisição de bens de Capital para Empresas Exportadoras (RECAP), para incorporação ao seu ativo imobilizado (Lei nº 11.196/2005, artigo 12; Decreto nº 5.789/2006).</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>8481.80.99</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>ZFM - PIS</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>8481.80.99</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>8481.80.99</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>ZFM - Legislação</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>8481.80.99</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>ZFM - Observações</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+ZONA FRANCA DE MANAUS (ZFM) - Para os regimes cumulativo e não cumulativo, ficam reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas de vendas de mercadorias destinadas ao consumo (utilizadas diretamente ou para comercialização por atacado ou a varejo) ou à industrialização na Zona Franca de Manaus, por pessoa jurídica estabelecida fora da ZFM (Lei nº 10.996/2004, artigo 2º).
+Nas notas fiscais relativas à venda, deverá constar a expressão "Venda de mercadoria efetuada com alíquota zero da Contribuição para o PIS/Pasep e da COFINS - Lei nº 10.996/2004, artigo 2º".
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, terão a alíquota do PIS e da COFINS reduzidas a zero, exceto nas vendas de mercadorias que tenham como destinatárias pessoas jurídicas atacadistas e varejistas, sujeitas ao regime de apuração não cumulativa do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, §§ 3º e 4º). As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+MATÉRIAS-PRIMAS, PRODUTOS INTERMEDIÁRIOS E MATERIAIS DE EMBALAGEM - São reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas decorrentes da comercialização de matérias-primas, produtos intermediários e materiais de embalagem, produzidos na Zona Franca de Manaus para emprego em processo de industrialização por estabelecimentos industriais dos regimes cumulativo ou não cumulativo ali instalados, consoante projetos aprovados pelo Conselho de Administração da Superintendência da Zona Franca de Manaus (SUFRAMA) (Lei nº 10.637/2002, artigo 5º-A).
+REGIME NÃO CUMULATIVO - As alíquotas especiais para vendas realizadas por pessoa jurídica optante pelo regime não cumulativo estabelecida na Zona Franca de Manaus estão dispostas abaixo do item "Solução de Consulta".</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>9403.60.90</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Observações (Regra Geral)</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>REGRA GERAL - O código NCM pesquisado pode enquadrar-se dentre os produtos com benefícios fiscais de PIS e COFINS previstos em legislação. Antes de aplicar as alíquotas correspondentes ao regime tributário da pessoa jurídica é recomendado analisar as outras guias.
+CONDIÇÃO DO ADQUIRENTE - Antes de aplicar a alíquota básica, é importante verificar se a pessoa jurídica adquirente é habilitada em algum regime especial, se está localizada na Zona Franca de Manaus (ZFM) ou em Área de Livre Comércio (ALC), e se a receita é proveniente de exportação de mercadorias.
+SIMPLES NACIONAL - A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+DARF - As empresas optantes pelo regime cumulativo recolherão o PIS e a COFINS em DARF, nos códigos 8109 e 2172, respectivamente.
+Para o regime não cumulativo os códigos serão 6912 e 5856.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>9403.60.90</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Suspensão - PIS</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>9403.60.90</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Suspensão - COFINS</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>9403.60.90</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Suspensão - Legislação</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr"/>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>9403.60.90</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Suspensão - Observações</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da suspensão do PIS e da COFINS sobre as receitas de vendas de mercadorias, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+REGIME CUMULATIVO / NÃO CUMULATIVO - Aplica-se a suspensão do PIS e da COFINS nos casos de venda realizada a pessoa jurídica inscrita no Regime Especial de Tributação para Desenvolvimento da Atividade de Exibição Cinematográfica (RECINE) (Lei nº 12.599/2012, artigos 12 a 15; Decreto nº 7.729/2012).
+Prazo de vigência do benefício do RECINE: Até 31.12.2029 (Lei nº 13.594/2018).
+A partir de 01.04.2026, os incentivos e benefícios federais de natureza tributária são reduzidos, sendo aqueles de alíquota zero mediante a aplicação de alíquota correspondente a 10% da alíquota do sistema padrão de tributação. Desta forma, tendo em vista que para o PIS e a Cofins existem dois regimes de tributação, as alíquotas devem corresponder a 10% das alíquotas padrão de cada um dos regimes:
+a) Regime cumulativo - PIS: 0,065%; Cofins: 0,3%;
+b) Regime não cumulativo - PIS: 0,165%; Cofins: 0,76%. (Lei Complementar nº 224/2025, artigo 4º, caput e § 4º, inciso I)
+Ressalta-se que o § 1°, do artigo 2°, da IN RFB n° 2.305/2025 limita a redução dos benefícios àqueles discriminados no demonstrativo de gastos tributários anexo à Lei Orçamentária Anual de 2026. O Recine está discriminado, sofrendo redução do benefício.
+Quanto à aplicação da redução dos benefícios, no caso da suspensão, o artigo 6°, da IN RFB n° 2.305/2025 estabelece que a redução não se aplica aos benefícios de suspensão em que se verifique apenas um diferimento temporal no recolhimento do tributo. Logo, tendo em vista que o inciso II, do § 3°, do artigo 14, da Lei n° 12.599/2012 estabelece que a suspensão do PIS/Cofins converte-se em alíquota zero após a incorporação do bem ou material de construção no ativo imobilizado ou sua utilização no complexo de exibição cinematográfica ou cinema itinerante, situação na qual a operação fica sujeita à redução do benefício disposto na Lei Complementar nº 224/2025.
+Preventivamente, a sugestão é de que no cálculo para demonstrar o aumento da carga deve ser aplicado 10% das alíquotas do sistema padrão de PIS/Cofins sobre as vendas ou importação, baseado no artigo 7° da IN RFB 2.305/2025. Tal sugestão é um entendimento que poderá ser confirmado ou reformulado mediante esclarecimento da RFB.
+Visto que essas informações não estão claras na legislação, recomenda-se ao contribuinte buscar o serviço do Receita Soluciona, por meio das Confederações Nacionais de Representação de Categorias Econômicas, às Centrais Sindicais, aos Órgãos de Registro de Classe com atuação nacional e Organizações Associativas Patronais e Empresarias.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>9403.60.90</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>ZFM - PIS</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>9403.60.90</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr"/>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>9403.60.90</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>ZFM - Legislação</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>9403.60.90</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>ZFM - Observações</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+ZONA FRANCA DE MANAUS (ZFM) - Para os regimes cumulativo e não cumulativo, ficam reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas de vendas de mercadorias destinadas ao consumo (utilizadas diretamente ou para comercialização por atacado ou a varejo) ou à industrialização na Zona Franca de Manaus, por pessoa jurídica estabelecida fora da ZFM (Lei nº 10.996/2004, artigo 2º).
+Nas notas fiscais relativas à venda, deverá constar a expressão "Venda de mercadoria efetuada com alíquota zero da Contribuição para o PIS/Pasep e da COFINS - Lei nº 10.996/2004, artigo 2º".
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, terão a alíquota do PIS e da COFINS reduzidas a zero, exceto nas vendas de mercadorias que tenham como destinatárias pessoas jurídicas atacadistas e varejistas, sujeitas ao regime de apuração não cumulativa do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, §§ 3º e 4º). As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+MATÉRIAS-PRIMAS, PRODUTOS INTERMEDIÁRIOS E MATERIAIS DE EMBALAGEM - São reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas decorrentes da comercialização de matérias-primas, produtos intermediários e materiais de embalagem, produzidos na Zona Franca de Manaus para emprego em processo de industrialização por estabelecimentos industriais dos regimes cumulativo ou não cumulativo ali instalados, consoante projetos aprovados pelo Conselho de Administração da Superintendência da Zona Franca de Manaus (SUFRAMA) (Lei nº 10.637/2002, artigo 5º-A).
+REGIME NÃO CUMULATIVO - As alíquotas especiais para vendas realizadas por pessoa jurídica optante pelo regime não cumulativo estabelecida na Zona Franca de Manaus estão dispostas abaixo do item "Solução de Consulta".</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>3004.90.99</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Observações (Regra Geral)</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>CONCEITO DE INCIDÊNCIA MONOFÁSICA - O sistema de tributação monofásica é um tratamento tributário próprio e específico, previsto em relação ao PIS e a COFINS incidentes sobre a receita bruta decorrente da venda de determinados produtos, geralmente a fim de concentrar a tributação nas etapas de produção e importação, desonerando as etapas subsequentes de comercialização.
+A concentração da tributação ocorre com a aplicação de alíquotas maiores que as usualmente aplicadas na tributação das demais receitas.
+O álcool e as bebidas frias relacionadas no artigo 14 da Lei nº 13.097/2015 são exceções à regra, visto que o distribuidor também é responsável pelo recolhimento do PIS e da COFINS.
+SIMPLES NACIONAL - As leis que estabelecem a incidência monofásica não trazem dispensa no recolhimento da alíquota concentrada quando se trata de importador ou fabricante optante pelo Simples Nacional. Deste modo, o importador e o fabricante deverão proceder o recolhimento do PIS e da COFINS em DARF separado, mediante a aplicação das alíquotas diferenciadas previstas em legislação própria conforme o produto.
+Deve ser destacada a receita decorrente da venda desse produto, aplicando-se, sobre tal receita, a alíquota efetiva calculada com base no Anexo II da Lei Complementar nº 123/2006, mas sem considerar os percentuais destinados ao PIS e a COFINS.
+Para tanto, o importador e a indústria devem selecionar a atividade de "venda de mercadorias industrializadas, com substituição tributária/tributação monofásica", indicando a opção tributação monofásica em relação ao PIS e a COFINS, a fim de que o aplicativo desconsidere os percentuais desses tributos sobre a receita destacada, ou seja, o recolhimento não será realizado pelo DAS e sim em DARF separado (Lei Complementar nº 123/2006, artigo 18, § 4º-A, inciso I).
+Desde 01.01.2018, a atividade de produção e venda no atacado de bebidas alcoólicas não está vedada ao ingresso ao Simples Nacional, desde que praticada por:
+a) micro e pequenas cervejarias;
+b) micro e pequenas vinícolas;
+c) produtores de licores;
+d) micro e pequenas destilarias.
+As ME e EPP optantes pelo Simples Nacional deverão obrigatoriamente estar registradas no Ministério da Agricultura, Pecuária e Abastecimento e obedecerão também à regulamentação da Agência Nacional de Vigilância Sanitária e da Secretaria da Receita Federal do Brasil quanto à produção e à comercialização de bebidas alcoólicas (Lei Complementar nº 123/2006, artigo 17, § 5º).
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+REGIME CUMULATIVO / NÃO CUMULATIVO (IMPORTADOR OU INDÚSTRIA) - A receita bruta auferida por importador ou por indústria, optantes pelos regimes cumulativo ou não cumulativo, sujeita-se à incidência monofásica do PIS e da COFINS sobre os produtos constantes no artigo 1º da Lei nº 10.147/2000.
+INDUSTRIALIZAÇÃO POR ENCOMENDA - Na industrialização por encomenda, exceto sobre os medicamentos relacionados no artigo 1º, inciso I, alíneas "a" e "b" da Lei nº 10.147/2000, o PIS e a COFINS incidirão sobre a receita auferida pela pessoa jurídica executora da encomenda às alíquotas de 1,65% (PIS) e 7,60% (COFINS), independentemente do regime de apuração a que está submetida a pessoa jurídica. O encomendante deve recolher o PIS e a COFINS mediante as alíquotas monofásicas (Lei nº 11.051/2004, artigo 10, § 2º e Lei nº 10.833/2003, artigo 25, inciso I).
+DARF - As empresas optantes pelo Simples Nacional recolherão o PIS e a COFINS em DARF, nos códigos 8109 e 2172, respectivamente (Lei nº 10.833/2003, artigo 10, inciso III).
+Para as empresas optantes pelo regime cumulativo, o recolhimento será nos códigos 8109 e 2172 e para as optantes pelo regime não cumulativo, será nos códigos 6912 e 5856.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>3004.90.99</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>ZFM - PIS</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>3004.90.99</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>3004.90.99</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>ZFM - Legislação</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>3004.90.99</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>ZFM - Observações</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+ZONA FRANCA DE MANAUS (ZFM) - Para os regimes cumulativo e não cumulativo, ficam reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas de vendas de mercadorias destinadas ao consumo (utilizadas diretamente ou para comercialização por atacado ou a varejo) ou à industrialização na Zona Franca de Manaus, por pessoa jurídica estabelecida fora da ZFM (Lei nº 10.996/2004, artigo 2º).
+Nas notas fiscais relativas à venda, deverá constar a expressão "Venda de mercadoria efetuada com alíquota zero da Contribuição para o PIS/Pasep e da COFINS - Lei nº 10.996/2004, artigo 2º".
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, terão a alíquota do PIS e da COFINS reduzidas a zero, exceto nas vendas de mercadorias que tenham como destinatárias pessoas jurídicas atacadistas e varejistas, sujeitas ao regime de apuração não cumulativa do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, §§ 3º e 4º). As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+MATÉRIAS-PRIMAS, PRODUTOS INTERMEDIÁRIOS E MATERIAIS DE EMBALAGEM - São reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas decorrentes da comercialização de matérias-primas, produtos intermediários e materiais de embalagem, produzidos na Zona Franca de Manaus para emprego em processo de industrialização por estabelecimentos industriais dos regimes cumulativo ou não cumulativo ali instalados, consoante projetos aprovados pelo Conselho de Administração da Superintendência da Zona Franca de Manaus (SUFRAMA) (Lei nº 10.637/2002, artigo 5º-A).
+REGIME NÃO CUMULATIVO - As alíquotas especiais para vendas realizadas por pessoa jurídica optante pelo regime não cumulativo estabelecida na Zona Franca de Manaus estão dispostas abaixo do item "Solução de Consulta".</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>8443.31.00</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Observações (Regra Geral)</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>REGRA GERAL - O código NCM pesquisado não se encontra dentre os produtos com benefícios fiscais de PIS e COFINS previstos em legislação. Antes de aplicar as alíquotas correspondentes ao regime tributário da pessoa jurídica é recomendado analisar as outras guias.
+CONDIÇÃO DO ADQUIRENTE - Antes de aplicar a alíquota básica, é importante verificar se a pessoa jurídica adquirente é habilitada em algum regime especial, se está localizada na Zona Franca de Manaus (ZFM) ou em Área de Livre Comércio (ALC), e se a receita é proveniente de exportação de mercadorias.
+SIMPLES NACIONAL - A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+DARF - As empresas optantes pelo regime cumulativo recolherão o PIS e a COFINS em DARF, nos códigos 8109 e 2172, respectivamente.
+Para o regime não cumulativo os códigos serão 6912 e 5856.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>8443.31.00</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>ZFM - PIS</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>8443.31.00</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>8443.31.00</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>ZFM - Legislação</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>8443.31.00</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>ZFM - Observações</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+ZONA FRANCA DE MANAUS (ZFM) - Para os regimes cumulativo e não cumulativo, ficam reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas de vendas de mercadorias destinadas ao consumo (utilizadas diretamente ou para comercialização por atacado ou a varejo) ou à industrialização na Zona Franca de Manaus, por pessoa jurídica estabelecida fora da ZFM (Lei nº 10.996/2004, artigo 2º).
+Nas notas fiscais relativas à venda, deverá constar a expressão "Venda de mercadoria efetuada com alíquota zero da Contribuição para o PIS/Pasep e da COFINS - Lei nº 10.996/2004, artigo 2º".
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, terão a alíquota do PIS e da COFINS reduzidas a zero, exceto nas vendas de mercadorias que tenham como destinatárias pessoas jurídicas atacadistas e varejistas, sujeitas ao regime de apuração não cumulativa do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, §§ 3º e 4º). As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+MATÉRIAS-PRIMAS, PRODUTOS INTERMEDIÁRIOS E MATERIAIS DE EMBALAGEM - São reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas decorrentes da comercialização de matérias-primas, produtos intermediários e materiais de embalagem, produzidos na Zona Franca de Manaus para emprego em processo de industrialização por estabelecimentos industriais dos regimes cumulativo ou não cumulativo ali instalados, consoante projetos aprovados pelo Conselho de Administração da Superintendência da Zona Franca de Manaus (SUFRAMA) (Lei nº 10.637/2002, artigo 5º-A).
+REGIME NÃO CUMULATIVO - As alíquotas especiais para vendas realizadas por pessoa jurídica optante pelo regime não cumulativo estabelecida na Zona Franca de Manaus estão dispostas abaixo do item "Solução de Consulta".</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>1006.30.21</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Observações (Regra Geral)</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+REGIME CUMULATIVO / NÃO CUMULATIVO - Aplica-se à alíquota zero do PIS e da COFINS à receita bruta de venda no mercado interno (Lei nº 10.925/2004, artigo 1º, inciso V).</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>1006.30.21</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>ZFM - PIS</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>1006.30.21</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr"/>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>1006.30.21</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>ZFM - Legislação</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>1006.30.21</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>ZFM - Observações</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+ZONA FRANCA DE MANAUS (ZFM) - Para os regimes cumulativo e não cumulativo, ficam reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas de vendas de mercadorias destinadas ao consumo (utilizadas diretamente ou para comercialização por atacado ou a varejo) ou à industrialização na Zona Franca de Manaus, por pessoa jurídica estabelecida fora da ZFM (Lei nº 10.996/2004, artigo 2º).
+Nas notas fiscais relativas à venda, deverá constar a expressão "Venda de mercadoria efetuada com alíquota zero da Contribuição para o PIS/Pasep e da COFINS - Lei nº 10.996/2004, artigo 2º".
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, terão a alíquota do PIS e da COFINS reduzidas a zero, exceto nas vendas de mercadorias que tenham como destinatárias pessoas jurídicas atacadistas e varejistas, sujeitas ao regime de apuração não cumulativa do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, §§ 3º e 4º). As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+MATÉRIAS-PRIMAS, PRODUTOS INTERMEDIÁRIOS E MATERIAIS DE EMBALAGEM - São reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas decorrentes da comercialização de matérias-primas, produtos intermediários e materiais de embalagem, produzidos na Zona Franca de Manaus para emprego em processo de industrialização por estabelecimentos industriais dos regimes cumulativo ou não cumulativo ali instalados, consoante projetos aprovados pelo Conselho de Administração da Superintendência da Zona Franca de Manaus (SUFRAMA) (Lei nº 10.637/2002, artigo 5º-A).
+REGIME NÃO CUMULATIVO - As alíquotas especiais para vendas realizadas por pessoa jurídica optante pelo regime não cumulativo estabelecida na Zona Franca de Manaus estão dispostas abaixo do item "Solução de Consulta".</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>8708.29.99</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Observações (Regra Geral)</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>REGRA GERAL - O código NCM pesquisado não se encontra dentre os produtos com benefícios fiscais de PIS e COFINS previstos em legislação. Antes de aplicar as alíquotas correspondentes ao regime tributário da pessoa jurídica é recomendado analisar as outras guias.
+INCIDÊNCIA MONOFÁSICA - Caberá a aplicação da incidência monofásica para os produtos constantes dos Anexos I e II da Lei nº 10.485/2002, caso o produto seja destinado ao setor automotivo, conforme previsto Solução de Consulta Cosit nº 55/2018.
+O item 27 da referida solução de consulta, prevê que: Se pelas suas características, dimensões, finalidades, for possível evidenciar não ter aplicação no setor automotivo, deverão ser aplicadas as alíquotas gerais de acordo com a sistemática de tributação do vendedor, Lucro Real, Lucro Presumido ou Simples Nacional, haja vista não se subsumir às previsões da Lei nº 10.485/2002.
+Nesta concepção o setor automotivo engloba os veículos automotores terrestres (tais como carros, ônibus, caminhões, tratores, entre outros), motocicletas e as máquinas agrícolas autopropulsadas, não compreendendo na incidência monofásica, portanto, as autopeças constantes nos Anexos I e II destinadas à embarcações e aeronaves (Solução de Consulta Interna Cosit nº 01/2019; Solução de Consulta nº 4.005/2020, da 4ª Região Fiscal; Solução de Consulta COSIT nº 149/2018).
+O entendimento expresso na Solução de Consulta Cosit nº 55/2018 também é reforçado com a previsão do § 4º, do artigo 427 da IN nº 2.121/2022, incluído pela Instrução Normativa RFB nº 2.152/2023, que indica a aplicação das alíquotas de regra geral, em caso que os produtos dos Anexos I e II não sejam partes ou componentes das máquinas, dos veículos e dos implementos citados no artigo 1º da Lei nº 10.485/2002.
+Adicionalmente informamos que a Solução de Consulta Cosit e a Solução de Divergência, a partir da data de sua publicação, têm efeito vinculante no âmbito da RFB, respaldam o sujeito passivo que as aplicar, independentemente de ser o consulente, desde que se enquadre na hipótese por elas abrangida, sem prejuízo de que a autoridade fiscal, em procedimento de fiscalização, verifique seu efetivo enquadramento (IN RFB nº 2.058/2021, artigo 33, e artigo 39, § 2º).
+PRODUTOS USADOS - Os produtos usados não estão sujeitos a incidência monofásica do PIS e da COFINS (Lei nº 10.485/2002, artigo 6º).
+CONDIÇÃO DO ADQUIRENTE - Antes de aplicar a alíquota básica, é importante verificar se a pessoa jurídica adquirente é habilitada em algum regime especial, se está localizada na Zona Franca de Manaus (ZFM) ou em Área de Livre Comércio (ALC), e se a receita é proveniente de exportação de mercadorias.
+SIMPLES NACIONAL - A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+DARF - As empresas optantes pelo regime cumulativo recolherão o PIS e a COFINS em DARF, nos códigos 8109 e 2172, respectivamente.
+Para o regime não cumulativo os códigos serão 6912 e 5856.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>8708.29.99</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>ZFM - PIS</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>8708.29.99</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>8708.29.99</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>ZFM - Legislação</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Lei nº 10.485/2002, artigos 1º e 3º</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>8708.29.99</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>ZFM - Observações</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>VENDA A MONTADORAS DE VEÍCULOS - Não se aplica a substituição tributária na venda de autopeças, pneus novos e câmaras de ar para montadoras de veículos. (Lei nº 11.196/2005, artigo 65, § 6º).
+Não haverá crédito de PIS e COFINS nas aquisições feitas pelas montadoras de veículos estabelecidas na ZFM, pela compra dos referidos produtos, mesmo sendo a título de insumo ou imobilizado (Lei nº 11.196/2005, artigo 65, § 6º).
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica estabelecida fora dessas áreas, terão o mesmo tratamento da substituição tributária prevista para fabricante ou importador estabelecido fora da Zona Franca de Manaus. Porém, a redução a zero e a respectiva substituição tributária não se aplicam às vendas para adquirente atacadista ou varejista sujeito ao regime não cumulativo situado nas ALC (Lei nº 11.196/2005, artigos 2º, § 4º.
+As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+TRIBUTAÇÃO - A tributação de produtos monofásicos destinados ao consumo ou industrialização a Pessoas Jurídicas localizadas na ZFM possuirá dois momentos: a contribuição própria do vendedor localizado fora da área incentivada (redução a zero conforme prevê a Lei nº 10.996/2004, artigo 2º) e a contribuição como sujeito passivo por substituição tributária (responsável tributário), recolhendo antecipadamente o PIS e a COFINS do contribuinte situado na ZFM onde aplicará alíquotas de acordo com a legislação pertinente ao produto (Lei nº 11.196/2005, artigos 64 e 65; ADI nº 4.254).
+PRODUTOS USADOS - Os produtos usados não estão sujeitos a incidência monofásica do PIS e da COFINS (Lei nº 10.485/2002, artigo 6º).
+ALÍQUOTAS - O fabricante ou importador dos produtos monofásicos citados no artigo 65 da Lei nº 11.196/2005 estabelecido fora da ZFM, fica obrigado a cobrar e recolher como substituto tributário o PIS e a COFINS devidos pela pessoa jurídica estabelecida na ZFM.
+Até 24.09.2020, as alíquotas eram de 2,30% (PIS) e de 10,80% (COFINS) nas vendas para comerciantes atacadistas, varejistas ou consumidores, ou de 1,65% (PIS) e 7,6% (COFINS) nas vendas a fabricantes de veículos e máquinas do artigo 1º da Lei nº 10.485/2002 ou para fabricantes de autopeças dos Anexos I e II da mesma lei. (Lei nº 11.196/2005, artigo 65, § 1º, inciso V e Lei nº 10.485/2002, artigo 3º, inciso II).
+A partir da vinculação da ADI nº 4.254, em 25.09.2020, o Supremo Tribunal Federal (STF) declarou a inconstitucionalidade das alíquotas majoradas citadas no artigo 65 da Lei nº 11.196/2005 e, em decorrência desse julgamento, o Ministro proferiu decisão determinando a aplicação das alíquotas gerais de 1,65% (PIS) e 7,6% (COFINS) para suprir a lacuna legislativa.
+Posteriormente, emitiu-se o Parecer SEI nº 298/2023 com vigência a partir de 30.03.2023, que concluiu pela inaplicabilidade legal das alíquotas estabelecidas pelo Ministro do STF e, determinou não ser possível a tributação sobre a revenda realizada pelas empresas situadas na ZFM, e consequentemente a substituição tributária pelo fabricante/importador, até que nova legislação fosse promulgada para fixar tais percentuais.
+Embora tenha sido publicada no DOU de 18.07.2023, a Instrução Normativa RFB nº 2.152/2023 consolidando no § 2º do artigo 545 e § 2º do artigo 551 da Instrução Normativa RFB nº 2.121/2022 a utilização das alíquotas de 1,65% (PIS) e 7,6% (COFINS), no mesmo sentido da ADI. Contudo, pela leitura do relatório complementar das Soluções de Consulta Cosit n° 271/2023 (item 20 do relatório) e nº 176/2024 (item 18 do relatório), a autoridade fiscal reconhece a necessidade de atualização do texto da Instrução Normativa para que ela seja adequada à redação do Parecer SEI nº 298/2023.
+Assim, interpreta-se que as alíquotas para o fabricante/importador na substituição tributária são:
+a) até 24.09.2020: 2,30% (PIS) e de 10,80% (COFINS) - nas vendas para comerciantes atacadistas, varejistas ou consumidores, ou de 1,65% (PIS) e 7,6% (COFINS) nas vendas a fabricantes de veículos e máquinas do artigo 1º da Lei nº 10.485/2002 ou para fabricantes de autopeças dos Anexos I e II da mesma lei. (Lei nº 11.196/2005, artigo 65, § 1º, inciso V);
+b) de 25.09.2020 em diante: inexistência de alíquotas para o importador/fabricante em decorrência de lacuna normativa, essa a ensejar, atualmente, a ausência de tributação na operação de revenda pela pessoa jurídica localizada na ZFM. ADI nº 4.254; Parecer SEI nº 298/2023; SC Cosit n° 271/2023 e nº 176/2024.
+DARF - As empresas optantes pelo regime cumulativo e não cumulativo recolherão o PIS e a COFINS em DARF, sobre as receitas de vendas à Zona Franca de Manaus (Substituição Tributária), nos códigos 1921 e 1840, respectivamente.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>0207.14.00</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Observações (Regra Geral)</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+REGIME CUMULATIVO / NÃO CUMULATIVO - O produto está sujeito à alíquota zero do PIS e da COFINS sobre a receita decorrente da venda no mercado interno (Lei nº 10.925/2004, artigo 1º, inciso XIX e § 4º) .
+Também aplica-se a alíquota zero e sobre a receita bruta decorrente das saídas do estabelecimento industrial, na industrialização por conta e ordem de terceiros, dos bens e produtos classificados nas posições NCM 0103, 0105, 0203, 02.06.30.00, 0206.4, 0207 e 0210.1 (Lei nº 10.925/2004, artigo 1º, § 4º).</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>0207.14.00</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>ZFM - PIS</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>0207.14.00</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>0207.14.00</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>ZFM - Legislação</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr"/>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>0207.14.00</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>ZFM - Observações</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+ZONA FRANCA DE MANAUS (ZFM) - Para os regimes cumulativo e não cumulativo, ficam reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas de vendas de mercadorias destinadas ao consumo (utilizadas diretamente ou para comercialização por atacado ou a varejo) ou à industrialização na Zona Franca de Manaus, por pessoa jurídica estabelecida fora da ZFM (Lei nº 10.996/2004, artigo 2º).
+Nas notas fiscais relativas à venda, deverá constar a expressão "Venda de mercadoria efetuada com alíquota zero da Contribuição para o PIS/Pasep e da COFINS - Lei nº 10.996/2004, artigo 2º".
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, terão a alíquota do PIS e da COFINS reduzidas a zero, exceto nas vendas de mercadorias que tenham como destinatárias pessoas jurídicas atacadistas e varejistas, sujeitas ao regime de apuração não cumulativa do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, §§ 3º e 4º). As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+MATÉRIAS-PRIMAS, PRODUTOS INTERMEDIÁRIOS E MATERIAIS DE EMBALAGEM - São reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas decorrentes da comercialização de matérias-primas, produtos intermediários e materiais de embalagem, produzidos na Zona Franca de Manaus para emprego em processo de industrialização por estabelecimentos industriais dos regimes cumulativo ou não cumulativo ali instalados, consoante projetos aprovados pelo Conselho de Administração da Superintendência da Zona Franca de Manaus (SUFRAMA) (Lei nº 10.637/2002, artigo 5º-A).
+REGIME NÃO CUMULATIVO - As alíquotas especiais para vendas realizadas por pessoa jurídica optante pelo regime não cumulativo estabelecida na Zona Franca de Manaus estão dispostas abaixo do item "Solução de Consulta".</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>1507.90.11</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Observações (Regra Geral)</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr"/>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>REGRA GERAL - O código NCM pesquisado pode enquadrar-se dentre os produtos com benefícios fiscais de PIS e COFINS previstos em legislação. Antes de aplicar as alíquotas correspondentes ao regime tributário da pessoa jurídica é recomendado analisar as outras guias.
+CONDIÇÃO DO ADQUIRENTE - Antes de aplicar a alíquota básica, é importante verificar se a pessoa jurídica adquirente é habilitada em algum regime especial, se está localizada na Zona Franca de Manaus (ZFM) ou em Área de Livre Comércio (ALC), e se a receita é proveniente de exportação de mercadorias.
+SIMPLES NACIONAL - A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+DARF - As empresas optantes pelo regime cumulativo recolherão o PIS e a COFINS em DARF, nos códigos 8109 e 2172, respectivamente.
+Para o regime não cumulativo os códigos serão 6912 e 5856.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>1507.90.11</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>ZFM - PIS</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>1507.90.11</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr"/>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>1507.90.11</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>ZFM - Legislação</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr"/>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>1507.90.11</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>ZFM - Observações</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr"/>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+ZONA FRANCA DE MANAUS (ZFM) - Para os regimes cumulativo e não cumulativo, ficam reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas de vendas de mercadorias destinadas ao consumo (utilizadas diretamente ou para comercialização por atacado ou a varejo) ou à industrialização na Zona Franca de Manaus, por pessoa jurídica estabelecida fora da ZFM (Lei nº 10.996/2004, artigo 2º).
+Nas notas fiscais relativas à venda, deverá constar a expressão "Venda de mercadoria efetuada com alíquota zero da Contribuição para o PIS/Pasep e da COFINS - Lei nº 10.996/2004, artigo 2º".
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, terão a alíquota do PIS e da COFINS reduzidas a zero, exceto nas vendas de mercadorias que tenham como destinatárias pessoas jurídicas atacadistas e varejistas, sujeitas ao regime de apuração não cumulativa do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, §§ 3º e 4º). As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+MATÉRIAS-PRIMAS, PRODUTOS INTERMEDIÁRIOS E MATERIAIS DE EMBALAGEM - São reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas decorrentes da comercialização de matérias-primas, produtos intermediários e materiais de embalagem, produzidos na Zona Franca de Manaus para emprego em processo de industrialização por estabelecimentos industriais dos regimes cumulativo ou não cumulativo ali instalados, consoante projetos aprovados pelo Conselho de Administração da Superintendência da Zona Franca de Manaus (SUFRAMA) (Lei nº 10.637/2002, artigo 5º-A).
+REGIME NÃO CUMULATIVO - As alíquotas especiais para vendas realizadas por pessoa jurídica optante pelo regime não cumulativo estabelecida na Zona Franca de Manaus estão dispostas abaixo do item "Solução de Consulta".</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>2710.19.32</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Observações (Regra Geral)</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr"/>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>REGRA GERAL - O código NCM pesquisado não se encontra dentre os produtos com benefícios fiscais de PIS e COFINS previstos em legislação. Antes de aplicar as alíquotas correspondentes ao regime tributário da pessoa jurídica é recomendado analisar as outras guias.
+CONDIÇÃO DO ADQUIRENTE - Antes de aplicar a alíquota básica, é importante verificar se a pessoa jurídica adquirente é habilitada em algum regime especial, se está localizada na Zona Franca de Manaus (ZFM) ou em Área de Livre Comércio (ALC), e se a receita é proveniente de exportação de mercadorias.
+SIMPLES NACIONAL - A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+DARF - As empresas optantes pelo regime cumulativo recolherão o PIS e a COFINS em DARF, nos códigos 8109 e 2172, respectivamente.
+Para o regime não cumulativo os códigos serão 6912 e 5856.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>2710.19.32</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>ZFM - PIS</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr"/>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>2710.19.32</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr"/>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>2710.19.32</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>ZFM - Legislação</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr"/>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>2710.19.32</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>ZFM - Observações</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr"/>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+ZONA FRANCA DE MANAUS (ZFM) - Para os regimes cumulativo e não cumulativo, ficam reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas de vendas de mercadorias destinadas ao consumo (utilizadas diretamente ou para comercialização por atacado ou a varejo) ou à industrialização na Zona Franca de Manaus, por pessoa jurídica estabelecida fora da ZFM (Lei nº 10.996/2004, artigo 2º).
+Nas notas fiscais relativas à venda, deverá constar a expressão "Venda de mercadoria efetuada com alíquota zero da Contribuição para o PIS/Pasep e da COFINS - Lei nº 10.996/2004, artigo 2º".
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, terão a alíquota do PIS e da COFINS reduzidas a zero, exceto nas vendas de mercadorias que tenham como destinatárias pessoas jurídicas atacadistas e varejistas, sujeitas ao regime de apuração não cumulativa do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, §§ 3º e 4º). As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+MATÉRIAS-PRIMAS, PRODUTOS INTERMEDIÁRIOS E MATERIAIS DE EMBALAGEM - São reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas decorrentes da comercialização de matérias-primas, produtos intermediários e materiais de embalagem, produzidos na Zona Franca de Manaus para emprego em processo de industrialização por estabelecimentos industriais dos regimes cumulativo ou não cumulativo ali instalados, consoante projetos aprovados pelo Conselho de Administração da Superintendência da Zona Franca de Manaus (SUFRAMA) (Lei nº 10.637/2002, artigo 5º-A).
+REGIME NÃO CUMULATIVO - As alíquotas especiais para vendas realizadas por pessoa jurídica optante pelo regime não cumulativo estabelecida na Zona Franca de Manaus estão dispostas abaixo do item "Solução de Consulta".</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>3926.90.90</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Observações (Regra Geral)</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr"/>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>REGRA GERAL - O código NCM pesquisado pode enquadrar-se dentre os produtos com benefícios fiscais de PIS e COFINS previstos em legislação. Antes de aplicar as alíquotas correspondentes ao regime tributário da pessoa jurídica é recomendado analisar as outras guias.
+CONDIÇÃO DO ADQUIRENTE - Antes de aplicar a alíquota básica, é importante verificar se a pessoa jurídica adquirente é habilitada em algum regime especial, se está localizada na Zona Franca de Manaus (ZFM) ou em Área de Livre Comércio (ALC), e se a receita é proveniente de exportação de mercadorias.
+SIMPLES NACIONAL - A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+DARF - As empresas optantes pelo regime cumulativo recolherão o PIS e a COFINS em DARF, nos códigos 8109 e 2172, respectivamente.
+Para o regime não cumulativo os códigos serão 6912 e 5856.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>3926.90.90</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>ZFM - PIS</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr"/>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>3926.90.90</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr"/>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>3926.90.90</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>ZFM - Legislação</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr"/>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>3926.90.90</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>ZFM - Observações</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr"/>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+ZONA FRANCA DE MANAUS (ZFM) - Para os regimes cumulativo e não cumulativo, ficam reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas de vendas de mercadorias destinadas ao consumo (utilizadas diretamente ou para comercialização por atacado ou a varejo) ou à industrialização na Zona Franca de Manaus, por pessoa jurídica estabelecida fora da ZFM (Lei nº 10.996/2004, artigo 2º).
+Nas notas fiscais relativas à venda, deverá constar a expressão "Venda de mercadoria efetuada com alíquota zero da Contribuição para o PIS/Pasep e da COFINS - Lei nº 10.996/2004, artigo 2º".
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, terão a alíquota do PIS e da COFINS reduzidas a zero, exceto nas vendas de mercadorias que tenham como destinatárias pessoas jurídicas atacadistas e varejistas, sujeitas ao regime de apuração não cumulativa do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, §§ 3º e 4º). As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+MATÉRIAS-PRIMAS, PRODUTOS INTERMEDIÁRIOS E MATERIAIS DE EMBALAGEM - São reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas decorrentes da comercialização de matérias-primas, produtos intermediários e materiais de embalagem, produzidos na Zona Franca de Manaus para emprego em processo de industrialização por estabelecimentos industriais dos regimes cumulativo ou não cumulativo ali instalados, consoante projetos aprovados pelo Conselho de Administração da Superintendência da Zona Franca de Manaus (SUFRAMA) (Lei nº 10.637/2002, artigo 5º-A).
+REGIME NÃO CUMULATIVO - As alíquotas especiais para vendas realizadas por pessoa jurídica optante pelo regime não cumulativo estabelecida na Zona Franca de Manaus estão dispostas abaixo do item "Solução de Consulta".</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>9403.60.00</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Observações (Regra Geral)</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr"/>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>REGRA GERAL - O código NCM pesquisado pode enquadrar-se dentre os produtos com benefícios fiscais de PIS e COFINS previstos em legislação. Antes de aplicar as alíquotas correspondentes ao regime tributário da pessoa jurídica é recomendado analisar as outras guias.
+CONDIÇÃO DO ADQUIRENTE - Antes de aplicar a alíquota básica, é importante verificar se a pessoa jurídica adquirente é habilitada em algum regime especial, se está localizada na Zona Franca de Manaus (ZFM) ou em Área de Livre Comércio (ALC), e se a receita é proveniente de exportação de mercadorias.
+SIMPLES NACIONAL - A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+DARF - As empresas optantes pelo regime cumulativo recolherão o PIS e a COFINS em DARF, nos códigos 8109 e 2172, respectivamente.
+Para o regime não cumulativo os códigos serão 6912 e 5856.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>9403.60.00</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Suspensão - PIS</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr"/>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>9403.60.00</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Suspensão - COFINS</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr"/>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>9403.60.00</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Suspensão - Legislação</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr"/>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>9403.60.00</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Suspensão - Observações</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr"/>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da suspensão do PIS e da COFINS sobre as receitas de vendas de mercadorias, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+REGIME CUMULATIVO / NÃO CUMULATIVO - Aplica-se a suspensão do PIS e da COFINS nos casos de venda realizada a pessoa jurídica inscrita no Regime Especial de Tributação para Desenvolvimento da Atividade de Exibição Cinematográfica (RECINE) (Lei nº 12.599/2012, artigos 12 a 15; Decreto nº 7.729/2012).
+Prazo de vigência do benefício do RECINE: Até 31.12.2029 (Lei nº 13.594/2018).
+A partir de 01.04.2026, os incentivos e benefícios federais de natureza tributária são reduzidos, sendo aqueles de alíquota zero mediante a aplicação de alíquota correspondente a 10% da alíquota do sistema padrão de tributação. Desta forma, tendo em vista que para o PIS e a Cofins existem dois regimes de tributação, as alíquotas devem corresponder a 10% das alíquotas padrão de cada um dos regimes:
+a) Regime cumulativo - PIS: 0,065%; Cofins: 0,3%;
+b) Regime não cumulativo - PIS: 0,165%; Cofins: 0,76%. (Lei Complementar nº 224/2025, artigo 4º, caput e § 4º, inciso I)
+Ressalta-se que o § 1°, do artigo 2°, da IN RFB n° 2.305/2025 limita a redução dos benefícios àqueles discriminados no demonstrativo de gastos tributários anexo à Lei Orçamentária Anual de 2026. O Recine está discriminado, sofrendo redução do benefício.
+Quanto à aplicação da redução dos benefícios, no caso da suspensão, o artigo 6°, da IN RFB n° 2.305/2025 estabelece que a redução não se aplica aos benefícios de suspensão em que se verifique apenas um diferimento temporal no recolhimento do tributo. Logo, tendo em vista que o inciso II, do § 3°, do artigo 14, da Lei n° 12.599/2012 estabelece que a suspensão do PIS/Cofins converte-se em alíquota zero após a incorporação do bem ou material de construção no ativo imobilizado ou sua utilização no complexo de exibição cinematográfica ou cinema itinerante, situação na qual a operação fica sujeita à redução do benefício disposto na Lei Complementar nº 224/2025.
+Preventivamente, a sugestão é de que no cálculo para demonstrar o aumento da carga deve ser aplicado 10% das alíquotas do sistema padrão de PIS/Cofins sobre as vendas ou importação, baseado no artigo 7° da IN RFB 2.305/2025. Tal sugestão é um entendimento que poderá ser confirmado ou reformulado mediante esclarecimento da RFB.
+Visto que essas informações não estão claras na legislação, recomenda-se ao contribuinte buscar o serviço do Receita Soluciona, por meio das Confederações Nacionais de Representação de Categorias Econômicas, às Centrais Sindicais, aos Órgãos de Registro de Classe com atuação nacional e Organizações Associativas Patronais e Empresarias.</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>9403.60.00</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>ZFM - PIS</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr"/>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>9403.60.00</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr"/>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>9403.60.00</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>ZFM - Legislação</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr"/>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>9403.60.00</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>ZFM - Observações</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr"/>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+ZONA FRANCA DE MANAUS (ZFM) - Para os regimes cumulativo e não cumulativo, ficam reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas de vendas de mercadorias destinadas ao consumo (utilizadas diretamente ou para comercialização por atacado ou a varejo) ou à industrialização na Zona Franca de Manaus, por pessoa jurídica estabelecida fora da ZFM (Lei nº 10.996/2004, artigo 2º).
+Nas notas fiscais relativas à venda, deverá constar a expressão "Venda de mercadoria efetuada com alíquota zero da Contribuição para o PIS/Pasep e da COFINS - Lei nº 10.996/2004, artigo 2º".
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, terão a alíquota do PIS e da COFINS reduzidas a zero, exceto nas vendas de mercadorias que tenham como destinatárias pessoas jurídicas atacadistas e varejistas, sujeitas ao regime de apuração não cumulativa do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, §§ 3º e 4º). As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+MATÉRIAS-PRIMAS, PRODUTOS INTERMEDIÁRIOS E MATERIAIS DE EMBALAGEM - São reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas decorrentes da comercialização de matérias-primas, produtos intermediários e materiais de embalagem, produzidos na Zona Franca de Manaus para emprego em processo de industrialização por estabelecimentos industriais dos regimes cumulativo ou não cumulativo ali instalados, consoante projetos aprovados pelo Conselho de Administração da Superintendência da Zona Franca de Manaus (SUFRAMA) (Lei nº 10.637/2002, artigo 5º-A).
+REGIME NÃO CUMULATIVO - As alíquotas especiais para vendas realizadas por pessoa jurídica optante pelo regime não cumulativo estabelecida na Zona Franca de Manaus estão dispostas abaixo do item "Solução de Consulta".</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>8517.12.31</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Observações (Regra Geral)</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr"/>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>REGRA GERAL - O código NCM pesquisado pode enquadrar-se dentre os produtos com benefícios fiscais de PIS e COFINS previstos em legislação. Antes de aplicar as alíquotas correspondentes ao regime tributário da pessoa jurídica é recomendado analisar as outras guias.
+CONDIÇÃO DO ADQUIRENTE - Antes de aplicar a alíquota básica, é importante verificar se a pessoa jurídica adquirente é habilitada em algum regime especial, se está localizada na Zona Franca de Manaus (ZFM) ou em Área de Livre Comércio (ALC), e se a receita é proveniente de exportação de mercadorias.
+SIMPLES NACIONAL - A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+DARF - As empresas optantes pelo regime cumulativo recolherão o PIS e a COFINS em DARF, nos códigos 8109 e 2172, respectivamente.
+Para o regime não cumulativo os códigos serão 6912 e 5856.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>8517.12.31</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Suspensão - PIS</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr"/>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>8517.12.31</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Suspensão - COFINS</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr"/>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>8517.12.31</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Suspensão - Legislação</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr"/>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>8517.12.31</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Suspensão - Observações</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr"/>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da suspensão do PIS e da COFINS sobre as receitas de vendas de mercadorias, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+REGIME CUMULATIVO / NÃO CUMULATIVO - Aplica-se a suspensão do PIS e da COFINS nos casos de venda realizada a pessoa jurídica inscrita no Regime Especial de Tributação para Desenvolvimento da Atividade de Exibição Cinematográfica (RECINE) (Lei nº 12.599/2012, artigos 12 a 15; Decreto nº 7.729/2012).
+Prazo de vigência do benefício do RECINE: Até 31.12.2029 (Lei nº 13.594/2018).
+Também se aplica a suspensão no caso de venda de bens novos, destinados ao desenvolvimento, no País, de software e de serviços de tecnologia da informação, quando os referidos bens forem adquiridos por pessoa jurídica beneficiária do Regime Especial de Tributação para a Plataforma de Exportação de Serviços de Tecnologia da Informação (REPES) para incorporação ao seu ativo imobilizado (Lei nº 11.196/2005, artigos 4º e 11; Decreto nº 5.713/2006, artigo 1º).
+A partir de 01.04.2026, os incentivos e benefícios federais de natureza tributária são reduzidos, sendo aqueles de alíquota zero mediante a aplicação de alíquota correspondente a 10% da alíquota do sistema padrão de tributação. Desta forma, tendo em vista que para o PIS e a Cofins existem dois regimes de tributação, as alíquotas devem corresponder a 10% das alíquotas padrão de cada um dos regimes:
+a) Regime cumulativo - PIS: 0,065%; Cofins: 0,3%;
+b) Regime não cumulativo - PIS: 0,165%; Cofins: 0,76%. (Lei Complementar nº 224/2025, artigo 4º, caput e § 4º, inciso I)
+Ressalta-se que o § 1°, do artigo 2°, da IN RFB n° 2.305/2025 limita a redução dos benefícios àqueles discriminados no demonstrativo de gastos tributários anexo à Lei Orçamentária Anual de 2026. O Recine está discriminado, sofrendo redução do benefício.
+O Repes não está discriminado no demonstrativo de gastos tributários, não se sujeitando à redução estabelecida na Lei Complementar nº 224/2025.
+Quanto à aplicação da redução dos benefícios, no caso da suspensão, o artigo 6°, da IN RFB n° 2.305/2025 estabelece que a redução não se aplica aos benefícios de suspensão em que se verifique apenas um diferimento temporal no recolhimento do tributo. Logo, tendo em vista que o inciso II, do § 3°, do artigo 14, da Lei n° 12.599/2012 estabelece que a suspensão do PIS/Cofins converte-se em alíquota zero após a incorporação do bem ou material de construção no ativo imobilizado ou sua utilização no complexo de exibição cinematográfica ou cinema itinerante, situação na qual a operação fica sujeita à redução do benefício disposto na Lei Complementar nº 224/2025.
+Preventivamente, a sugestão é de que no cálculo para demonstrar o aumento da carga deve ser aplicado 10% das alíquotas do sistema padrão de PIS/Cofins sobre as vendas ou importação, baseado no artigo 7° da IN RFB 2.305/2025. Tal sugestão é um entendimento que poderá ser confirmado ou reformulado mediante esclarecimento da RFB.
+Visto que essas informações não estão claras na legislação, recomenda-se ao contribuinte buscar o serviço do Receita Soluciona, por meio das Confederações Nacionais de Representação de Categorias Econômicas, às Centrais Sindicais, aos Órgãos de Registro de Classe com atuação nacional e Organizações Associativas Patronais e Empresarias.</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>8517.12.31</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>ZFM - PIS</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr"/>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>8517.12.31</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr"/>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>8517.12.31</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>ZFM - Legislação</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr"/>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>8517.12.31</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>ZFM - Observações</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr"/>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+ZONA FRANCA DE MANAUS (ZFM) - Para os regimes cumulativo e não cumulativo, ficam reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas de vendas de mercadorias destinadas ao consumo (utilizadas diretamente ou para comercialização por atacado ou a varejo) ou à industrialização na Zona Franca de Manaus, por pessoa jurídica estabelecida fora da ZFM (Lei nº 10.996/2004, artigo 2º).
+Nas notas fiscais relativas à venda, deverá constar a expressão "Venda de mercadoria efetuada com alíquota zero da Contribuição para o PIS/Pasep e da COFINS - Lei nº 10.996/2004, artigo 2º".
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, terão a alíquota do PIS e da COFINS reduzidas a zero, exceto nas vendas de mercadorias que tenham como destinatárias pessoas jurídicas atacadistas e varejistas, sujeitas ao regime de apuração não cumulativa do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, §§ 3º e 4º). As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+MATÉRIAS-PRIMAS, PRODUTOS INTERMEDIÁRIOS E MATERIAIS DE EMBALAGEM - São reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas decorrentes da comercialização de matérias-primas, produtos intermediários e materiais de embalagem, produzidos na Zona Franca de Manaus para emprego em processo de industrialização por estabelecimentos industriais dos regimes cumulativo ou não cumulativo ali instalados, consoante projetos aprovados pelo Conselho de Administração da Superintendência da Zona Franca de Manaus (SUFRAMA) (Lei nº 10.637/2002, artigo 5º-A).
+REGIME NÃO CUMULATIVO - As alíquotas especiais para vendas realizadas por pessoa jurídica optante pelo regime não cumulativo estabelecida na Zona Franca de Manaus estão dispostas abaixo do item "Solução de Consulta".</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>0402.21.10</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Observações (Regra Geral)</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr"/>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+REGIME CUMULATIVO / NÃO CUMULATIVO - Aplica-se a alíquota zero do PIS e da COFINS à venda, no mercado interno, de (Lei nº 10.925/2004, artigo 1º, inciso XI):
+a) leite fluido pasteurizado ou industrializado, na forma de ultrapasteurizado, destinados ao consumo humano ou utilizados na industrialização de produtos que se destinam ao consumo humano;
+b) leite em pó, integral, semidesnatado ou desnatado, destinados ao consumo humano ou utilizados na industrialização de produtos que se destinam ao consumo humano;
+c) leite fermentado, bebidas e compostos lácteos e fórmulas infantis, assim definidas conforme previsão legal específica das instruções normativas do Ministério da Agricultura, Pecuária e Abastecimento, destinados ao consumo humano ou utilizados na industrialização de produtos que se destinam ao consumo humano.
+O benefício é aplicável apenas ao leite extraído de vacas. Portanto, não se aplica o benefício ao leite de cabra e seus derivados. (Soluções de Consulta Cosit n° 265/2023 e n° 44/2025)
+As definições de leite fermentado, bebidas e compostos lácteos e fórmulas infantis estão contidas nos seguintes dispositivos legais:
+- Leite Fermentado (Instrução Normativa MAPA nº 46/2007, Anexo, item 2.1);
+- Bebidas Lácteas (Instrução Normativa MAPA nº 16/2005, Anexo, item 2.1.1);
+- Compostos Lácteos (Instrução Normativa MAPA nº 28/2007, Anexo, item 2.1.1);
+- Fórmulas Infantis (Lei nº 11.265/2006, artigo 3º, incisos XVIII a XXI).
+Conforme o Acórdão DRJ/SPO (Delegacia da Receita Federal do Brasil de Julgamento em São Paulo) nº 1664862, de 22.01.2015, a venda de leite condensado e creme de leite não se enquadra na hipótese de alíquota zero prevista no artigo 1º, inciso XI, da Lei nº 10.925/2004).</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>0402.21.10</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>ZFM - PIS</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr"/>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>0402.21.10</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr"/>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>0402.21.10</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>ZFM - Legislação</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr"/>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2026-04-17 18:52</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>0402.21.10</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>ZFM - Observações</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr"/>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+ZONA FRANCA DE MANAUS (ZFM) - Para os regimes cumulativo e não cumulativo, ficam reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas de vendas de mercadorias destinadas ao consumo (utilizadas diretamente ou para comercialização por atacado ou a varejo) ou à industrialização na Zona Franca de Manaus, por pessoa jurídica estabelecida fora da ZFM (Lei nº 10.996/2004, artigo 2º).
+Nas notas fiscais relativas à venda, deverá constar a expressão "Venda de mercadoria efetuada com alíquota zero da Contribuição para o PIS/Pasep e da COFINS - Lei nº 10.996/2004, artigo 2º".
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, terão a alíquota do PIS e da COFINS reduzidas a zero, exceto nas vendas de mercadorias que tenham como destinatárias pessoas jurídicas atacadistas e varejistas, sujeitas ao regime de apuração não cumulativa do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, §§ 3º e 4º). As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+MATÉRIAS-PRIMAS, PRODUTOS INTERMEDIÁRIOS E MATERIAIS DE EMBALAGEM - São reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas decorrentes da comercialização de matérias-primas, produtos intermediários e materiais de embalagem, produzidos na Zona Franca de Manaus para emprego em processo de industrialização por estabelecimentos industriais dos regimes cumulativo ou não cumulativo ali instalados, consoante projetos aprovados pelo Conselho de Administração da Superintendência da Zona Franca de Manaus (SUFRAMA) (Lei nº 10.637/2002, artigo 5º-A).
+REGIME NÃO CUMULATIVO - As alíquotas especiais para vendas realizadas por pessoa jurídica optante pelo regime não cumulativo estabelecida na Zona Franca de Manaus estão dispostas abaixo do item "Solução de Consulta".</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: mudança na ordem das colunas da tabela do excel
</commit_message>
<xml_diff>
--- a/bcoDados.xlsx
+++ b/bcoDados.xlsx
@@ -605,142 +605,142 @@
       </c>
       <c r="W1" s="4" t="inlineStr">
         <is>
+          <t>Crédito Presumido - PIS</t>
+        </is>
+      </c>
+      <c r="X1" s="4" t="inlineStr">
+        <is>
+          <t>Crédito Presumido - COFINS</t>
+        </is>
+      </c>
+      <c r="Y1" s="4" t="inlineStr">
+        <is>
+          <t>Crédito Presumido - Legislação</t>
+        </is>
+      </c>
+      <c r="Z1" s="4" t="inlineStr">
+        <is>
+          <t>Crédito Presumido - Observações</t>
+        </is>
+      </c>
+      <c r="AA1" s="4" t="inlineStr">
+        <is>
           <t>Monofásico - Importador / Fabricante - PIS</t>
         </is>
       </c>
-      <c r="X1" s="4" t="inlineStr">
+      <c r="AB1" s="4" t="inlineStr">
         <is>
           <t>Monofásico - Importador / Fabricante - COFINS</t>
         </is>
       </c>
-      <c r="Y1" s="4" t="inlineStr">
+      <c r="AC1" s="4" t="inlineStr">
         <is>
           <t>Monofásico - Importador / Fabricante - Legislação</t>
         </is>
       </c>
-      <c r="Z1" s="4" t="inlineStr">
+      <c r="AD1" s="4" t="inlineStr">
         <is>
           <t>Monofásico - Importador / Fabricante - Observações</t>
         </is>
       </c>
-      <c r="AA1" s="4" t="inlineStr">
+      <c r="AE1" s="4" t="inlineStr">
         <is>
           <t>Monofásico - Atacado - PIS</t>
         </is>
       </c>
-      <c r="AB1" s="4" t="inlineStr">
+      <c r="AF1" s="4" t="inlineStr">
         <is>
           <t>Monofásico - Atacado - COFINS</t>
         </is>
       </c>
-      <c r="AC1" s="4" t="inlineStr">
+      <c r="AG1" s="4" t="inlineStr">
         <is>
           <t>Monofásico - Atacado - Legislação</t>
         </is>
       </c>
-      <c r="AD1" s="4" t="inlineStr">
+      <c r="AH1" s="4" t="inlineStr">
         <is>
           <t>Monofásico - Atacado - Observações</t>
         </is>
       </c>
-      <c r="AE1" s="4" t="inlineStr">
+      <c r="AI1" s="4" t="inlineStr">
         <is>
           <t>Monofásico - Varejo - PIS</t>
         </is>
       </c>
-      <c r="AF1" s="4" t="inlineStr">
+      <c r="AJ1" s="4" t="inlineStr">
         <is>
           <t>Monofásico - Varejo - COFINS</t>
         </is>
       </c>
-      <c r="AG1" s="4" t="inlineStr">
+      <c r="AK1" s="4" t="inlineStr">
         <is>
           <t>Monofásico - Varejo - Legislação</t>
         </is>
       </c>
-      <c r="AH1" s="4" t="inlineStr">
+      <c r="AL1" s="4" t="inlineStr">
         <is>
           <t>Monofásico - Varejo - Observações</t>
         </is>
       </c>
-      <c r="AI1" s="4" t="inlineStr">
+      <c r="AM1" s="4" t="inlineStr">
         <is>
           <t>ZFM - Monofásico - PIS</t>
         </is>
       </c>
-      <c r="AJ1" s="4" t="inlineStr">
+      <c r="AN1" s="4" t="inlineStr">
         <is>
           <t>ZFM - Monofásico - COFINS</t>
         </is>
       </c>
-      <c r="AK1" s="4" t="inlineStr">
+      <c r="AO1" s="4" t="inlineStr">
         <is>
           <t>ZFM - Monofásico - Legislação</t>
         </is>
       </c>
-      <c r="AL1" s="4" t="inlineStr">
+      <c r="AP1" s="4" t="inlineStr">
         <is>
           <t>ZFM - Monofásico - Observações</t>
         </is>
       </c>
-      <c r="AM1" s="4" t="inlineStr">
+      <c r="AQ1" s="4" t="inlineStr">
         <is>
           <t>Bebidas Frias - PIS</t>
         </is>
       </c>
-      <c r="AN1" s="4" t="inlineStr">
+      <c r="AR1" s="4" t="inlineStr">
         <is>
           <t>Bebidas Frias - COFINS</t>
         </is>
       </c>
-      <c r="AO1" s="4" t="inlineStr">
+      <c r="AS1" s="4" t="inlineStr">
         <is>
           <t>Bebidas Frias - Legislação</t>
         </is>
       </c>
-      <c r="AP1" s="4" t="inlineStr">
+      <c r="AT1" s="4" t="inlineStr">
         <is>
           <t>Bebidas Frias - Observações</t>
         </is>
       </c>
-      <c r="AQ1" s="4" t="inlineStr">
+      <c r="AU1" s="4" t="inlineStr">
         <is>
           <t>Bebidas Frias - Unid. de Medida - PIS</t>
         </is>
       </c>
-      <c r="AR1" s="4" t="inlineStr">
+      <c r="AV1" s="4" t="inlineStr">
         <is>
           <t>Bebidas Frias - Unid. de Medida - COFINS</t>
         </is>
       </c>
-      <c r="AS1" s="4" t="inlineStr">
+      <c r="AW1" s="4" t="inlineStr">
         <is>
           <t>Bebidas Frias - Unid. de Medida - Legislação</t>
         </is>
       </c>
-      <c r="AT1" s="4" t="inlineStr">
+      <c r="AX1" s="4" t="inlineStr">
         <is>
           <t>Bebidas Frias - Unid. de Medida - Observações</t>
-        </is>
-      </c>
-      <c r="AU1" s="4" t="inlineStr">
-        <is>
-          <t>Crédito Presumido - PIS</t>
-        </is>
-      </c>
-      <c r="AV1" s="4" t="inlineStr">
-        <is>
-          <t>Crédito Presumido - COFINS</t>
-        </is>
-      </c>
-      <c r="AW1" s="4" t="inlineStr">
-        <is>
-          <t>Crédito Presumido - Legislação</t>
-        </is>
-      </c>
-      <c r="AX1" s="4" t="inlineStr">
-        <is>
-          <t>Crédito Presumido - Observações</t>
         </is>
       </c>
     </row>
@@ -966,10 +966,10 @@
 O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
         </is>
       </c>
-      <c r="K3" s="1" t="inlineStr"/>
-      <c r="L3" s="1" t="inlineStr"/>
-      <c r="M3" s="1" t="inlineStr"/>
-      <c r="N3" s="1" t="inlineStr"/>
+      <c r="K3" s="1" t="n"/>
+      <c r="L3" s="1" t="n"/>
+      <c r="M3" s="1" t="n"/>
+      <c r="N3" s="1" t="n"/>
       <c r="O3" s="1" t="inlineStr">
         <is>
           <t>Vide observações</t>
@@ -1124,10 +1124,10 @@
 O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
         </is>
       </c>
-      <c r="K4" s="1" t="inlineStr"/>
-      <c r="L4" s="1" t="inlineStr"/>
-      <c r="M4" s="1" t="inlineStr"/>
-      <c r="N4" s="1" t="inlineStr"/>
+      <c r="K4" s="1" t="n"/>
+      <c r="L4" s="1" t="n"/>
+      <c r="M4" s="1" t="n"/>
+      <c r="N4" s="1" t="n"/>
       <c r="O4" s="1" t="inlineStr">
         <is>
           <t>Vide observações</t>
@@ -1267,10 +1267,10 @@
 O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
         </is>
       </c>
-      <c r="K5" s="1" t="inlineStr"/>
-      <c r="L5" s="1" t="inlineStr"/>
-      <c r="M5" s="1" t="inlineStr"/>
-      <c r="N5" s="1" t="inlineStr"/>
+      <c r="K5" s="1" t="n"/>
+      <c r="L5" s="1" t="n"/>
+      <c r="M5" s="1" t="n"/>
+      <c r="N5" s="1" t="n"/>
       <c r="O5" s="1" t="inlineStr">
         <is>
           <t>Vide observações</t>
@@ -1313,22 +1313,26 @@
       <c r="T5" s="1" t="n"/>
       <c r="U5" s="1" t="n"/>
       <c r="V5" s="1" t="n"/>
-      <c r="W5" s="1" t="inlineStr">
+      <c r="W5" s="1" t="n"/>
+      <c r="X5" s="1" t="n"/>
+      <c r="Y5" s="1" t="n"/>
+      <c r="Z5" s="1" t="n"/>
+      <c r="AA5" s="1" t="inlineStr">
         <is>
           <t>2,00%</t>
         </is>
       </c>
-      <c r="X5" s="1" t="inlineStr">
+      <c r="AB5" s="1" t="inlineStr">
         <is>
           <t>9,60%</t>
         </is>
       </c>
-      <c r="Y5" s="1" t="inlineStr">
+      <c r="AC5" s="1" t="inlineStr">
         <is>
           <t>Lei Complementar nº 123/2006; Lei nº 10.485/2002, artigo 1º</t>
         </is>
       </c>
-      <c r="Z5" s="1" t="inlineStr">
+      <c r="AD5" s="1" t="inlineStr">
         <is>
           <t>CONCEITO DE INCIDÊNCIA MONOFÁSICA - O sistema de tributação monofásica é um tratamento tributário próprio e específico, previsto em relação ao PIS e a COFINS incidentes sobre a receita bruta decorrente da venda de determinados produtos, geralmente a fim de concentrar a tributação nas etapas de produção e importação, desonerando as etapas subsequentes de comercialização.
 A concentração da tributação ocorre com a aplicação de alíquotas maiores que as usualmente aplicadas na tributação das demais receitas.
@@ -1351,22 +1355,22 @@
 O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
         </is>
       </c>
-      <c r="AA5" s="1" t="inlineStr">
-        <is>
-          <t>Vide observações</t>
-        </is>
-      </c>
-      <c r="AB5" s="1" t="inlineStr">
-        <is>
-          <t>Vide observações</t>
-        </is>
-      </c>
-      <c r="AC5" s="1" t="inlineStr">
+      <c r="AE5" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="AF5" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="AG5" s="1" t="inlineStr">
         <is>
           <t>Lei Complementar nº 123/2006</t>
         </is>
       </c>
-      <c r="AD5" s="1" t="inlineStr">
+      <c r="AH5" s="1" t="inlineStr">
         <is>
           <t>CONCEITO DE INCIDÊNCIA MONOFÁSICA - O sistema de tributação monofásica é um tratamento tributário próprio e específico, previsto em relação ao PIS e a COFINS incidentes sobre a receita bruta decorrente da venda de determinados produtos, geralmente a fim de concentrar a tributação nas etapas de produção e importação, desonerando as etapas subsequentes de comercialização.
 A concentração da tributação ocorre com a aplicação de alíquotas maiores que as usualmente aplicadas na tributação das demais receitas.
@@ -1377,22 +1381,22 @@
 PRODUTOS USADOS - Os produtos usados não estão sujeitos a incidência monofásica do PIS e da COFINS (Lei nº 10.485/2002, artigo 6º).</t>
         </is>
       </c>
-      <c r="AE5" s="1" t="inlineStr">
-        <is>
-          <t>Vide observações</t>
-        </is>
-      </c>
-      <c r="AF5" s="1" t="inlineStr">
-        <is>
-          <t>Vide observações</t>
-        </is>
-      </c>
-      <c r="AG5" s="1" t="inlineStr">
+      <c r="AI5" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="AJ5" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="AK5" s="1" t="inlineStr">
         <is>
           <t>Lei Complementar nº 123/2006</t>
         </is>
       </c>
-      <c r="AH5" s="1" t="inlineStr">
+      <c r="AL5" s="1" t="inlineStr">
         <is>
           <t>CONCEITO DE INCIDÊNCIA MONOFÁSICA - O sistema de tributação monofásica é um tratamento tributário próprio e específico, previsto em relação ao PIS e a COFINS incidentes sobre a receita bruta decorrente da venda de determinados produtos, geralmente a fim de concentrar a tributação nas etapas de produção e importação, desonerando as etapas subsequentes de comercialização.
 A concentração da tributação ocorre com a aplicação de alíquotas maiores que as usualmente aplicadas na tributação das demais receitas.
@@ -1403,22 +1407,22 @@
 PRODUTOS USADOS - Os produtos usados não estão sujeitos a incidência monofásica do PIS e da COFINS (Lei nº 10.485/2002, artigo 6º).</t>
         </is>
       </c>
-      <c r="AI5" s="1" t="inlineStr">
-        <is>
-          <t>Vide observações</t>
-        </is>
-      </c>
-      <c r="AJ5" s="1" t="inlineStr">
-        <is>
-          <t>Vide observações</t>
-        </is>
-      </c>
-      <c r="AK5" s="1" t="inlineStr">
+      <c r="AM5" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="AN5" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="AO5" s="1" t="inlineStr">
         <is>
           <t>Lei nº 10.485/2002, artigo 1º; Lei nº 11.196/2005, artigo 65</t>
         </is>
       </c>
-      <c r="AL5" s="1" t="inlineStr">
+      <c r="AP5" s="1" t="inlineStr">
         <is>
           <t>ALÍQUOTA - O fabricante ou importador dos produtos monofásicos citados no artigo 65 da Lei nº 11.196/2005 estabelecido fora da ZFM, fica obrigado a cobrar e recolher como substituto tributário o PIS e a COFINS devidos pela pessoa jurídica estabelecida na ZFM.
 Até 24.09.2020, as alíquotas eram de 2% (PIS) e de 9,6% (COFINS) (Lei nº 11.196/2005, artigo 65, § 1º, inciso III e Lei nº 10.485/2002, artigo 1º).
@@ -1441,10 +1445,6 @@
 O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
         </is>
       </c>
-      <c r="AM5" s="1" t="n"/>
-      <c r="AN5" s="1" t="n"/>
-      <c r="AO5" s="1" t="n"/>
-      <c r="AP5" s="1" t="n"/>
       <c r="AQ5" s="1" t="n"/>
       <c r="AR5" s="1" t="n"/>
       <c r="AS5" s="1" t="n"/>
@@ -1493,7 +1493,7 @@
           <t>Bebidas Frias (Monofásico)</t>
         </is>
       </c>
-      <c r="I6" s="1" t="inlineStr"/>
+      <c r="I6" s="1" t="n"/>
       <c r="J6" s="1" t="inlineStr">
         <is>
           <t>CONCEITO DE INCIDÊNCIA MONOFÁSICA - As bebidas frias listadas no artigo 14 da Lei nº 13.097/2015 estão sujeitas a incidência monofásica, conforme prevê o artigo 25 da referida Lei. O sistema de tributação monofásica é um tratamento tributário próprio e específico, previsto em relação ao PIS e a COFINS incidentes sobre a receita bruta decorrente da venda de determinados produtos, onde usualmente a tributação ocorre de forma concentrada no produtor e importador, e no caso das bebidas frias ocorrerá também no atacadista, desonerando as etapas subsequentes de comercialização. A concentração da tributação ocorre com a aplicação de alíquotas maiores que as usualmente aplicadas na tributação das demais receitas.
@@ -1515,10 +1515,10 @@
 O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
         </is>
       </c>
-      <c r="K6" s="1" t="inlineStr"/>
-      <c r="L6" s="1" t="inlineStr"/>
-      <c r="M6" s="1" t="inlineStr"/>
-      <c r="N6" s="1" t="inlineStr"/>
+      <c r="K6" s="1" t="n"/>
+      <c r="L6" s="1" t="n"/>
+      <c r="M6" s="1" t="n"/>
+      <c r="N6" s="1" t="n"/>
       <c r="O6" s="1" t="inlineStr">
         <is>
           <t>Vide observações</t>
@@ -1547,10 +1547,29 @@
       <c r="T6" s="1" t="n"/>
       <c r="U6" s="1" t="n"/>
       <c r="V6" s="1" t="n"/>
-      <c r="W6" s="1" t="n"/>
-      <c r="X6" s="1" t="n"/>
-      <c r="Y6" s="1" t="n"/>
-      <c r="Z6" s="1" t="n"/>
+      <c r="W6" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="X6" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="Y6" s="1" t="inlineStr">
+        <is>
+          <t>Decreto nº 8.442/2015, artigo 25</t>
+        </is>
+      </c>
+      <c r="Z6" s="1" t="inlineStr">
+        <is>
+          <t>CONDIÇÃO - REGIME CUMULATIVO - Será concedido crédito presumido de PIS e COFINS à pessoa jurídica sujeita ao regime cumulativo (exceto a pessoa jurídica optante pelo Simples Nacional) em relação à aquisição no mercado interno do produto pesquisado, a depender do regime tributário do vendedor, nos termos dispostos abaixo.
+ALÍQUOTAS - AQUISIÇÕES DO LUCRO PRESUMIDO / REAL - A pessoa jurídica sujeita ao regime de apuração cumulativa (exceto a pessoa jurídica optante pelo Simples Nacional) poderá descontar crédito presumido do PIS e COFINS em relação à aquisição no mercado interno do produto pesquisado, conforme os valores informados na nota fiscal do vendedor (Decreto nº 8.442/2015, artigos 25).
+ALÍQUOTAS - AQUISIÇÕES DO SIMPLES NACIONAL - Nas aquisições de produtos de pessoa jurídica optante pelo Simples Nacional, os créditos presumidos serão calculados mediante a aplicação sobre o valor de aquisição constante do documento fiscal o percentual correspondente a 0,38% (PIS) e 1,60% (COFINS) (Decreto nº 8.442/2015, artigos 25 e 29).
+VEDAÇÃO AO CRÉDITO - Não será permitido a utilização do crédito presumido pela pessoa jurídica varejista, em relação ao produto revendido com a aplicação da alíquota zero, de acordo com o artigo 27 do Decreto nº 8.442/2015.</t>
+        </is>
+      </c>
       <c r="AA6" s="1" t="n"/>
       <c r="AB6" s="1" t="n"/>
       <c r="AC6" s="1" t="n"/>
@@ -1563,10 +1582,14 @@
       <c r="AJ6" s="1" t="n"/>
       <c r="AK6" s="1" t="n"/>
       <c r="AL6" s="1" t="n"/>
-      <c r="AM6" s="1" t="inlineStr"/>
-      <c r="AN6" s="1" t="inlineStr"/>
-      <c r="AO6" s="1" t="inlineStr"/>
-      <c r="AP6" s="1" t="inlineStr">
+      <c r="AM6" s="1" t="n"/>
+      <c r="AN6" s="1" t="n"/>
+      <c r="AO6" s="1" t="n"/>
+      <c r="AP6" s="1" t="n"/>
+      <c r="AQ6" s="1" t="n"/>
+      <c r="AR6" s="1" t="n"/>
+      <c r="AS6" s="1" t="n"/>
+      <c r="AT6" s="1" t="inlineStr">
         <is>
           <t>CONCEITO DE INCIDÊNCIA MONOFÁSICA - As bebidas frias listadas no artigo 14 da Lei nº 13.097/2015 estão sujeitas a incidência monofásica, conforme prevê o artigo 25 da referida Lei. O sistema de tributação monofásica é um tratamento tributário próprio e específico, previsto em relação ao PIS e a COFINS incidentes sobre a receita bruta decorrente da venda de determinados produtos, onde usualmente a tributação ocorre de forma concentrada no produtor e importador, e no caso das bebidas frias ocorrerá também no atacadista, desonerando as etapas subsequentes de comercialização. A concentração da tributação ocorre com a aplicação de alíquotas maiores que as usualmente aplicadas na tributação das demais receitas.
 Em relação aos produtos classificados nas posições 22.01 e 22.02 da Tipi, o alcance da incidência monofásica é exclusivamente para água e refrigerantes, refrescos, cerveja sem álcool, repositores hidroeletrolíticos, bebidas energéticas e compostos líquidos prontos para o consumo que contenham como ingrediente principal inositol, glucoronolactona, taurina ou cafeína, segundo o parágrafo único do artigo 1º do Decreto nº 8.442/2015.
@@ -1587,37 +1610,14 @@
 O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
         </is>
       </c>
-      <c r="AQ6" s="1" t="inlineStr"/>
-      <c r="AR6" s="1" t="inlineStr"/>
-      <c r="AS6" s="1" t="inlineStr"/>
-      <c r="AT6" s="1" t="inlineStr">
+      <c r="AU6" s="1" t="n"/>
+      <c r="AV6" s="1" t="n"/>
+      <c r="AW6" s="1" t="n"/>
+      <c r="AX6" s="1" t="inlineStr">
         <is>
           <t>RECOLHIMENTO - São responsáveis pelo recolhimento do PIS e da COFINS, os importadores, fabricantes e atacadistas dos produtos relacionados no artigo 14 da Lei nº 13.097/2015.
 SIMPLES NACIONAL - A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento, pois neste regime tributário não caberá a aplicação das alíquotas correspondentes à incidência monofásica em função do disposto no artigo 25, § 2º da Lei nº 13.097/2015.
 Cabe destacar que a atividade de produção e venda no atacado de bebidas alcoólicas estava vedada terminantemente ao Simples Nacional até 31/12/2017, passando a ser autorizada nos casos excepcionais de produção ou venda no atacado por micro e pequenos produtores. A atividade de produção e venda no atacado de cervejas sem álcool permanecerá vedada mesmo após 31/12/2017 (Lei Complementar nº 123/2006, artigo 17, inciso X, alíneas "b" e "c").</t>
-        </is>
-      </c>
-      <c r="AU6" s="1" t="inlineStr">
-        <is>
-          <t>Vide observações</t>
-        </is>
-      </c>
-      <c r="AV6" s="1" t="inlineStr">
-        <is>
-          <t>Vide observações</t>
-        </is>
-      </c>
-      <c r="AW6" s="1" t="inlineStr">
-        <is>
-          <t>Decreto nº 8.442/2015, artigo 25</t>
-        </is>
-      </c>
-      <c r="AX6" s="1" t="inlineStr">
-        <is>
-          <t>CONDIÇÃO - REGIME CUMULATIVO - Será concedido crédito presumido de PIS e COFINS à pessoa jurídica sujeita ao regime cumulativo (exceto a pessoa jurídica optante pelo Simples Nacional) em relação à aquisição no mercado interno do produto pesquisado, a depender do regime tributário do vendedor, nos termos dispostos abaixo.
-ALÍQUOTAS - AQUISIÇÕES DO LUCRO PRESUMIDO / REAL - A pessoa jurídica sujeita ao regime de apuração cumulativa (exceto a pessoa jurídica optante pelo Simples Nacional) poderá descontar crédito presumido do PIS e COFINS em relação à aquisição no mercado interno do produto pesquisado, conforme os valores informados na nota fiscal do vendedor (Decreto nº 8.442/2015, artigos 25).
-ALÍQUOTAS - AQUISIÇÕES DO SIMPLES NACIONAL - Nas aquisições de produtos de pessoa jurídica optante pelo Simples Nacional, os créditos presumidos serão calculados mediante a aplicação sobre o valor de aquisição constante do documento fiscal o percentual correspondente a 0,38% (PIS) e 1,60% (COFINS) (Decreto nº 8.442/2015, artigos 25 e 29).
-VEDAÇÃO AO CRÉDITO - Não será permitido a utilização do crédito presumido pela pessoa jurídica varejista, em relação ao produto revendido com a aplicação da alíquota zero, de acordo com o artigo 27 do Decreto nº 8.442/2015.</t>
         </is>
       </c>
     </row>
@@ -1743,10 +1743,30 @@
       <c r="T7" s="1" t="n"/>
       <c r="U7" s="1" t="n"/>
       <c r="V7" s="1" t="n"/>
-      <c r="W7" s="1" t="n"/>
-      <c r="X7" s="1" t="n"/>
-      <c r="Y7" s="1" t="n"/>
-      <c r="Z7" s="1" t="n"/>
+      <c r="W7" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="X7" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="Y7" s="1" t="inlineStr">
+        <is>
+          <t>MP nº 1.034/2021, artigo 3º</t>
+        </is>
+      </c>
+      <c r="Z7" s="1" t="inlineStr">
+        <is>
+          <t>CONDIÇÃO - De 01.07.2021 à 14.07.2021 (período que vigou a MP nº 1.034/2021), a pessoa jurídica fabricante de conector 3 vias para infusão com torneira, de plástico, destinada ao uso em hospitais, clínicas, consultórios médicos e campanhas de vacinação, poderia deduzir crédito presumido na apuração do PIS e COFINS devidas em cada período de apuração (MP nº 1.034/2021, artigo 3º, caput e Anexo, item 43).
+Entretanto, o crédito presumido somente era aplicado aos insumos derivados de produtos da indústria petroquímica que eram beneficiados pelo Regime Especial da Indústria Química (REIQ), de que tratam os §§ 15, 16 e 23 do artigo 8º da Lei nº 10.865/2004, e os artigos 56 ao 57-B da Lei nº 11.196/2005, anteriormente à sua revogação, ou seja, até 30.06.2021; e os adquiridos a partir da revogação do REIQ em 01.07.2021 (MP nº 1.034/2021, artigo 3º, parágrafo único, incisos I e II e artigo 5º, inciso II).
+ALÍQUOTA - O crédito presumido era determinado mediante a aplicação das alíquotas de 0,65% (PIS) e 3% (COFINS) sobre (MP nº 1.034/2021, artigo 3º, caput e incisos I e II).
+a) o custo de aquisição, no caso de insumos nacionais adquiridos para fabricação dos produtos relacionados no item “Condição”; e
+b) o valor aduaneiro dos insumos por ela importados, no caso de insumos importados para fabricação dos produtos também relacionados no item “Condição”.</t>
+        </is>
+      </c>
       <c r="AA7" s="1" t="n"/>
       <c r="AB7" s="1" t="n"/>
       <c r="AC7" s="1" t="n"/>
@@ -1767,30 +1787,10 @@
       <c r="AR7" s="1" t="n"/>
       <c r="AS7" s="1" t="n"/>
       <c r="AT7" s="1" t="n"/>
-      <c r="AU7" s="1" t="inlineStr">
-        <is>
-          <t>Vide observações</t>
-        </is>
-      </c>
-      <c r="AV7" s="1" t="inlineStr">
-        <is>
-          <t>Vide observações</t>
-        </is>
-      </c>
-      <c r="AW7" s="1" t="inlineStr">
-        <is>
-          <t>MP nº 1.034/2021, artigo 3º</t>
-        </is>
-      </c>
-      <c r="AX7" s="1" t="inlineStr">
-        <is>
-          <t>CONDIÇÃO - De 01.07.2021 à 14.07.2021 (período que vigou a MP nº 1.034/2021), a pessoa jurídica fabricante de conector 3 vias para infusão com torneira, de plástico, destinada ao uso em hospitais, clínicas, consultórios médicos e campanhas de vacinação, poderia deduzir crédito presumido na apuração do PIS e COFINS devidas em cada período de apuração (MP nº 1.034/2021, artigo 3º, caput e Anexo, item 43).
-Entretanto, o crédito presumido somente era aplicado aos insumos derivados de produtos da indústria petroquímica que eram beneficiados pelo Regime Especial da Indústria Química (REIQ), de que tratam os §§ 15, 16 e 23 do artigo 8º da Lei nº 10.865/2004, e os artigos 56 ao 57-B da Lei nº 11.196/2005, anteriormente à sua revogação, ou seja, até 30.06.2021; e os adquiridos a partir da revogação do REIQ em 01.07.2021 (MP nº 1.034/2021, artigo 3º, parágrafo único, incisos I e II e artigo 5º, inciso II).
-ALÍQUOTA - O crédito presumido era determinado mediante a aplicação das alíquotas de 0,65% (PIS) e 3% (COFINS) sobre (MP nº 1.034/2021, artigo 3º, caput e incisos I e II).
-a) o custo de aquisição, no caso de insumos nacionais adquiridos para fabricação dos produtos relacionados no item “Condição”; e
-b) o valor aduaneiro dos insumos por ela importados, no caso de insumos importados para fabricação dos produtos também relacionados no item “Condição”.</t>
-        </is>
-      </c>
+      <c r="AU7" s="1" t="n"/>
+      <c r="AV7" s="1" t="n"/>
+      <c r="AW7" s="1" t="n"/>
+      <c r="AX7" s="1" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
@@ -2016,10 +2016,10 @@
 O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
         </is>
       </c>
-      <c r="K9" s="1" t="inlineStr"/>
-      <c r="L9" s="1" t="inlineStr"/>
-      <c r="M9" s="1" t="inlineStr"/>
-      <c r="N9" s="1" t="inlineStr"/>
+      <c r="K9" s="1" t="n"/>
+      <c r="L9" s="1" t="n"/>
+      <c r="M9" s="1" t="n"/>
+      <c r="N9" s="1" t="n"/>
       <c r="O9" s="1" t="inlineStr">
         <is>
           <t>Vide observações</t>
@@ -2065,20 +2065,45 @@
       <c r="V9" s="1" t="n"/>
       <c r="W9" s="1" t="inlineStr">
         <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="X9" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="Y9" s="1" t="inlineStr">
+        <is>
+          <t>Lei Complementar nº 123/2006</t>
+        </is>
+      </c>
+      <c r="Z9" s="1" t="inlineStr">
+        <is>
+          <t>CONDIÇÃO - Será concedido o regime especial de utilização de crédito presumido às pessoas jurídicas que procedam à industrialização ou à importação de medicamentos submetidos às alíquotas concentradas da Contribuição para o PIS e COFINS, sujeitos à prescrição médica e identificados por tarja vermelha ou preta, e que, visando assegurar a repercussão nos preços da redução da carga tributária tenham firmado com a União, compromisso de ajustamento de conduta, nos termos do § 6º do artigo 5º da Lei nº 7.347/85 ou que cumpram a sistemática estabelecida pela Câmara de Regulação do Mercado de Medicamentos (CMED) para utilização do crédito presumido na forma determinada pela Lei nº 10.742/2003 (Lei nº 10.147/2000, artigo 3º, § 2º).
+A concessão do regime especial depende de habilitação perante a CMED e a Receita Federal (RFB).
+ALÍQUOTA - O crédito presumido será determinado mediante a aplicação das alíquotas de 2,10% (PIS) e 9,90% (COFINS) sobre a receita bruta decorrente da venda desse medicamento (Lei nº 10.147/2000, artigo 3º, § 1º).
+A partir de 01/04/2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. No caso dos créditos presumidos, o aproveitamento fica limitado a 90% do valor original, sendo cancelada a parcela não utilizada. Desta forma, os contribuintes devem calcular o crédito presumido utilizando as alíquotas originais constantes na legislação, porém, apropriando valores correspondentes a 90% do crédito original. (Lei Complementar nº 224/2025, artigo 4º, caput e § 4º, inciso IV)
+REGIME CUMULATIVO / NÃO CUMULATIVO - São beneficiários do crédito presumido sobre o segmento farmacêutico as pessoas jurídicas que procedam à industrialização ou à importação dos produtos mencionados no artigo 3º da Lei nº 10.147/2000, optantes pelo regime cumulativo e não cumulativo.
+SIMPLES NACIONAL - Não é concedido crédito presumido as pessoas jurídicas optantes pelo Simples Nacional.</t>
+        </is>
+      </c>
+      <c r="AA9" s="1" t="inlineStr">
+        <is>
           <t>2,10%</t>
         </is>
       </c>
-      <c r="X9" s="1" t="inlineStr">
+      <c r="AB9" s="1" t="inlineStr">
         <is>
           <t>9,90%</t>
         </is>
       </c>
-      <c r="Y9" s="1" t="inlineStr">
+      <c r="AC9" s="1" t="inlineStr">
         <is>
           <t>Lei Complementar nº 123/2006; Lei nº 10.147/2000, artigo 1º, inciso I, alínea "a"</t>
         </is>
       </c>
-      <c r="Z9" s="1" t="inlineStr">
+      <c r="AD9" s="1" t="inlineStr">
         <is>
           <t>CONCEITO DE INCIDÊNCIA MONOFÁSICA - O sistema de tributação monofásica é um tratamento tributário próprio e específico, previsto em relação ao PIS e a COFINS incidentes sobre a receita bruta decorrente da venda de determinados produtos, geralmente a fim de concentrar a tributação nas etapas de produção e importação, desonerando as etapas subsequentes de comercialização.
 A concentração da tributação ocorre com a aplicação de alíquotas maiores que as usualmente aplicadas na tributação das demais receitas.
@@ -2100,22 +2125,22 @@
 O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
         </is>
       </c>
-      <c r="AA9" s="1" t="inlineStr">
-        <is>
-          <t>Vide observações</t>
-        </is>
-      </c>
-      <c r="AB9" s="1" t="inlineStr">
-        <is>
-          <t>Vide observações</t>
-        </is>
-      </c>
-      <c r="AC9" s="1" t="inlineStr">
+      <c r="AE9" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="AF9" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="AG9" s="1" t="inlineStr">
         <is>
           <t>Lei Complementar nº 123/2006</t>
         </is>
       </c>
-      <c r="AD9" s="1" t="inlineStr">
+      <c r="AH9" s="1" t="inlineStr">
         <is>
           <t>CONCEITO DE INCIDÊNCIA MONOFÁSICA - O sistema de tributação monofásica é um tratamento tributário próprio e específico, previsto em relação ao PIS e a COFINS incidentes sobre a receita bruta decorrente da venda de determinados produtos, geralmente a fim de concentrar a tributação nas etapas de produção e importação, desonerando as etapas subsequentes de comercialização.
 A concentração da tributação ocorre com a aplicação de alíquotas maiores que as usualmente aplicadas na tributação das demais receitas.
@@ -2125,22 +2150,22 @@
 REGIME CUMULATIVO / NÃO CUMULATIVO (COMÉRCIO) - Para as pessoas jurídicas não enquadradas na condição de industrial ou de importador, aplica-se a alíquota zero (Lei nº 10.147/2000, artigo 2º).</t>
         </is>
       </c>
-      <c r="AE9" s="1" t="inlineStr">
-        <is>
-          <t>Vide observações</t>
-        </is>
-      </c>
-      <c r="AF9" s="1" t="inlineStr">
-        <is>
-          <t>Vide observações</t>
-        </is>
-      </c>
-      <c r="AG9" s="1" t="inlineStr">
+      <c r="AI9" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="AJ9" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="AK9" s="1" t="inlineStr">
         <is>
           <t>Lei Complementar nº 123/2006</t>
         </is>
       </c>
-      <c r="AH9" s="1" t="inlineStr">
+      <c r="AL9" s="1" t="inlineStr">
         <is>
           <t>CONCEITO DE INCIDÊNCIA MONOFÁSICA - O sistema de tributação monofásica é um tratamento tributário próprio e específico, previsto em relação ao PIS e a COFINS incidentes sobre a receita bruta decorrente da venda de determinados produtos, geralmente a fim de concentrar a tributação nas etapas de produção e importação, desonerando as etapas subsequentes de comercialização.
 A concentração da tributação ocorre com a aplicação de alíquotas maiores que as usualmente aplicadas na tributação das demais receitas.
@@ -2150,10 +2175,6 @@
 REGIME CUMULATIVO / NÃO CUMULATIVO (COMÉRCIO) - Para as pessoas jurídicas não enquadradas na condição de industrial ou de importador, aplica-se a alíquota zero (Lei nº 10.147/2000, artigo 2º).</t>
         </is>
       </c>
-      <c r="AI9" s="1" t="n"/>
-      <c r="AJ9" s="1" t="n"/>
-      <c r="AK9" s="1" t="n"/>
-      <c r="AL9" s="1" t="n"/>
       <c r="AM9" s="1" t="n"/>
       <c r="AN9" s="1" t="n"/>
       <c r="AO9" s="1" t="n"/>
@@ -2162,31 +2183,10 @@
       <c r="AR9" s="1" t="n"/>
       <c r="AS9" s="1" t="n"/>
       <c r="AT9" s="1" t="n"/>
-      <c r="AU9" s="1" t="inlineStr">
-        <is>
-          <t>Vide observações</t>
-        </is>
-      </c>
-      <c r="AV9" s="1" t="inlineStr">
-        <is>
-          <t>Vide observações</t>
-        </is>
-      </c>
-      <c r="AW9" s="1" t="inlineStr">
-        <is>
-          <t>Lei Complementar nº 123/2006</t>
-        </is>
-      </c>
-      <c r="AX9" s="1" t="inlineStr">
-        <is>
-          <t>CONDIÇÃO - Será concedido o regime especial de utilização de crédito presumido às pessoas jurídicas que procedam à industrialização ou à importação de medicamentos submetidos às alíquotas concentradas da Contribuição para o PIS e COFINS, sujeitos à prescrição médica e identificados por tarja vermelha ou preta, e que, visando assegurar a repercussão nos preços da redução da carga tributária tenham firmado com a União, compromisso de ajustamento de conduta, nos termos do § 6º do artigo 5º da Lei nº 7.347/85 ou que cumpram a sistemática estabelecida pela Câmara de Regulação do Mercado de Medicamentos (CMED) para utilização do crédito presumido na forma determinada pela Lei nº 10.742/2003 (Lei nº 10.147/2000, artigo 3º, § 2º).
-A concessão do regime especial depende de habilitação perante a CMED e a Receita Federal (RFB).
-ALÍQUOTA - O crédito presumido será determinado mediante a aplicação das alíquotas de 2,10% (PIS) e 9,90% (COFINS) sobre a receita bruta decorrente da venda desse medicamento (Lei nº 10.147/2000, artigo 3º, § 1º).
-A partir de 01/04/2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. No caso dos créditos presumidos, o aproveitamento fica limitado a 90% do valor original, sendo cancelada a parcela não utilizada. Desta forma, os contribuintes devem calcular o crédito presumido utilizando as alíquotas originais constantes na legislação, porém, apropriando valores correspondentes a 90% do crédito original. (Lei Complementar nº 224/2025, artigo 4º, caput e § 4º, inciso IV)
-REGIME CUMULATIVO / NÃO CUMULATIVO - São beneficiários do crédito presumido sobre o segmento farmacêutico as pessoas jurídicas que procedam à industrialização ou à importação dos produtos mencionados no artigo 3º da Lei nº 10.147/2000, optantes pelo regime cumulativo e não cumulativo.
-SIMPLES NACIONAL - Não é concedido crédito presumido as pessoas jurídicas optantes pelo Simples Nacional.</t>
-        </is>
-      </c>
+      <c r="AU9" s="1" t="n"/>
+      <c r="AV9" s="1" t="n"/>
+      <c r="AW9" s="1" t="n"/>
+      <c r="AX9" s="1" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
@@ -2243,10 +2243,10 @@
 O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
         </is>
       </c>
-      <c r="K10" s="1" t="inlineStr"/>
-      <c r="L10" s="1" t="inlineStr"/>
-      <c r="M10" s="1" t="inlineStr"/>
-      <c r="N10" s="1" t="inlineStr"/>
+      <c r="K10" s="1" t="n"/>
+      <c r="L10" s="1" t="n"/>
+      <c r="M10" s="1" t="n"/>
+      <c r="N10" s="1" t="n"/>
       <c r="O10" s="1" t="inlineStr">
         <is>
           <t>Vide observações</t>
@@ -2371,10 +2371,10 @@
 REGIME CUMULATIVO / NÃO CUMULATIVO - Aplica-se à alíquota zero do PIS e da COFINS à receita bruta de venda no mercado interno (Lei nº 10.925/2004, artigo 1º, inciso V).</t>
         </is>
       </c>
-      <c r="K11" s="1" t="inlineStr"/>
-      <c r="L11" s="1" t="inlineStr"/>
-      <c r="M11" s="1" t="inlineStr"/>
-      <c r="N11" s="1" t="inlineStr"/>
+      <c r="K11" s="1" t="n"/>
+      <c r="L11" s="1" t="n"/>
+      <c r="M11" s="1" t="n"/>
+      <c r="N11" s="1" t="n"/>
       <c r="O11" s="1" t="inlineStr">
         <is>
           <t>Vide observações</t>
@@ -2437,10 +2437,31 @@
 REGIME CUMULATIVO / NÃO CUMULATIVO - Aplica-se à alíquota zero do PIS e da COFINS à receita bruta de venda no mercado interno (Lei nº 10.925/2004, artigo 1º, inciso V).</t>
         </is>
       </c>
-      <c r="W11" s="1" t="n"/>
-      <c r="X11" s="1" t="n"/>
-      <c r="Y11" s="1" t="n"/>
-      <c r="Z11" s="1" t="n"/>
+      <c r="W11" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="X11" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="Y11" s="1" t="inlineStr">
+        <is>
+          <t>Lei nº 10.925/2004, artigo 8°, caput, e § 1° e artigo 15, § 2º</t>
+        </is>
+      </c>
+      <c r="Z11" s="1" t="inlineStr">
+        <is>
+          <t>ALÍQUOTA - O crédito presumido será determinado mediante a aplicação das alíquotas de 0,5775% (PIS) e 2,66% (COFINS) sobre o valor de aquisição dos produtos agropecuários utilizados como insumo na fabricação do produto pesquisado quando este é destinado à alimentação humana ou animal.
+O crédito presumido será apurado no caso dos produtos agropecuários: (Lei n° 10.925/2004, artigo 8°, caput e § 1°)
+- adquiridos de pessoa jurídica domiciliada no País, com suspensão da exigibilidade das contribuições na forma dos artigos 560 e 561 da IN RFB nº 2.121/2022;
+- adquiridos de pessoa física residente no País; ou
+- recebidos de cooperado, pessoa física ou jurídica, residente ou domiciliada no País.
+SIMPLES NACIONAL / REGIME CUMULATIVO - Não é concedido crédito presumido as pessoas jurídicas optantes pelo Simples Nacional e para as que apurem o PIS e COFINS pelo regime cumulativo. O crédito presumido é concedido nas aquisições do produto pesquisado pela indústria do regime não cumulativo, desde que cumpridos os requisitos legais.</t>
+        </is>
+      </c>
       <c r="AA11" s="1" t="n"/>
       <c r="AB11" s="1" t="n"/>
       <c r="AC11" s="1" t="n"/>
@@ -2461,31 +2482,10 @@
       <c r="AR11" s="1" t="n"/>
       <c r="AS11" s="1" t="n"/>
       <c r="AT11" s="1" t="n"/>
-      <c r="AU11" s="1" t="inlineStr">
-        <is>
-          <t>Vide observações</t>
-        </is>
-      </c>
-      <c r="AV11" s="1" t="inlineStr">
-        <is>
-          <t>Vide observações</t>
-        </is>
-      </c>
-      <c r="AW11" s="1" t="inlineStr">
-        <is>
-          <t>Lei nº 10.925/2004, artigo 8°, caput, e § 1° e artigo 15, § 2º</t>
-        </is>
-      </c>
-      <c r="AX11" s="1" t="inlineStr">
-        <is>
-          <t>ALÍQUOTA - O crédito presumido será determinado mediante a aplicação das alíquotas de 0,5775% (PIS) e 2,66% (COFINS) sobre o valor de aquisição dos produtos agropecuários utilizados como insumo na fabricação do produto pesquisado quando este é destinado à alimentação humana ou animal.
-O crédito presumido será apurado no caso dos produtos agropecuários: (Lei n° 10.925/2004, artigo 8°, caput e § 1°)
-- adquiridos de pessoa jurídica domiciliada no País, com suspensão da exigibilidade das contribuições na forma dos artigos 560 e 561 da IN RFB nº 2.121/2022;
-- adquiridos de pessoa física residente no País; ou
-- recebidos de cooperado, pessoa física ou jurídica, residente ou domiciliada no País.
-SIMPLES NACIONAL / REGIME CUMULATIVO - Não é concedido crédito presumido as pessoas jurídicas optantes pelo Simples Nacional e para as que apurem o PIS e COFINS pelo regime cumulativo. O crédito presumido é concedido nas aquisições do produto pesquisado pela indústria do regime não cumulativo, desde que cumpridos os requisitos legais.</t>
-        </is>
-      </c>
+      <c r="AU11" s="1" t="n"/>
+      <c r="AV11" s="1" t="n"/>
+      <c r="AW11" s="1" t="n"/>
+      <c r="AX11" s="1" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
@@ -2548,10 +2548,10 @@
 O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
         </is>
       </c>
-      <c r="K12" s="1" t="inlineStr"/>
-      <c r="L12" s="1" t="inlineStr"/>
-      <c r="M12" s="1" t="inlineStr"/>
-      <c r="N12" s="1" t="inlineStr"/>
+      <c r="K12" s="1" t="n"/>
+      <c r="L12" s="1" t="n"/>
+      <c r="M12" s="1" t="n"/>
+      <c r="N12" s="1" t="n"/>
       <c r="O12" s="1" t="inlineStr">
         <is>
           <t>Vide observações</t>
@@ -2596,22 +2596,26 @@
       <c r="T12" s="1" t="n"/>
       <c r="U12" s="1" t="n"/>
       <c r="V12" s="1" t="n"/>
-      <c r="W12" s="1" t="inlineStr">
-        <is>
-          <t>Vide observações</t>
-        </is>
-      </c>
-      <c r="X12" s="1" t="inlineStr">
-        <is>
-          <t>Vide observações</t>
-        </is>
-      </c>
-      <c r="Y12" s="1" t="inlineStr">
+      <c r="W12" s="1" t="n"/>
+      <c r="X12" s="1" t="n"/>
+      <c r="Y12" s="1" t="n"/>
+      <c r="Z12" s="1" t="n"/>
+      <c r="AA12" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="AB12" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="AC12" s="1" t="inlineStr">
         <is>
           <t>Lei Complementar nº 123/2006; Lei nº 10.485/2002, artigos 1º e 3º</t>
         </is>
       </c>
-      <c r="Z12" s="1" t="inlineStr">
+      <c r="AD12" s="1" t="inlineStr">
         <is>
           <t>CONCEITO DE INCIDÊNCIA MONOFÁSICA - O sistema de tributação monofásica é um tratamento tributário próprio e específico, previsto em relação ao PIS e a COFINS incidentes sobre a receita bruta decorrente da venda de determinados produtos, geralmente a fim de concentrar a tributação nas etapas de produção e importação, desonerando as etapas subsequentes de comercialização.
 A concentração da tributação ocorre com a aplicação de alíquotas maiores que as usualmente aplicadas na tributação das demais receitas.
@@ -2636,22 +2640,22 @@
 O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
         </is>
       </c>
-      <c r="AA12" s="1" t="inlineStr">
-        <is>
-          <t>Vide observações</t>
-        </is>
-      </c>
-      <c r="AB12" s="1" t="inlineStr">
-        <is>
-          <t>Vide observações</t>
-        </is>
-      </c>
-      <c r="AC12" s="1" t="inlineStr">
+      <c r="AE12" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="AF12" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="AG12" s="1" t="inlineStr">
         <is>
           <t>Lei Complementar nº 123/2006</t>
         </is>
       </c>
-      <c r="AD12" s="1" t="inlineStr">
+      <c r="AH12" s="1" t="inlineStr">
         <is>
           <t>CONCEITO DE INCIDÊNCIA MONOFÁSICA - O sistema de tributação monofásica é um tratamento tributário próprio e específico, previsto em relação ao PIS e a COFINS incidentes sobre a receita bruta decorrente da venda de determinados produtos, geralmente a fim de concentrar a tributação nas etapas de produção e importação, desonerando as etapas subsequentes de comercialização.
 A concentração da tributação ocorre com a aplicação de alíquotas maiores que as usualmente aplicadas na tributação das demais receitas.
@@ -2662,22 +2666,22 @@
 PRODUTOS USADOS - Os produtos usados não estão sujeitos a incidência monofásica do PIS e da COFINS (Lei nº 10.485/2002, artigo 6º).</t>
         </is>
       </c>
-      <c r="AE12" s="1" t="inlineStr">
-        <is>
-          <t>Vide observações</t>
-        </is>
-      </c>
-      <c r="AF12" s="1" t="inlineStr">
-        <is>
-          <t>Vide observações</t>
-        </is>
-      </c>
-      <c r="AG12" s="1" t="inlineStr">
+      <c r="AI12" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="AJ12" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="AK12" s="1" t="inlineStr">
         <is>
           <t>Lei Complementar nº 123/2006</t>
         </is>
       </c>
-      <c r="AH12" s="1" t="inlineStr">
+      <c r="AL12" s="1" t="inlineStr">
         <is>
           <t>CONCEITO DE INCIDÊNCIA MONOFÁSICA - O sistema de tributação monofásica é um tratamento tributário próprio e específico, previsto em relação ao PIS e a COFINS incidentes sobre a receita bruta decorrente da venda de determinados produtos, geralmente a fim de concentrar a tributação nas etapas de produção e importação, desonerando as etapas subsequentes de comercialização.
 A concentração da tributação ocorre com a aplicação de alíquotas maiores que as usualmente aplicadas na tributação das demais receitas.
@@ -2688,22 +2692,22 @@
 PRODUTOS USADOS - Os produtos usados não estão sujeitos a incidência monofásica do PIS e da COFINS (Lei nº 10.485/2002, artigo 6º).</t>
         </is>
       </c>
-      <c r="AI12" s="1" t="inlineStr">
-        <is>
-          <t>Vide observações</t>
-        </is>
-      </c>
-      <c r="AJ12" s="1" t="inlineStr">
-        <is>
-          <t>Vide observações</t>
-        </is>
-      </c>
-      <c r="AK12" s="1" t="inlineStr">
+      <c r="AM12" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="AN12" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="AO12" s="1" t="inlineStr">
         <is>
           <t>Lei nº 10.485/2002, artigos 1º e 3º</t>
         </is>
       </c>
-      <c r="AL12" s="1" t="inlineStr">
+      <c r="AP12" s="1" t="inlineStr">
         <is>
           <t>VENDA A MONTADORAS DE VEÍCULOS - Não se aplica a substituição tributária na venda de autopeças, pneus novos e câmaras de ar para montadoras de veículos. (Lei nº 11.196/2005, artigo 65, § 6º).
 Não haverá crédito de PIS e COFINS nas aquisições feitas pelas montadoras de veículos estabelecidas na ZFM, pela compra dos referidos produtos, mesmo sendo a título de insumo ou imobilizado (Lei nº 11.196/2005, artigo 65, § 6º).
@@ -2728,10 +2732,6 @@
 O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
         </is>
       </c>
-      <c r="AM12" s="1" t="n"/>
-      <c r="AN12" s="1" t="n"/>
-      <c r="AO12" s="1" t="n"/>
-      <c r="AP12" s="1" t="n"/>
       <c r="AQ12" s="1" t="n"/>
       <c r="AR12" s="1" t="n"/>
       <c r="AS12" s="1" t="n"/>
@@ -2794,10 +2794,10 @@
 Também aplica-se a alíquota zero e sobre a receita bruta decorrente das saídas do estabelecimento industrial, na industrialização por conta e ordem de terceiros, dos bens e produtos classificados nas posições NCM 0103, 0105, 0203, 02.06.30.00, 0206.4, 0207 e 0210.1 (Lei nº 10.925/2004, artigo 1º, § 4º).</t>
         </is>
       </c>
-      <c r="K13" s="1" t="inlineStr"/>
-      <c r="L13" s="1" t="inlineStr"/>
-      <c r="M13" s="1" t="inlineStr"/>
-      <c r="N13" s="1" t="inlineStr"/>
+      <c r="K13" s="1" t="n"/>
+      <c r="L13" s="1" t="n"/>
+      <c r="M13" s="1" t="n"/>
+      <c r="N13" s="1" t="n"/>
       <c r="O13" s="1" t="inlineStr">
         <is>
           <t>Vide observações</t>
@@ -2861,10 +2861,28 @@
 Também aplica-se a alíquota zero e sobre a receita bruta decorrente das saídas do estabelecimento industrial, na industrialização por conta e ordem de terceiros, dos bens e produtos classificados nas posições NCM 0103, 0105, 0203, 02.06.30.00, 0206.4, 0207 e 0210.1 (Lei nº 10.925/2004, artigo 1º, § 4º).</t>
         </is>
       </c>
-      <c r="W13" s="1" t="n"/>
-      <c r="X13" s="1" t="n"/>
-      <c r="Y13" s="1" t="n"/>
-      <c r="Z13" s="1" t="n"/>
+      <c r="W13" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="X13" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="Y13" s="1" t="inlineStr">
+        <is>
+          <t>Lei nº 12.350/2010, artigo 56; MP nº 609/2013 (convertida na Lei nº 12.839/2013)</t>
+        </is>
+      </c>
+      <c r="Z13" s="1" t="inlineStr">
+        <is>
+          <t>CONDIÇÃO - REGIME NÃO CUMULATIVO - A pessoa jurídica tributada com base no lucro real que adquirir para industrialização produtos cuja comercialização seja fomentada com as alíquotas zero do PIS e COFINS previstas na alínea b (02.03, 0206.30.00, 0206.4, 02.07, 02.09 e 0210.1 e carne de frango classificada no código 0210.99.00) do inciso XIX do artigo 1º da Lei nº 10.865/2004, poderá descontar crédito presumido das referidas contribuições, devidas em cada período de apuração (Lei 12.350/2010, artigo 56).
+ALÍQUOTA - O crédito presumido será determinado mediante a aplicação das alíquotas de 0,1980% (PIS) e 0,9120% (COFINS), calculados conforme as disposições do item CONDIÇÃO - REGIME NÃO CUMULATIVO, mencionados anteriormente (Lei nº 12.350/2010, artigo 56).
+SIMPLES NACIONAL / REGIME CUMULATIVO - Não é concedido crédito presumido as pessoas jurídicas optantes pelo Simples Nacional e para as que apurem o PIS e COFINS pelo regime cumulativo. O crédito presumido é concedido nas aquisições do produto pesquisado pela indústria do regime não cumulativo, desde que cumpridos os requisitos legais.</t>
+        </is>
+      </c>
       <c r="AA13" s="1" t="n"/>
       <c r="AB13" s="1" t="n"/>
       <c r="AC13" s="1" t="n"/>
@@ -2885,28 +2903,10 @@
       <c r="AR13" s="1" t="n"/>
       <c r="AS13" s="1" t="n"/>
       <c r="AT13" s="1" t="n"/>
-      <c r="AU13" s="1" t="inlineStr">
-        <is>
-          <t>Vide observações</t>
-        </is>
-      </c>
-      <c r="AV13" s="1" t="inlineStr">
-        <is>
-          <t>Vide observações</t>
-        </is>
-      </c>
-      <c r="AW13" s="1" t="inlineStr">
-        <is>
-          <t>Lei nº 12.350/2010, artigo 56; MP nº 609/2013 (convertida na Lei nº 12.839/2013)</t>
-        </is>
-      </c>
-      <c r="AX13" s="1" t="inlineStr">
-        <is>
-          <t>CONDIÇÃO - REGIME NÃO CUMULATIVO - A pessoa jurídica tributada com base no lucro real que adquirir para industrialização produtos cuja comercialização seja fomentada com as alíquotas zero do PIS e COFINS previstas na alínea b (02.03, 0206.30.00, 0206.4, 02.07, 02.09 e 0210.1 e carne de frango classificada no código 0210.99.00) do inciso XIX do artigo 1º da Lei nº 10.865/2004, poderá descontar crédito presumido das referidas contribuições, devidas em cada período de apuração (Lei 12.350/2010, artigo 56).
-ALÍQUOTA - O crédito presumido será determinado mediante a aplicação das alíquotas de 0,1980% (PIS) e 0,9120% (COFINS), calculados conforme as disposições do item CONDIÇÃO - REGIME NÃO CUMULATIVO, mencionados anteriormente (Lei nº 12.350/2010, artigo 56).
-SIMPLES NACIONAL / REGIME CUMULATIVO - Não é concedido crédito presumido as pessoas jurídicas optantes pelo Simples Nacional e para as que apurem o PIS e COFINS pelo regime cumulativo. O crédito presumido é concedido nas aquisições do produto pesquisado pela indústria do regime não cumulativo, desde que cumpridos os requisitos legais.</t>
-        </is>
-      </c>
+      <c r="AU13" s="1" t="n"/>
+      <c r="AV13" s="1" t="n"/>
+      <c r="AW13" s="1" t="n"/>
+      <c r="AX13" s="1" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
@@ -2963,10 +2963,10 @@
 O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
         </is>
       </c>
-      <c r="K14" s="1" t="inlineStr"/>
-      <c r="L14" s="1" t="inlineStr"/>
-      <c r="M14" s="1" t="inlineStr"/>
-      <c r="N14" s="1" t="inlineStr"/>
+      <c r="K14" s="1" t="n"/>
+      <c r="L14" s="1" t="n"/>
+      <c r="M14" s="1" t="n"/>
+      <c r="N14" s="1" t="n"/>
       <c r="O14" s="1" t="inlineStr">
         <is>
           <t>Vide observações</t>
@@ -3034,10 +3034,29 @@
 b) Regime não cumulativo - PIS: 0,165%; Cofins: 0,76%. (Lei Complementar nº 224/2025, artigo 4º, caput e § 4º, inciso I)</t>
         </is>
       </c>
-      <c r="W14" s="1" t="n"/>
-      <c r="X14" s="1" t="n"/>
-      <c r="Y14" s="1" t="n"/>
-      <c r="Z14" s="1" t="n"/>
+      <c r="W14" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="X14" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="Y14" s="1" t="inlineStr">
+        <is>
+          <t>Lei nº 12.865/2013, artigo 31</t>
+        </is>
+      </c>
+      <c r="Z14" s="1" t="inlineStr">
+        <is>
+          <t>CONDIÇÃO - REGIME NÃO CUMULATIVO - CRÉDITO PRESUMIDO SOBRE A VENDA - Será concedido crédito presumido a pessoa jurídica que adota a modalidade não cumulativa do PIS e COFINS que realiza a venda no mercado interno ou da exportação do produto classificado no código 1507 da Tipi (Lei nº 12.865/2013, artigo 31).
+Do montante do crédito calculado, deve-se subtrair o valor resultante da aplicação das alíquotas de 0,4455% (PIS) e 2,052% (Cofins) sobre o valor de aquisição de óleo de soja classificado no código 15.07 da Tipi utilizado como insumo na produção de óleo de soja classificado no código 1507.90.1 da Tipi.
+OBS.: A subtração de crédito somente se aplica em caso de insumos adquiridos de pessoa jurídica.
+SIMPLES NACIONAL / REGIME CUMULATIVO - Não é concedido crédito presumido as pessoas jurídicas optantes pelo Simples Nacional e para as que apurem o PIS e COFINS pelo regime cumulativo. O crédito presumido é concedido na venda do produto pesquisado pelas pessoas jurídicas do regime não cumulativo.</t>
+        </is>
+      </c>
       <c r="AA14" s="1" t="n"/>
       <c r="AB14" s="1" t="n"/>
       <c r="AC14" s="1" t="n"/>
@@ -3058,29 +3077,10 @@
       <c r="AR14" s="1" t="n"/>
       <c r="AS14" s="1" t="n"/>
       <c r="AT14" s="1" t="n"/>
-      <c r="AU14" s="1" t="inlineStr">
-        <is>
-          <t>Vide observações</t>
-        </is>
-      </c>
-      <c r="AV14" s="1" t="inlineStr">
-        <is>
-          <t>Vide observações</t>
-        </is>
-      </c>
-      <c r="AW14" s="1" t="inlineStr">
-        <is>
-          <t>Lei nº 12.865/2013, artigo 31</t>
-        </is>
-      </c>
-      <c r="AX14" s="1" t="inlineStr">
-        <is>
-          <t>CONDIÇÃO - REGIME NÃO CUMULATIVO - CRÉDITO PRESUMIDO SOBRE A VENDA - Será concedido crédito presumido a pessoa jurídica que adota a modalidade não cumulativa do PIS e COFINS que realiza a venda no mercado interno ou da exportação do produto classificado no código 1507 da Tipi (Lei nº 12.865/2013, artigo 31).
-Do montante do crédito calculado, deve-se subtrair o valor resultante da aplicação das alíquotas de 0,4455% (PIS) e 2,052% (Cofins) sobre o valor de aquisição de óleo de soja classificado no código 15.07 da Tipi utilizado como insumo na produção de óleo de soja classificado no código 1507.90.1 da Tipi.
-OBS.: A subtração de crédito somente se aplica em caso de insumos adquiridos de pessoa jurídica.
-SIMPLES NACIONAL / REGIME CUMULATIVO - Não é concedido crédito presumido as pessoas jurídicas optantes pelo Simples Nacional e para as que apurem o PIS e COFINS pelo regime cumulativo. O crédito presumido é concedido na venda do produto pesquisado pelas pessoas jurídicas do regime não cumulativo.</t>
-        </is>
-      </c>
+      <c r="AU14" s="1" t="n"/>
+      <c r="AV14" s="1" t="n"/>
+      <c r="AW14" s="1" t="n"/>
+      <c r="AX14" s="1" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -3137,10 +3137,10 @@
 O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
         </is>
       </c>
-      <c r="K15" s="1" t="inlineStr"/>
-      <c r="L15" s="1" t="inlineStr"/>
-      <c r="M15" s="1" t="inlineStr"/>
-      <c r="N15" s="1" t="inlineStr"/>
+      <c r="K15" s="1" t="n"/>
+      <c r="L15" s="1" t="n"/>
+      <c r="M15" s="1" t="n"/>
+      <c r="N15" s="1" t="n"/>
       <c r="O15" s="1" t="inlineStr">
         <is>
           <t>Vide observações</t>
@@ -3268,10 +3268,10 @@
 O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
         </is>
       </c>
-      <c r="K16" s="1" t="inlineStr"/>
-      <c r="L16" s="1" t="inlineStr"/>
-      <c r="M16" s="1" t="inlineStr"/>
-      <c r="N16" s="1" t="inlineStr"/>
+      <c r="K16" s="1" t="n"/>
+      <c r="L16" s="1" t="n"/>
+      <c r="M16" s="1" t="n"/>
+      <c r="N16" s="1" t="n"/>
       <c r="O16" s="1" t="inlineStr">
         <is>
           <t>Vide observações</t>
@@ -3751,10 +3751,10 @@
 Conforme o Acórdão DRJ/SPO (Delegacia da Receita Federal do Brasil de Julgamento em São Paulo) nº 1664862, de 22.01.2015, a venda de leite condensado e creme de leite não se enquadra na hipótese de alíquota zero prevista no artigo 1º, inciso XI, da Lei nº 10.925/2004).</t>
         </is>
       </c>
-      <c r="K19" s="1" t="inlineStr"/>
-      <c r="L19" s="1" t="inlineStr"/>
-      <c r="M19" s="1" t="inlineStr"/>
-      <c r="N19" s="1" t="inlineStr"/>
+      <c r="K19" s="1" t="n"/>
+      <c r="L19" s="1" t="n"/>
+      <c r="M19" s="1" t="n"/>
+      <c r="N19" s="1" t="n"/>
       <c r="O19" s="1" t="inlineStr">
         <is>
           <t>Vide observações</t>
@@ -3827,10 +3827,31 @@
 Conforme o Acórdão DRJ/SPO (Delegacia da Receita Federal do Brasil de Julgamento em São Paulo) nº 1664862, de 22.01.2015, a venda de leite condensado e creme de leite não se enquadra na hipótese de alíquota zero prevista no artigo 1º, inciso XI, da Lei nº 10.925/2004).</t>
         </is>
       </c>
-      <c r="W19" s="1" t="n"/>
-      <c r="X19" s="1" t="n"/>
-      <c r="Y19" s="1" t="n"/>
-      <c r="Z19" s="1" t="n"/>
+      <c r="W19" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="X19" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="Y19" s="1" t="inlineStr">
+        <is>
+          <t>Lei nº 10.925/2004, artigo 8º; Lei nº 12.865/2013, artigo 30</t>
+        </is>
+      </c>
+      <c r="Z19" s="1" t="inlineStr">
+        <is>
+          <t>ALÍQUOTA - O crédito presumido será determinado mediante a aplicação das alíquotas de 0,99% (PIS) e 4,56% (COFINS) sobre o valor de aquisição dos produtos agropecuários utilizados como insumo na fabricação do produto pesquisado quando este é destinado à alimentação humana ou animal.
+O crédito presumido será apurado no caso dos produtos agropecuários:
+- adquiridos de pessoa jurídica domiciliada no País, com suspensão da exigibilidade das contribuições na forma dos artigos 560 e 561 da IN RFB nº 2.121/2022;
+- adquiridos de pessoa física residente no País; ou
+- recebidos de cooperado, pessoa física ou jurídica, residente ou domiciliada no País (Lei nº 10.925/2004, artigo 8º; Lei nº 12.865/2013, artigo 30).
+SIMPLES NACIONAL / REGIME CUMULATIVO - Não é concedido crédito presumido as pessoas jurídicas optantes pelo Simples Nacional e para as que apurem o PIS e COFINS pelo regime cumulativo. O crédito presumido é concedido nas aquisições do produto pesquisado pela indústria do regime não cumulativo, desde que cumpridos os requisitos legais.</t>
+        </is>
+      </c>
       <c r="AA19" s="1" t="n"/>
       <c r="AB19" s="1" t="n"/>
       <c r="AC19" s="1" t="n"/>
@@ -3851,31 +3872,10 @@
       <c r="AR19" s="1" t="n"/>
       <c r="AS19" s="1" t="n"/>
       <c r="AT19" s="1" t="n"/>
-      <c r="AU19" s="1" t="inlineStr">
-        <is>
-          <t>Vide observações</t>
-        </is>
-      </c>
-      <c r="AV19" s="1" t="inlineStr">
-        <is>
-          <t>Vide observações</t>
-        </is>
-      </c>
-      <c r="AW19" s="1" t="inlineStr">
-        <is>
-          <t>Lei nº 10.925/2004, artigo 8º; Lei nº 12.865/2013, artigo 30</t>
-        </is>
-      </c>
-      <c r="AX19" s="1" t="inlineStr">
-        <is>
-          <t>ALÍQUOTA - O crédito presumido será determinado mediante a aplicação das alíquotas de 0,99% (PIS) e 4,56% (COFINS) sobre o valor de aquisição dos produtos agropecuários utilizados como insumo na fabricação do produto pesquisado quando este é destinado à alimentação humana ou animal.
-O crédito presumido será apurado no caso dos produtos agropecuários:
-- adquiridos de pessoa jurídica domiciliada no País, com suspensão da exigibilidade das contribuições na forma dos artigos 560 e 561 da IN RFB nº 2.121/2022;
-- adquiridos de pessoa física residente no País; ou
-- recebidos de cooperado, pessoa física ou jurídica, residente ou domiciliada no País (Lei nº 10.925/2004, artigo 8º; Lei nº 12.865/2013, artigo 30).
-SIMPLES NACIONAL / REGIME CUMULATIVO - Não é concedido crédito presumido as pessoas jurídicas optantes pelo Simples Nacional e para as que apurem o PIS e COFINS pelo regime cumulativo. O crédito presumido é concedido nas aquisições do produto pesquisado pela indústria do regime não cumulativo, desde que cumpridos os requisitos legais.</t>
-        </is>
-      </c>
+      <c r="AU19" s="1" t="n"/>
+      <c r="AV19" s="1" t="n"/>
+      <c r="AW19" s="1" t="n"/>
+      <c r="AX19" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix: ajuste para pegar o nome mais completo do ncm
</commit_message>
<xml_diff>
--- a/bcoDados.xlsx
+++ b/bcoDados.xlsx
@@ -755,7 +755,7 @@
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>8471.41.00 — Que contenham, no mesmo corpo, pelo menos uma unidade central de processamento e, mesmo combinadas, uma unidade de entrada e uma unidade de saída</t>
+          <t>Máquinas automáticas para processamento de dados e suas unidades; leitores magnéticos ou ópticos, máquinas para registrar dados em suporte sob forma codificada, e máquinas para processamento desses dados, não especificadas nem compreendidas noutras posições — Que contenham, no mesmo corpo, pelo menos uma unidade central de processamento e, mesmo combinadas, uma unidade de entrada e uma unidade de saída</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
@@ -922,7 +922,7 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>3926.90.90 — Outras</t>
+          <t>Outras obras de plástico e obras de outras matérias das posições 39.01 a 39.14 — Outras</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
@@ -1080,7 +1080,7 @@
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>6109.10.00 — De algodão</t>
+          <t>Camisetas (T-shirts), camisetas interiores (camisolas interiores*), e artigos semelhantes, de malha — De algodão</t>
         </is>
       </c>
       <c r="D4" s="1" t="inlineStr">
@@ -1211,7 +1211,7 @@
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>8703.21.00 — De cilindrada não superior a 1.000 cm3</t>
+          <t>Automóveis de passageiros e outros veículos automóveis principalmente concebidos para transporte de pessoas (exceto os da posição 87.02), incluindo os veículos de uso misto (station wagons) e os automóveis de corrida — De cilindrada não superior a 1.000 cm3</t>
         </is>
       </c>
       <c r="D5" s="1" t="inlineStr">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>6 — Operação Tributável a Alíquota Zero.</t>
+          <t>Águas, incluindo as águas minerais e as águas gaseificadas, adicionadas de açúcar ou de outros edulcorantes ou aromatizadas e outras bebidas não alcoólicas, exceto sucos (sumos) de fruta ou de produtos hortícolas da posição 20.09 — Operação Tributável a Alíquota Zero.</t>
         </is>
       </c>
       <c r="D6" s="1" t="inlineStr">
@@ -1493,7 +1493,7 @@
           <t>Bebidas Frias (Monofásico)</t>
         </is>
       </c>
-      <c r="I6" s="1" t="n"/>
+      <c r="I6" s="1" t="inlineStr"/>
       <c r="J6" s="1" t="inlineStr">
         <is>
           <t>CONCEITO DE INCIDÊNCIA MONOFÁSICA - As bebidas frias listadas no artigo 14 da Lei nº 13.097/2015 estão sujeitas a incidência monofásica, conforme prevê o artigo 25 da referida Lei. O sistema de tributação monofásica é um tratamento tributário próprio e específico, previsto em relação ao PIS e a COFINS incidentes sobre a receita bruta decorrente da venda de determinados produtos, onde usualmente a tributação ocorre de forma concentrada no produtor e importador, e no caso das bebidas frias ocorrerá também no atacadista, desonerando as etapas subsequentes de comercialização. A concentração da tributação ocorre com a aplicação de alíquotas maiores que as usualmente aplicadas na tributação das demais receitas.
@@ -1586,9 +1586,9 @@
       <c r="AN6" s="1" t="n"/>
       <c r="AO6" s="1" t="n"/>
       <c r="AP6" s="1" t="n"/>
-      <c r="AQ6" s="1" t="n"/>
-      <c r="AR6" s="1" t="n"/>
-      <c r="AS6" s="1" t="n"/>
+      <c r="AQ6" s="1" t="inlineStr"/>
+      <c r="AR6" s="1" t="inlineStr"/>
+      <c r="AS6" s="1" t="inlineStr"/>
       <c r="AT6" s="1" t="inlineStr">
         <is>
           <t>CONCEITO DE INCIDÊNCIA MONOFÁSICA - As bebidas frias listadas no artigo 14 da Lei nº 13.097/2015 estão sujeitas a incidência monofásica, conforme prevê o artigo 25 da referida Lei. O sistema de tributação monofásica é um tratamento tributário próprio e específico, previsto em relação ao PIS e a COFINS incidentes sobre a receita bruta decorrente da venda de determinados produtos, onde usualmente a tributação ocorre de forma concentrada no produtor e importador, e no caso das bebidas frias ocorrerá também no atacadista, desonerando as etapas subsequentes de comercialização. A concentração da tributação ocorre com a aplicação de alíquotas maiores que as usualmente aplicadas na tributação das demais receitas.
@@ -1610,9 +1610,9 @@
 O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
         </is>
       </c>
-      <c r="AU6" s="1" t="n"/>
-      <c r="AV6" s="1" t="n"/>
-      <c r="AW6" s="1" t="n"/>
+      <c r="AU6" s="1" t="inlineStr"/>
+      <c r="AV6" s="1" t="inlineStr"/>
+      <c r="AW6" s="1" t="inlineStr"/>
       <c r="AX6" s="1" t="inlineStr">
         <is>
           <t>RECOLHIMENTO - São responsáveis pelo recolhimento do PIS e da COFINS, os importadores, fabricantes e atacadistas dos produtos relacionados no artigo 14 da Lei nº 13.097/2015.
@@ -1632,7 +1632,7 @@
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
-          <t>8481.80.99 — Outros</t>
+          <t>Torneiras, válvulas (incluindo as redutoras de pressão e as termostáticas) e dispositivos semelhantes, para canalizações, caldeiras, reservatórios, cubas e outros recipientes — Outros</t>
         </is>
       </c>
       <c r="D7" s="1" t="inlineStr">
@@ -1803,7 +1803,7 @@
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
-          <t>9403.60.00 — Outros móveis de madeira</t>
+          <t>Outros móveis e suas partes — Outros móveis de madeira</t>
         </is>
       </c>
       <c r="D8" s="1" t="inlineStr">
@@ -1961,7 +1961,7 @@
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
-          <t>3004.90.99 — Outros</t>
+          <t>Medicamentos (exceto os produtos das posições 30.02, 30.05 ou 30.06) constituídos por produtos misturados ou não misturados, preparados para fins terapêuticos ou profiláticos, apresentados em doses (incluindo os destinados a serem administrados por via percutânea) ou acondicionados para venda a retalho — Outros</t>
         </is>
       </c>
       <c r="D9" s="1" t="inlineStr">
@@ -2199,7 +2199,7 @@
       </c>
       <c r="C10" s="1" t="inlineStr">
         <is>
-          <t>8443.31.11 — De jato de tinta líquida, com largura de impressão inferior ou igual a 420 mm</t>
+          <t>Máquinas e aparelhos de impressão por meio de placas, cilindros e outros elementos de impressão da posição 84.42; outras impressoras, aparelhos de copiar e aparelhos de telecopiar (fax), mesmo combinados entre si; partes e acessórios — De jato de tinta líquida, com largura de impressão inferior ou igual a 420 mm</t>
         </is>
       </c>
       <c r="D10" s="1" t="inlineStr">
@@ -2330,7 +2330,7 @@
       </c>
       <c r="C11" s="1" t="inlineStr">
         <is>
-          <t>1006.30.21 — Polido ou brunido</t>
+          <t>Arroz — Polido ou brunido</t>
         </is>
       </c>
       <c r="D11" s="1" t="inlineStr">
@@ -2498,7 +2498,7 @@
       </c>
       <c r="C12" s="1" t="inlineStr">
         <is>
-          <t>8708.29.99 — Outros</t>
+          <t>Partes e acessórios dos veículos automóveis das posições 87.01 a 87.05 — Outros</t>
         </is>
       </c>
       <c r="D12" s="1" t="inlineStr">
@@ -2752,7 +2752,7 @@
       </c>
       <c r="C13" s="1" t="inlineStr">
         <is>
-          <t>0207.14.11 — Peitos</t>
+          <t>Carnes e miudezas, comestíveis, frescas, refrigeradas ou congeladas, das aves da posição 01.05 — Peitos</t>
         </is>
       </c>
       <c r="D13" s="1" t="inlineStr">
@@ -2919,7 +2919,7 @@
       </c>
       <c r="C14" s="1" t="inlineStr">
         <is>
-          <t>1507.90.11 — Em recipientes com capacidade inferior ou igual a 5 l</t>
+          <t>Óleo de soja e respectivas frações, mesmo refinados, mas não quimicamente modificados — Em recipientes com capacidade inferior ou igual a 5 l</t>
         </is>
       </c>
       <c r="D14" s="1" t="inlineStr">
@@ -3093,7 +3093,7 @@
       </c>
       <c r="C15" s="1" t="inlineStr">
         <is>
-          <t>2710.19.32 — Com aditivos</t>
+          <t>Óleos de petróleo ou de minerais betuminosos, exceto óleos brutos; preparações não especificadas nem compreendidas noutras posições, que contenham, como constituintes básicos, 70 % ou mais, em peso, de óleos de petróleo ou de minerais betuminosos; resíduos de óleos — Com aditivos</t>
         </is>
       </c>
       <c r="D15" s="1" t="inlineStr">
@@ -3224,7 +3224,7 @@
       </c>
       <c r="C16" s="1" t="inlineStr">
         <is>
-          <t>3926.90.90 — Outras</t>
+          <t>Outras obras de plástico e obras de outras matérias das posições 39.01 a 39.14 — Outras</t>
         </is>
       </c>
       <c r="D16" s="1" t="inlineStr">
@@ -3382,7 +3382,7 @@
       </c>
       <c r="C17" s="1" t="inlineStr">
         <is>
-          <t>9403.60.00 — Outros móveis de madeira</t>
+          <t>Outros móveis e suas partes — Outros móveis de madeira</t>
         </is>
       </c>
       <c r="D17" s="1" t="inlineStr">
@@ -3540,7 +3540,7 @@
       </c>
       <c r="C18" s="1" t="inlineStr">
         <is>
-          <t>8517.11.00 — Aparelhos telefônicos por fio com unidade auscultador-microfone sem fio</t>
+          <t>Aparelhos telefônicos, incluindo os telefones inteligentes (smartphones) e outros telefones para redes celulares ou para outras redes sem fio; outros aparelhos para a transmissão ou recepção de voz, imagens ou outros dados, incluindo os aparelhos para comunicação em redes por fio ou redes sem fio (tal como uma rede local (LAN) ou uma rede de área estendida (longa distância) (WAN)), exceto os aparelhos das posições 84.43, 85.25, 85.27 ou 85.28 — Aparelhos telefônicos por fio com unidade auscultador-microfone sem fio</t>
         </is>
       </c>
       <c r="D18" s="1" t="inlineStr">
@@ -3700,7 +3700,7 @@
       </c>
       <c r="C19" s="1" t="inlineStr">
         <is>
-          <t>0402.21.10 — Leite integral</t>
+          <t>Leite e creme de leite (nata), concentrados ou adicionados de açúcar ou de outros edulcorantes — Leite integral</t>
         </is>
       </c>
       <c r="D19" s="1" t="inlineStr">
@@ -3891,7 +3891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F251"/>
+  <dimension ref="A1:F269"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -11370,6 +11370,582 @@
         </is>
       </c>
     </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>2026-04-20 12:33</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>8471.41.90</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>8471.41.00 — Que contenham, no mesmo corpo, pelo menos uma unidade central de processamento e, mesmo combinadas, uma unidade de entrada e uma unidade de saída</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>Máquinas automáticas para processamento de dados e suas unidades; leitores magnéticos ou ópticos, máquinas para registrar dados em suporte sob forma codificada, e máquinas para processamento desses dados, não especificadas nem compreendidas noutras posições — Que contenham, no mesmo corpo, pelo menos uma unidade central de processamento e, mesmo combinadas, uma unidade de entrada e uma unidade de saída</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>2026-04-20 12:33</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>3926.90.90</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>3926.90.90 — Outras</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>Outras obras de plástico e obras de outras matérias das posições 39.01 a 39.14 — Outras</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>2026-04-20 12:33</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>6109.10.00</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>6109.10.00 — De algodão</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>Camisetas (T-shirts), camisetas interiores (camisolas interiores*), e artigos semelhantes, de malha — De algodão</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>2026-04-20 12:33</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>8703.21.10</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>8703.21.00 — De cilindrada não superior a 1.000 cm3</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>Automóveis de passageiros e outros veículos automóveis principalmente concebidos para transporte de pessoas (exceto os da posição 87.02), incluindo os veículos de uso misto (station wagons) e os automóveis de corrida — De cilindrada não superior a 1.000 cm3</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>2026-04-20 12:33</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>2202.10.00</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>6 — Operação Tributável a Alíquota Zero.</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>Águas, incluindo as águas minerais e as águas gaseificadas, adicionadas de açúcar ou de outros edulcorantes ou aromatizadas e outras bebidas não alcoólicas, exceto sucos (sumos) de fruta ou de produtos hortícolas da posição 20.09 — Operação Tributável a Alíquota Zero.</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>2026-04-20 12:33</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>8481.80.99</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>8481.80.99 — Outros</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>Torneiras, válvulas (incluindo as redutoras de pressão e as termostáticas) e dispositivos semelhantes, para canalizações, caldeiras, reservatórios, cubas e outros recipientes — Outros</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>2026-04-20 12:33</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>9403.60.90</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>9403.60.00 — Outros móveis de madeira</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>Outros móveis e suas partes — Outros móveis de madeira</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>2026-04-20 12:33</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>3004.90.99</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>3004.90.99 — Outros</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>Medicamentos (exceto os produtos das posições 30.02, 30.05 ou 30.06) constituídos por produtos misturados ou não misturados, preparados para fins terapêuticos ou profiláticos, apresentados em doses (incluindo os destinados a serem administrados por via percutânea) ou acondicionados para venda a retalho — Outros</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>2026-04-20 12:33</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>8443.31.00</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>8443.31.11 — De jato de tinta líquida, com largura de impressão inferior ou igual a 420 mm</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>Máquinas e aparelhos de impressão por meio de placas, cilindros e outros elementos de impressão da posição 84.42; outras impressoras, aparelhos de copiar e aparelhos de telecopiar (fax), mesmo combinados entre si; partes e acessórios — De jato de tinta líquida, com largura de impressão inferior ou igual a 420 mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>2026-04-20 12:33</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>1006.30.21</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>1006.30.21 — Polido ou brunido</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>Arroz — Polido ou brunido</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>2026-04-20 12:33</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>8708.29.99</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>8708.29.99 — Outros</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>Partes e acessórios dos veículos automóveis das posições 87.01 a 87.05 — Outros</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>2026-04-20 12:33</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>0207.14.00</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>0207.14.11 — Peitos</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>Carnes e miudezas, comestíveis, frescas, refrigeradas ou congeladas, das aves da posição 01.05 — Peitos</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>2026-04-20 12:33</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>1507.90.11</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>1507.90.11 — Em recipientes com capacidade inferior ou igual a 5 l</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>Óleo de soja e respectivas frações, mesmo refinados, mas não quimicamente modificados — Em recipientes com capacidade inferior ou igual a 5 l</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>2026-04-20 12:33</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>2710.19.32</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>2710.19.32 — Com aditivos</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>Óleos de petróleo ou de minerais betuminosos, exceto óleos brutos; preparações não especificadas nem compreendidas noutras posições, que contenham, como constituintes básicos, 70 % ou mais, em peso, de óleos de petróleo ou de minerais betuminosos; resíduos de óleos — Com aditivos</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>2026-04-20 12:33</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>3926.90.90</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>3926.90.90 — Outras</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>Outras obras de plástico e obras de outras matérias das posições 39.01 a 39.14 — Outras</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>2026-04-20 12:33</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>9403.60.00</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>9403.60.00 — Outros móveis de madeira</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>Outros móveis e suas partes — Outros móveis de madeira</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>2026-04-20 12:33</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>8517.12.31</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>8517.11.00 — Aparelhos telefônicos por fio com unidade auscultador-microfone sem fio</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>Aparelhos telefônicos, incluindo os telefones inteligentes (smartphones) e outros telefones para redes celulares ou para outras redes sem fio; outros aparelhos para a transmissão ou recepção de voz, imagens ou outros dados, incluindo os aparelhos para comunicação em redes por fio ou redes sem fio (tal como uma rede local (LAN) ou uma rede de área estendida (longa distância) (WAN)), exceto os aparelhos das posições 84.43, 85.25, 85.27 ou 85.28 — Aparelhos telefônicos por fio com unidade auscultador-microfone sem fio</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>2026-04-20 12:33</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>0402.21.10</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>0402.21.10 — Leite integral</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>Leite e creme de leite (nata), concentrados ou adicionados de açúcar ou de outros edulcorantes — Leite integral</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: ajuste para pegar o PIS/COFINS certo de ZFM
</commit_message>
<xml_diff>
--- a/bcoDados.xlsx
+++ b/bcoDados.xlsx
@@ -1006,10 +1006,14 @@
       </c>
       <c r="U2" s="1" t="inlineStr">
         <is>
-          <t>CRÉDITO ZONA FRANCA DE MANAUS - De acordo com o §§ 12, art. 3º da Lei nº 10.637/2002 e o § 17, art. 3º da Lei nº 10.833/2003, ressalvado o disposto no § 2° do referido artigo e nos §§ 1° a 3° do art. 2°, na aquisição de mercadoria produzida por pessoa jurídica estabelecida na ZFM, consoante projeto aprovado pela Suframa, o crédito será determinado mediante a aplicação da alíquota: PIS a) de alíquota de 1% e, b) de 1,65%, na situação de que trata a alínea ""b"" do inciso II do § 4° do art. 2° da Lei nº 10.637/2002. COFINS a) de 5,60%, nas operações com os bens referidos no inciso VI do art. 28 da Lei n° 11.196/2005; b) de 7,60%, na situação de que trata a alínea ""b"" do inciso II do § 5° do art. 2° desta Lei; e c) de 4,60%, nos demais casos. CRÉDITO ÁREA DE LIVRE COMÉRCIO - Segundo os §§ 15 e 16, art. 3º da Lei nº 10.637/2002 e §§ 23 e 24, art. 3º da Lei nº 10.833/2003, na hipótese de aquisição de mercadoria produzida por pessoa jurídica estabelecida nas Áreas de Livre Comércio, o crédito será determinado mediante a aplicação da alíquota: PIS - de 0,65%. COFINS - de 3%.</t>
-        </is>
-      </c>
-      <c r="V2" s="1" t="n"/>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="V2" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
       <c r="W2" s="1" t="n"/>
       <c r="X2" s="1" t="n"/>
       <c r="Y2" s="1" t="n"/>
@@ -1161,10 +1165,14 @@
       </c>
       <c r="U3" s="1" t="inlineStr">
         <is>
-          <t>CRÉDITO ZONA FRANCA DE MANAUS - De acordo com o §§ 12, art. 3º da Lei nº 10.637/2002 e o § 17, art. 3º da Lei nº 10.833/2003, ressalvado o disposto no § 2° do referido artigo e nos §§ 1° a 3° do art. 2°, na aquisição de mercadoria produzida por pessoa jurídica estabelecida na ZFM, consoante projeto aprovado pela Suframa, o crédito será determinado mediante a aplicação da alíquota: PIS a) de alíquota de 1% e, b) de 1,65%, na situação de que trata a alínea ""b"" do inciso II do § 4° do art. 2° da Lei nº 10.637/2002. COFINS a) de 5,60%, nas operações com os bens referidos no inciso VI do art. 28 da Lei n° 11.196/2005; b) de 7,60%, na situação de que trata a alínea ""b"" do inciso II do § 5° do art. 2° desta Lei; e c) de 4,60%, nos demais casos. CRÉDITO ÁREA DE LIVRE COMÉRCIO - Segundo os §§ 15 e 16, art. 3º da Lei nº 10.637/2002 e §§ 23 e 24, art. 3º da Lei nº 10.833/2003, na hipótese de aquisição de mercadoria produzida por pessoa jurídica estabelecida nas Áreas de Livre Comércio, o crédito será determinado mediante a aplicação da alíquota: PIS - de 0,65%. COFINS - de 3%.</t>
-        </is>
-      </c>
-      <c r="V3" s="1" t="n"/>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="V3" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
       <c r="W3" s="1" t="inlineStr">
         <is>
           <t>Cum: Lei nº 9.715/98, artigo 8º, inciso I; Lei nº 9.718/98, artigo 8º; Lei n° 10.865/2004, artigo 28, inciso XVII | N.Cum: Decreto nº 6.426/2008, artigo 1º, inciso III; Lei n° 10.865/2004, artigo 28, inciso XVII; Lei Complementar nº 224/2025</t>
@@ -1351,10 +1359,14 @@
       </c>
       <c r="U4" s="1" t="inlineStr">
         <is>
-          <t>CRÉDITO ZONA FRANCA DE MANAUS - De acordo com o §§ 12, art. 3º da Lei nº 10.637/2002 e o § 17, art. 3º da Lei nº 10.833/2003, ressalvado o disposto no § 2° do referido artigo e nos §§ 1° a 3° do art. 2°, na aquisição de mercadoria produzida por pessoa jurídica estabelecida na ZFM, consoante projeto aprovado pela Suframa, o crédito será determinado mediante a aplicação da alíquota: PIS a) de alíquota de 1% e, b) de 1,65%, na situação de que trata a alínea ""b"" do inciso II do § 4° do art. 2° da Lei nº 10.637/2002. COFINS a) de 5,60%, nas operações com os bens referidos no inciso VI do art. 28 da Lei n° 11.196/2005; b) de 7,60%, na situação de que trata a alínea ""b"" do inciso II do § 5° do art. 2° desta Lei; e c) de 4,60%, nos demais casos. CRÉDITO ÁREA DE LIVRE COMÉRCIO - Segundo os §§ 15 e 16, art. 3º da Lei nº 10.637/2002 e §§ 23 e 24, art. 3º da Lei nº 10.833/2003, na hipótese de aquisição de mercadoria produzida por pessoa jurídica estabelecida nas Áreas de Livre Comércio, o crédito será determinado mediante a aplicação da alíquota: PIS - de 0,65%. COFINS - de 3%.</t>
-        </is>
-      </c>
-      <c r="V4" s="1" t="n"/>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="V4" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
       <c r="W4" s="1" t="n"/>
       <c r="X4" s="1" t="n"/>
       <c r="Y4" s="1" t="n"/>
@@ -1641,7 +1653,7 @@
           <t>0,00%</t>
         </is>
       </c>
-      <c r="BA5" s="1" t="n"/>
+      <c r="BA5" s="1" t="inlineStr"/>
       <c r="BB5" s="1" t="inlineStr">
         <is>
           <t>ALÍQUOTA - O fabricante ou importador dos produtos monofásicos citados no artigo 65 da Lei nº 11.196/2005 estabelecido fora da ZFM, fica obrigado a cobrar e recolher como substituto tributário o PIS e a COFINS devidos pela pessoa jurídica estabelecida na ZFM.
@@ -1665,10 +1677,10 @@
 O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
         </is>
       </c>
-      <c r="BC5" s="1" t="n"/>
-      <c r="BD5" s="1" t="n"/>
-      <c r="BE5" s="1" t="n"/>
-      <c r="BF5" s="1" t="n"/>
+      <c r="BC5" s="1" t="inlineStr"/>
+      <c r="BD5" s="1" t="inlineStr"/>
+      <c r="BE5" s="1" t="inlineStr"/>
+      <c r="BF5" s="1" t="inlineStr"/>
       <c r="BG5" s="1" t="n"/>
       <c r="BH5" s="1" t="n"/>
       <c r="BI5" s="1" t="n"/>
@@ -1721,7 +1733,7 @@
           <t>Bebidas Frias (Monofásico)</t>
         </is>
       </c>
-      <c r="I6" s="1" t="n"/>
+      <c r="I6" s="1" t="inlineStr"/>
       <c r="J6" s="1" t="inlineStr">
         <is>
           <t>CONCEITO DE INCIDÊNCIA MONOFÁSICA - As bebidas frias listadas no artigo 14 da Lei nº 13.097/2015 estão sujeitas a incidência monofásica, conforme prevê o artigo 25 da referida Lei. O sistema de tributação monofásica é um tratamento tributário próprio e específico, previsto em relação ao PIS e a COFINS incidentes sobre a receita bruta decorrente da venda de determinados produtos, onde usualmente a tributação ocorre de forma concentrada no produtor e importador, e no caso das bebidas frias ocorrerá também no atacadista, desonerando as etapas subsequentes de comercialização. A concentração da tributação ocorre com a aplicação de alíquotas maiores que as usualmente aplicadas na tributação das demais receitas.
@@ -1775,10 +1787,14 @@
       </c>
       <c r="U6" s="1" t="inlineStr">
         <is>
-          <t>CRÉDITO ZONA FRANCA DE MANAUS - De acordo com o §§ 12, art. 3º da Lei nº 10.637/2002 e o § 17, art. 3º da Lei nº 10.833/2003, ressalvado o disposto no § 2° do referido artigo e nos §§ 1° a 3° do art. 2°, na aquisição de mercadoria produzida por pessoa jurídica estabelecida na ZFM, consoante projeto aprovado pela Suframa, o crédito será determinado mediante a aplicação da alíquota: PIS a) de alíquota de 1% e, b) de 1,65%, na situação de que trata a alínea ""b"" do inciso II do § 4° do art. 2° da Lei nº 10.637/2002. COFINS a) de 5,60%, nas operações com os bens referidos no inciso VI do art. 28 da Lei n° 11.196/2005; b) de 7,60%, na situação de que trata a alínea ""b"" do inciso II do § 5° do art. 2° desta Lei; e c) de 4,60%, nos demais casos. CRÉDITO ÁREA DE LIVRE COMÉRCIO - Segundo os §§ 15 e 16, art. 3º da Lei nº 10.637/2002 e §§ 23 e 24, art. 3º da Lei nº 10.833/2003, na hipótese de aquisição de mercadoria produzida por pessoa jurídica estabelecida nas Áreas de Livre Comércio, o crédito será determinado mediante a aplicação da alíquota: PIS - de 0,65%. COFINS - de 3%.</t>
-        </is>
-      </c>
-      <c r="V6" s="1" t="n"/>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="V6" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
       <c r="W6" s="1" t="n"/>
       <c r="X6" s="1" t="n"/>
       <c r="Y6" s="1" t="n"/>
@@ -1842,7 +1858,7 @@
       <c r="BD6" s="1" t="n"/>
       <c r="BE6" s="1" t="n"/>
       <c r="BF6" s="1" t="n"/>
-      <c r="BG6" s="1" t="n"/>
+      <c r="BG6" s="1" t="inlineStr"/>
       <c r="BH6" s="1" t="inlineStr">
         <is>
           <t>CONCEITO DE INCIDÊNCIA MONOFÁSICA - As bebidas frias listadas no artigo 14 da Lei nº 13.097/2015 estão sujeitas a incidência monofásica, conforme prevê o artigo 25 da referida Lei. O sistema de tributação monofásica é um tratamento tributário próprio e específico, previsto em relação ao PIS e a COFINS incidentes sobre a receita bruta decorrente da venda de determinados produtos, onde usualmente a tributação ocorre de forma concentrada no produtor e importador, e no caso das bebidas frias ocorrerá também no atacadista, desonerando as etapas subsequentes de comercialização. A concentração da tributação ocorre com a aplicação de alíquotas maiores que as usualmente aplicadas na tributação das demais receitas.
@@ -1864,11 +1880,11 @@
 O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
         </is>
       </c>
-      <c r="BI6" s="1" t="n"/>
-      <c r="BJ6" s="1" t="n"/>
-      <c r="BK6" s="1" t="n"/>
-      <c r="BL6" s="1" t="n"/>
-      <c r="BM6" s="1" t="n"/>
+      <c r="BI6" s="1" t="inlineStr"/>
+      <c r="BJ6" s="1" t="inlineStr"/>
+      <c r="BK6" s="1" t="inlineStr"/>
+      <c r="BL6" s="1" t="inlineStr"/>
+      <c r="BM6" s="1" t="inlineStr"/>
       <c r="BN6" s="1" t="inlineStr">
         <is>
           <t>RECOLHIMENTO - São responsáveis pelo recolhimento do PIS e da COFINS, os importadores, fabricantes e atacadistas dos produtos relacionados no artigo 14 da Lei nº 13.097/2015.
@@ -1876,10 +1892,10 @@
 Cabe destacar que a atividade de produção e venda no atacado de bebidas alcoólicas estava vedada terminantemente ao Simples Nacional até 31/12/2017, passando a ser autorizada nos casos excepcionais de produção ou venda no atacado por micro e pequenos produtores. A atividade de produção e venda no atacado de cervejas sem álcool permanecerá vedada mesmo após 31/12/2017 (Lei Complementar nº 123/2006, artigo 17, inciso X, alíneas "b" e "c").</t>
         </is>
       </c>
-      <c r="BO6" s="1" t="n"/>
-      <c r="BP6" s="1" t="n"/>
-      <c r="BQ6" s="1" t="n"/>
-      <c r="BR6" s="1" t="n"/>
+      <c r="BO6" s="1" t="inlineStr"/>
+      <c r="BP6" s="1" t="inlineStr"/>
+      <c r="BQ6" s="1" t="inlineStr"/>
+      <c r="BR6" s="1" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
@@ -2011,17 +2027,21 @@
       </c>
       <c r="U7" s="1" t="inlineStr">
         <is>
-          <t>CRÉDITO ZONA FRANCA DE MANAUS - De acordo com o §§ 12, art. 3º da Lei nº 10.637/2002 e o § 17, art. 3º da Lei nº 10.833/2003, ressalvado o disposto no § 2° do referido artigo e nos §§ 1° a 3° do art. 2°, na aquisição de mercadoria produzida por pessoa jurídica estabelecida na ZFM, consoante projeto aprovado pela Suframa, o crédito será determinado mediante a aplicação da alíquota: PIS a) de alíquota de 1% e, b) de 1,65%, na situação de que trata a alínea ""b"" do inciso II do § 4° do art. 2° da Lei nº 10.637/2002. COFINS a) de 5,60%, nas operações com os bens referidos no inciso VI do art. 28 da Lei n° 11.196/2005; b) de 7,60%, na situação de que trata a alínea ""b"" do inciso II do § 5° do art. 2° desta Lei; e c) de 4,60%, nos demais casos. CRÉDITO ÁREA DE LIVRE COMÉRCIO - Segundo os §§ 15 e 16, art. 3º da Lei nº 10.637/2002 e §§ 23 e 24, art. 3º da Lei nº 10.833/2003, na hipótese de aquisição de mercadoria produzida por pessoa jurídica estabelecida nas Áreas de Livre Comércio, o crédito será determinado mediante a aplicação da alíquota: PIS - de 0,65%. COFINS - de 3%.</t>
-        </is>
-      </c>
-      <c r="V7" s="1" t="n"/>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="V7" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
       <c r="W7" s="1" t="n"/>
       <c r="X7" s="1" t="n"/>
       <c r="Y7" s="1" t="n"/>
       <c r="Z7" s="1" t="n"/>
       <c r="AA7" s="1" t="n"/>
       <c r="AB7" s="1" t="n"/>
-      <c r="AC7" s="1" t="n"/>
+      <c r="AC7" s="1" t="inlineStr"/>
       <c r="AD7" s="1" t="inlineStr">
         <is>
           <t>CONDIÇÃO - De 01.07.2021 à 14.07.2021 (período que vigou a MP nº 1.034/2021), a pessoa jurídica fabricante de conector 3 vias para infusão com torneira, de plástico, destinada ao uso em hospitais, clínicas, consultórios médicos e campanhas de vacinação, poderia deduzir crédito presumido na apuração do PIS e COFINS devidas em cada período de apuração (MP nº 1.034/2021, artigo 3º, caput e Anexo, item 43).
@@ -2031,10 +2051,10 @@
 b) o valor aduaneiro dos insumos por ela importados, no caso de insumos importados para fabricação dos produtos também relacionados no item “Condição”.</t>
         </is>
       </c>
-      <c r="AE7" s="1" t="n"/>
-      <c r="AF7" s="1" t="n"/>
-      <c r="AG7" s="1" t="n"/>
-      <c r="AH7" s="1" t="n"/>
+      <c r="AE7" s="1" t="inlineStr"/>
+      <c r="AF7" s="1" t="inlineStr"/>
+      <c r="AG7" s="1" t="inlineStr"/>
+      <c r="AH7" s="1" t="inlineStr"/>
       <c r="AI7" s="1" t="n"/>
       <c r="AJ7" s="1" t="n"/>
       <c r="AK7" s="1" t="n"/>
@@ -2209,10 +2229,14 @@
       </c>
       <c r="U8" s="1" t="inlineStr">
         <is>
-          <t>CRÉDITO ZONA FRANCA DE MANAUS - De acordo com o §§ 12, art. 3º da Lei nº 10.637/2002 e o § 17, art. 3º da Lei nº 10.833/2003, ressalvado o disposto no § 2° do referido artigo e nos §§ 1° a 3° do art. 2°, na aquisição de mercadoria produzida por pessoa jurídica estabelecida na ZFM, consoante projeto aprovado pela Suframa, o crédito será determinado mediante a aplicação da alíquota: PIS a) de alíquota de 1% e, b) de 1,65%, na situação de que trata a alínea ""b"" do inciso II do § 4° do art. 2° da Lei nº 10.637/2002. COFINS a) de 5,60%, nas operações com os bens referidos no inciso VI do art. 28 da Lei n° 11.196/2005; b) de 7,60%, na situação de que trata a alínea ""b"" do inciso II do § 5° do art. 2° desta Lei; e c) de 4,60%, nos demais casos. CRÉDITO ÁREA DE LIVRE COMÉRCIO - Segundo os §§ 15 e 16, art. 3º da Lei nº 10.637/2002 e §§ 23 e 24, art. 3º da Lei nº 10.833/2003, na hipótese de aquisição de mercadoria produzida por pessoa jurídica estabelecida nas Áreas de Livre Comércio, o crédito será determinado mediante a aplicação da alíquota: PIS - de 0,65%. COFINS - de 3%.</t>
-        </is>
-      </c>
-      <c r="V8" s="1" t="n"/>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="V8" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
       <c r="W8" s="1" t="n"/>
       <c r="X8" s="1" t="n"/>
       <c r="Y8" s="1" t="n"/>
@@ -2375,10 +2399,14 @@
       </c>
       <c r="U9" s="1" t="inlineStr">
         <is>
-          <t>CRÉDITO ZONA FRANCA DE MANAUS - De acordo com o §§ 12, art. 3º da Lei nº 10.637/2002 e o § 17, art. 3º da Lei nº 10.833/2003, ressalvado o disposto no § 2° do referido artigo e nos §§ 1° a 3° do art. 2°, na aquisição de mercadoria produzida por pessoa jurídica estabelecida na ZFM, consoante projeto aprovado pela Suframa, o crédito será determinado mediante a aplicação da alíquota: PIS a) de alíquota de 1% e, b) de 1,65%, na situação de que trata a alínea ""b"" do inciso II do § 4° do art. 2° da Lei nº 10.637/2002. COFINS a) de 5,60%, nas operações com os bens referidos no inciso VI do art. 28 da Lei n° 11.196/2005; b) de 7,60%, na situação de que trata a alínea ""b"" do inciso II do § 5° do art. 2° desta Lei; e c) de 4,60%, nos demais casos. CRÉDITO ÁREA DE LIVRE COMÉRCIO - Segundo os §§ 15 e 16, art. 3º da Lei nº 10.637/2002 e §§ 23 e 24, art. 3º da Lei nº 10.833/2003, na hipótese de aquisição de mercadoria produzida por pessoa jurídica estabelecida nas Áreas de Livre Comércio, o crédito será determinado mediante a aplicação da alíquota: PIS - de 0,65%. COFINS - de 3%.</t>
-        </is>
-      </c>
-      <c r="V9" s="1" t="n"/>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="V9" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
       <c r="W9" s="1" t="n"/>
       <c r="X9" s="1" t="n"/>
       <c r="Y9" s="1" t="n"/>
@@ -2395,9 +2423,7 @@
           <t>CONDIÇÃO - Será concedido o regime especial de utilização de crédito presumido às pessoas jurídicas que procedam à industrialização ou à importação de medicamentos submetidos às alíquotas concentradas da Contribuição para o PIS e COFINS, sujeitos à prescrição médica e identificados por tarja vermelha ou preta, e que, visando assegurar a repercussão nos preços da redução da carga tributária tenham firmado com a União, compromisso de ajustamento de conduta, nos termos do § 6º do artigo 5º da Lei nº 7.347/85 ou que cumpram a sistemática estabelecida pela Câmara de Regulação do Mercado de Medicamentos (CMED) para utilização do crédito presumido na forma determinada pela Lei nº 10.742/2003 (Lei nº 10.147/2000, artigo 3º, § 2º).
 A concessão do regime especial depende de habilitação perante a CMED e a Receita Federal (RFB).
 ALÍQUOTA - O crédito presumido será determinado mediante a aplicação das alíquotas de 2,10% (PIS) e 9,90% (COFINS) sobre a receita bruta decorrente da venda desse medicamento (Lei nº 10.147/2000, artigo 3º, § 1º).
-A partir de 01/04/2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. No caso dos créditos presumidos, o aproveitamento fica limitado a 90% do valor original, sendo cancelada a parcela não utilizada. Desta forma, os contribuintes devem calcular o crédito presumido utilizando as alíquotas originais constantes na legislação, porém, apropriando valores correspondentes a 90% do crédito original. (Lei Complementar nº 224/2025, artigo 4º, caput e § 4º, inciso IV)
-REGIME CUMULATIVO / NÃO CUMULATIVO - São beneficiários do crédito presumido sobre o segmento farmacêutico as pessoas jurídicas que procedam à industrialização ou à importação dos produtos mencionados no artigo 3º da Lei nº 10.147/2000, optantes pelo regime cumulativo e não cumulativo.
-SIMPLES NACIONAL - Não é concedido crédito presumido as pessoas jurídicas optantes pelo Simples Nacional.</t>
+A partir de 01.04.2026, os incentivos e benefícios federais de natureza tributária são reduzidos, sendo aqueles de crédito presumido mediante aproveitamento limitado a 90% do valor original do crédito, cancelando-se o valor não aproveitado. (Lei Complementar nº 224/2025, artigo 4º, caput e § 4º, inciso IV)</t>
         </is>
       </c>
       <c r="AE9" s="1" t="inlineStr">
@@ -2412,10 +2438,14 @@
       </c>
       <c r="AG9" s="1" t="inlineStr">
         <is>
-          <t>Vide orientações do Registro F700 mencionado no campo NATUREZA DA DEDUÇÃO do item EFD-Contribuições a seguir.</t>
-        </is>
-      </c>
-      <c r="AH9" s="1" t="n"/>
+          <t>2,10%</t>
+        </is>
+      </c>
+      <c r="AH9" s="1" t="inlineStr">
+        <is>
+          <t>9,90%</t>
+        </is>
+      </c>
       <c r="AI9" s="1" t="inlineStr">
         <is>
           <t>Cum: Lei nº 10.147/2000, artigo 1º, inciso I, alínea "a" | N.Cum: Lei nº 10.147/2000, artigo 1º, inciso I, alínea "a"</t>
@@ -2654,10 +2684,14 @@
       </c>
       <c r="U10" s="1" t="inlineStr">
         <is>
-          <t>CRÉDITO ZONA FRANCA DE MANAUS - De acordo com o §§ 12, art. 3º da Lei nº 10.637/2002 e o § 17, art. 3º da Lei nº 10.833/2003, ressalvado o disposto no § 2° do referido artigo e nos §§ 1° a 3° do art. 2°, na aquisição de mercadoria produzida por pessoa jurídica estabelecida na ZFM, consoante projeto aprovado pela Suframa, o crédito será determinado mediante a aplicação da alíquota: PIS a) de alíquota de 1% e, b) de 1,65%, na situação de que trata a alínea ""b"" do inciso II do § 4° do art. 2° da Lei nº 10.637/2002. COFINS a) de 5,60%, nas operações com os bens referidos no inciso VI do art. 28 da Lei n° 11.196/2005; b) de 7,60%, na situação de que trata a alínea ""b"" do inciso II do § 5° do art. 2° desta Lei; e c) de 4,60%, nos demais casos. CRÉDITO ÁREA DE LIVRE COMÉRCIO - Segundo os §§ 15 e 16, art. 3º da Lei nº 10.637/2002 e §§ 23 e 24, art. 3º da Lei nº 10.833/2003, na hipótese de aquisição de mercadoria produzida por pessoa jurídica estabelecida nas Áreas de Livre Comércio, o crédito será determinado mediante a aplicação da alíquota: PIS - de 0,65%. COFINS - de 3%.</t>
-        </is>
-      </c>
-      <c r="V10" s="1" t="n"/>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="V10" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
       <c r="W10" s="1" t="n"/>
       <c r="X10" s="1" t="n"/>
       <c r="Y10" s="1" t="n"/>
@@ -2806,10 +2840,14 @@
       </c>
       <c r="U11" s="1" t="inlineStr">
         <is>
-          <t>CRÉDITO ZONA FRANCA DE MANAUS - De acordo com o §§ 12, art. 3º da Lei nº 10.637/2002 e o § 17, art. 3º da Lei nº 10.833/2003, ressalvado o disposto no § 2° do referido artigo e nos §§ 1° a 3° do art. 2°, na aquisição de mercadoria produzida por pessoa jurídica estabelecida na ZFM, consoante projeto aprovado pela Suframa, o crédito será determinado mediante a aplicação da alíquota: PIS a) de alíquota de 1% e, b) de 1,65%, na situação de que trata a alínea ""b"" do inciso II do § 4° do art. 2° da Lei nº 10.637/2002. COFINS a) de 5,60%, nas operações com os bens referidos no inciso VI do art. 28 da Lei n° 11.196/2005; b) de 7,60%, na situação de que trata a alínea ""b"" do inciso II do § 5° do art. 2° desta Lei; e c) de 4,60%, nos demais casos. CRÉDITO ÁREA DE LIVRE COMÉRCIO - Segundo os §§ 15 e 16, art. 3º da Lei nº 10.637/2002 e §§ 23 e 24, art. 3º da Lei nº 10.833/2003, na hipótese de aquisição de mercadoria produzida por pessoa jurídica estabelecida nas Áreas de Livre Comércio, o crédito será determinado mediante a aplicação da alíquota: PIS - de 0,65%. COFINS - de 3%.</t>
-        </is>
-      </c>
-      <c r="V11" s="1" t="n"/>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="V11" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
       <c r="W11" s="1" t="inlineStr">
         <is>
           <t>Cum: Lei nº 10.925/2004, artigo 1º, inciso V | N.Cum: Lei nº 10.925/2004, artigo 1º, inciso V</t>
@@ -2845,7 +2883,7 @@
       </c>
       <c r="AC11" s="1" t="inlineStr">
         <is>
-          <t>Cum: Lei nº 10.925/2004, artigo 8°, caput, e § 1° e artigo 15, § 2º | N.Cum: Lei nº 10.925/2004, artigo 8°, caput, e § 1° e artigo 15, § 2º</t>
+          <t>Cum: Lei nº 10.925/2004, artigo 8°, caput, e § 1° e artigo 15, § 2º | N.Cum: Lei nº 10.925/2004, artigo 8°, caput, e § 1° e artigo 15, § 2º; Lei Complementar nº 224/2025</t>
         </is>
       </c>
       <c r="AD11" s="1" t="inlineStr">
@@ -2855,7 +2893,7 @@
 - adquiridos de pessoa jurídica domiciliada no País, com suspensão da exigibilidade das contribuições na forma dos artigos 560 e 561 da IN RFB nº 2.121/2022;
 - adquiridos de pessoa física residente no País; ou
 - recebidos de cooperado, pessoa física ou jurídica, residente ou domiciliada no País.
-SIMPLES NACIONAL / REGIME CUMULATIVO - Não é concedido crédito presumido as pessoas jurídicas optantes pelo Simples Nacional e para as que apurem o PIS e COFINS pelo regime cumulativo. O crédito presumido é concedido nas aquisições do produto pesquisado pela indústria do regime não cumulativo, desde que cumpridos os requisitos legais.</t>
+A partir de 01.04.2026, os incentivos e benefícios federais de natureza tributária são reduzidos, sendo aqueles de crédito presumido mediante aproveitamento limitado a 90% do valor original do crédito, cancelando-se o valor não aproveitado. (Lei Complementar nº 224/2025, artigo 4º, caput e § 4º, inciso IV)</t>
         </is>
       </c>
       <c r="AE11" s="1" t="inlineStr">
@@ -2870,12 +2908,12 @@
       </c>
       <c r="AG11" s="1" t="inlineStr">
         <is>
-          <t>0,5775%</t>
+          <t>Vide observações</t>
         </is>
       </c>
       <c r="AH11" s="1" t="inlineStr">
         <is>
-          <t>2,66%</t>
+          <t>Vide observações</t>
         </is>
       </c>
       <c r="AI11" s="1" t="n"/>
@@ -3150,7 +3188,7 @@
           <t>0,00%</t>
         </is>
       </c>
-      <c r="BA12" s="1" t="n"/>
+      <c r="BA12" s="1" t="inlineStr"/>
       <c r="BB12" s="1" t="inlineStr">
         <is>
           <t>VENDA A MONTADORAS DE VEÍCULOS - Não se aplica a substituição tributária na venda de autopeças, pneus novos e câmaras de ar para montadoras de veículos. (Lei nº 11.196/2005, artigo 65, § 6º).
@@ -3176,10 +3214,10 @@
 O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
         </is>
       </c>
-      <c r="BC12" s="1" t="n"/>
-      <c r="BD12" s="1" t="n"/>
-      <c r="BE12" s="1" t="n"/>
-      <c r="BF12" s="1" t="n"/>
+      <c r="BC12" s="1" t="inlineStr"/>
+      <c r="BD12" s="1" t="inlineStr"/>
+      <c r="BE12" s="1" t="inlineStr"/>
+      <c r="BF12" s="1" t="inlineStr"/>
       <c r="BG12" s="1" t="n"/>
       <c r="BH12" s="1" t="n"/>
       <c r="BI12" s="1" t="n"/>
@@ -3293,10 +3331,14 @@
       </c>
       <c r="U13" s="1" t="inlineStr">
         <is>
-          <t>CRÉDITO ZONA FRANCA DE MANAUS - De acordo com o §§ 12, art. 3º da Lei nº 10.637/2002 e o § 17, art. 3º da Lei nº 10.833/2003, ressalvado o disposto no § 2° do referido artigo e nos §§ 1° a 3° do art. 2°, na aquisição de mercadoria produzida por pessoa jurídica estabelecida na ZFM, consoante projeto aprovado pela Suframa, o crédito será determinado mediante a aplicação da alíquota: PIS a) de alíquota de 1% e, b) de 1,65%, na situação de que trata a alínea ""b"" do inciso II do § 4° do art. 2° da Lei nº 10.637/2002. COFINS a) de 5,60%, nas operações com os bens referidos no inciso VI do art. 28 da Lei n° 11.196/2005; b) de 7,60%, na situação de que trata a alínea ""b"" do inciso II do § 5° do art. 2° desta Lei; e c) de 4,60%, nos demais casos. CRÉDITO ÁREA DE LIVRE COMÉRCIO - Segundo os §§ 15 e 16, art. 3º da Lei nº 10.637/2002 e §§ 23 e 24, art. 3º da Lei nº 10.833/2003, na hipótese de aquisição de mercadoria produzida por pessoa jurídica estabelecida nas Áreas de Livre Comércio, o crédito será determinado mediante a aplicação da alíquota: PIS - de 0,65%. COFINS - de 3%.</t>
-        </is>
-      </c>
-      <c r="V13" s="1" t="n"/>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="V13" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
       <c r="W13" s="1" t="inlineStr">
         <is>
           <t>Cum: Lei nº 10.925/2004, artigo 1º, inciso XIX e § 4º | N.Cum: Lei nº 10.925/2004, artigo 1º, inciso XIX e § 4º</t>
@@ -3502,10 +3544,14 @@
       </c>
       <c r="U14" s="1" t="inlineStr">
         <is>
-          <t>CRÉDITO ZONA FRANCA DE MANAUS - De acordo com o §§ 12, art. 3º da Lei nº 10.637/2002 e o § 17, art. 3º da Lei nº 10.833/2003, ressalvado o disposto no § 2° do referido artigo e nos §§ 1° a 3° do art. 2°, na aquisição de mercadoria produzida por pessoa jurídica estabelecida na ZFM, consoante projeto aprovado pela Suframa, o crédito será determinado mediante a aplicação da alíquota: PIS a) de alíquota de 1% e, b) de 1,65%, na situação de que trata a alínea ""b"" do inciso II do § 4° do art. 2° da Lei nº 10.637/2002. COFINS a) de 5,60%, nas operações com os bens referidos no inciso VI do art. 28 da Lei n° 11.196/2005; b) de 7,60%, na situação de que trata a alínea ""b"" do inciso II do § 5° do art. 2° desta Lei; e c) de 4,60%, nos demais casos. CRÉDITO ÁREA DE LIVRE COMÉRCIO - Segundo os §§ 15 e 16, art. 3º da Lei nº 10.637/2002 e §§ 23 e 24, art. 3º da Lei nº 10.833/2003, na hipótese de aquisição de mercadoria produzida por pessoa jurídica estabelecida nas Áreas de Livre Comércio, o crédito será determinado mediante a aplicação da alíquota: PIS - de 0,65%. COFINS - de 3%.</t>
-        </is>
-      </c>
-      <c r="V14" s="1" t="n"/>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="V14" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
       <c r="W14" s="1" t="inlineStr">
         <is>
           <t>Cum: Lei nº 10.925/2004, artigo 1º, inciso XXIII; Lei Complementar n° 224/2025 | N.Cum: Lei nº 10.925/2004, artigo 1º, inciso XXIII; Lei Complementar n° 224/2025</t>
@@ -3716,10 +3762,14 @@
       </c>
       <c r="U15" s="1" t="inlineStr">
         <is>
-          <t>CRÉDITO ZONA FRANCA DE MANAUS - De acordo com o §§ 12, art. 3º da Lei nº 10.637/2002 e o § 17, art. 3º da Lei nº 10.833/2003, ressalvado o disposto no § 2° do referido artigo e nos §§ 1° a 3° do art. 2°, na aquisição de mercadoria produzida por pessoa jurídica estabelecida na ZFM, consoante projeto aprovado pela Suframa, o crédito será determinado mediante a aplicação da alíquota: PIS a) de alíquota de 1% e, b) de 1,65%, na situação de que trata a alínea ""b"" do inciso II do § 4° do art. 2° da Lei nº 10.637/2002. COFINS a) de 5,60%, nas operações com os bens referidos no inciso VI do art. 28 da Lei n° 11.196/2005; b) de 7,60%, na situação de que trata a alínea ""b"" do inciso II do § 5° do art. 2° desta Lei; e c) de 4,60%, nos demais casos. CRÉDITO ÁREA DE LIVRE COMÉRCIO - Segundo os §§ 15 e 16, art. 3º da Lei nº 10.637/2002 e §§ 23 e 24, art. 3º da Lei nº 10.833/2003, na hipótese de aquisição de mercadoria produzida por pessoa jurídica estabelecida nas Áreas de Livre Comércio, o crédito será determinado mediante a aplicação da alíquota: PIS - de 0,65%. COFINS - de 3%.</t>
-        </is>
-      </c>
-      <c r="V15" s="1" t="n"/>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="V15" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
       <c r="W15" s="1" t="n"/>
       <c r="X15" s="1" t="n"/>
       <c r="Y15" s="1" t="n"/>
@@ -3871,10 +3921,14 @@
       </c>
       <c r="U16" s="1" t="inlineStr">
         <is>
-          <t>CRÉDITO ZONA FRANCA DE MANAUS - De acordo com o §§ 12, art. 3º da Lei nº 10.637/2002 e o § 17, art. 3º da Lei nº 10.833/2003, ressalvado o disposto no § 2° do referido artigo e nos §§ 1° a 3° do art. 2°, na aquisição de mercadoria produzida por pessoa jurídica estabelecida na ZFM, consoante projeto aprovado pela Suframa, o crédito será determinado mediante a aplicação da alíquota: PIS a) de alíquota de 1% e, b) de 1,65%, na situação de que trata a alínea ""b"" do inciso II do § 4° do art. 2° da Lei nº 10.637/2002. COFINS a) de 5,60%, nas operações com os bens referidos no inciso VI do art. 28 da Lei n° 11.196/2005; b) de 7,60%, na situação de que trata a alínea ""b"" do inciso II do § 5° do art. 2° desta Lei; e c) de 4,60%, nos demais casos. CRÉDITO ÁREA DE LIVRE COMÉRCIO - Segundo os §§ 15 e 16, art. 3º da Lei nº 10.637/2002 e §§ 23 e 24, art. 3º da Lei nº 10.833/2003, na hipótese de aquisição de mercadoria produzida por pessoa jurídica estabelecida nas Áreas de Livre Comércio, o crédito será determinado mediante a aplicação da alíquota: PIS - de 0,65%. COFINS - de 3%.</t>
-        </is>
-      </c>
-      <c r="V16" s="1" t="n"/>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="V16" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
       <c r="W16" s="1" t="inlineStr">
         <is>
           <t>Cum: Lei nº 9.715/98, artigo 8º, inciso I; Lei nº 9.718/98, artigo 8º; Lei n° 10.865/2004, artigo 28, inciso XVII | N.Cum: Decreto nº 6.426/2008, artigo 1º, inciso III; Lei n° 10.865/2004, artigo 28, inciso XVII; Lei Complementar nº 224/2025</t>
@@ -4096,10 +4150,14 @@
       </c>
       <c r="U17" s="1" t="inlineStr">
         <is>
-          <t>CRÉDITO ZONA FRANCA DE MANAUS - De acordo com o §§ 12, art. 3º da Lei nº 10.637/2002 e o § 17, art. 3º da Lei nº 10.833/2003, ressalvado o disposto no § 2° do referido artigo e nos §§ 1° a 3° do art. 2°, na aquisição de mercadoria produzida por pessoa jurídica estabelecida na ZFM, consoante projeto aprovado pela Suframa, o crédito será determinado mediante a aplicação da alíquota: PIS a) de alíquota de 1% e, b) de 1,65%, na situação de que trata a alínea ""b"" do inciso II do § 4° do art. 2° da Lei nº 10.637/2002. COFINS a) de 5,60%, nas operações com os bens referidos no inciso VI do art. 28 da Lei n° 11.196/2005; b) de 7,60%, na situação de que trata a alínea ""b"" do inciso II do § 5° do art. 2° desta Lei; e c) de 4,60%, nos demais casos. CRÉDITO ÁREA DE LIVRE COMÉRCIO - Segundo os §§ 15 e 16, art. 3º da Lei nº 10.637/2002 e §§ 23 e 24, art. 3º da Lei nº 10.833/2003, na hipótese de aquisição de mercadoria produzida por pessoa jurídica estabelecida nas Áreas de Livre Comércio, o crédito será determinado mediante a aplicação da alíquota: PIS - de 0,65%. COFINS - de 3%.</t>
-        </is>
-      </c>
-      <c r="V17" s="1" t="n"/>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="V17" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
       <c r="W17" s="1" t="n"/>
       <c r="X17" s="1" t="n"/>
       <c r="Y17" s="1" t="n"/>
@@ -4288,10 +4346,14 @@
       </c>
       <c r="U18" s="1" t="inlineStr">
         <is>
-          <t>CRÉDITO ZONA FRANCA DE MANAUS - De acordo com o §§ 12, art. 3º da Lei nº 10.637/2002 e o § 17, art. 3º da Lei nº 10.833/2003, ressalvado o disposto no § 2° do referido artigo e nos §§ 1° a 3° do art. 2°, na aquisição de mercadoria produzida por pessoa jurídica estabelecida na ZFM, consoante projeto aprovado pela Suframa, o crédito será determinado mediante a aplicação da alíquota: PIS a) de alíquota de 1% e, b) de 1,65%, na situação de que trata a alínea ""b"" do inciso II do § 4° do art. 2° da Lei nº 10.637/2002. COFINS a) de 5,60%, nas operações com os bens referidos no inciso VI do art. 28 da Lei n° 11.196/2005; b) de 7,60%, na situação de que trata a alínea ""b"" do inciso II do § 5° do art. 2° desta Lei; e c) de 4,60%, nos demais casos. CRÉDITO ÁREA DE LIVRE COMÉRCIO - Segundo os §§ 15 e 16, art. 3º da Lei nº 10.637/2002 e §§ 23 e 24, art. 3º da Lei nº 10.833/2003, na hipótese de aquisição de mercadoria produzida por pessoa jurídica estabelecida nas Áreas de Livre Comércio, o crédito será determinado mediante a aplicação da alíquota: PIS - de 0,65%. COFINS - de 3%.</t>
-        </is>
-      </c>
-      <c r="V18" s="1" t="n"/>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="V18" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
       <c r="W18" s="1" t="n"/>
       <c r="X18" s="1" t="n"/>
       <c r="Y18" s="1" t="n"/>
@@ -4450,10 +4512,14 @@
       </c>
       <c r="U19" s="1" t="inlineStr">
         <is>
-          <t>CRÉDITO ZONA FRANCA DE MANAUS - De acordo com o §§ 12, art. 3º da Lei nº 10.637/2002 e o § 17, art. 3º da Lei nº 10.833/2003, ressalvado o disposto no § 2° do referido artigo e nos §§ 1° a 3° do art. 2°, na aquisição de mercadoria produzida por pessoa jurídica estabelecida na ZFM, consoante projeto aprovado pela Suframa, o crédito será determinado mediante a aplicação da alíquota: PIS a) de alíquota de 1% e, b) de 1,65%, na situação de que trata a alínea ""b"" do inciso II do § 4° do art. 2° da Lei nº 10.637/2002. COFINS a) de 5,60%, nas operações com os bens referidos no inciso VI do art. 28 da Lei n° 11.196/2005; b) de 7,60%, na situação de que trata a alínea ""b"" do inciso II do § 5° do art. 2° desta Lei; e c) de 4,60%, nos demais casos. CRÉDITO ÁREA DE LIVRE COMÉRCIO - Segundo os §§ 15 e 16, art. 3º da Lei nº 10.637/2002 e §§ 23 e 24, art. 3º da Lei nº 10.833/2003, na hipótese de aquisição de mercadoria produzida por pessoa jurídica estabelecida nas Áreas de Livre Comércio, o crédito será determinado mediante a aplicação da alíquota: PIS - de 0,65%. COFINS - de 3%.</t>
-        </is>
-      </c>
-      <c r="V19" s="1" t="n"/>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="V19" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
       <c r="W19" s="1" t="inlineStr">
         <is>
           <t>Cum: Lei nº 10.925/2004, artigo 1º, inciso XI | N.Cum: Lei nº 10.925/2004, artigo 1º, inciso XI</t>
@@ -4499,7 +4565,7 @@
       </c>
       <c r="AC19" s="1" t="inlineStr">
         <is>
-          <t>Cum: Lei nº 10.925/2004, artigo 8º; Lei nº 12.865/2013, artigo 30 | N.Cum: Lei nº 10.925/2004, artigo 8º; Lei nº 12.865/2013, artigo 30</t>
+          <t>Cum: Lei nº 10.925/2004, artigo 8º; Lei nº 12.865/2013, artigo 30 | N.Cum: Lei nº 10.925/2004, artigo 8º; Lei nº 12.865/2013, artigo 30; Lei Complementar nº 224/2025</t>
         </is>
       </c>
       <c r="AD19" s="1" t="inlineStr">
@@ -4509,7 +4575,7 @@
 - adquiridos de pessoa jurídica domiciliada no País, com suspensão da exigibilidade das contribuições na forma dos artigos 560 e 561 da IN RFB nº 2.121/2022;
 - adquiridos de pessoa física residente no País; ou
 - recebidos de cooperado, pessoa física ou jurídica, residente ou domiciliada no País (Lei nº 10.925/2004, artigo 8º; Lei nº 12.865/2013, artigo 30).
-SIMPLES NACIONAL / REGIME CUMULATIVO - Não é concedido crédito presumido as pessoas jurídicas optantes pelo Simples Nacional e para as que apurem o PIS e COFINS pelo regime cumulativo. O crédito presumido é concedido nas aquisições do produto pesquisado pela indústria do regime não cumulativo, desde que cumpridos os requisitos legais.</t>
+A partir de 01.04.2026, os incentivos e benefícios federais de natureza tributária são reduzidos, sendo aqueles de crédito presumido mediante aproveitamento limitado a 90% do valor original do crédito, cancelando-se o valor não aproveitado. (Lei Complementar nº 224/2025, artigo 4º, caput e § 4º, inciso IV)</t>
         </is>
       </c>
       <c r="AE19" s="1" t="inlineStr">
@@ -4524,12 +4590,12 @@
       </c>
       <c r="AG19" s="1" t="inlineStr">
         <is>
-          <t>0,99%</t>
+          <t>Vide observações</t>
         </is>
       </c>
       <c r="AH19" s="1" t="inlineStr">
         <is>
-          <t>4,56%</t>
+          <t>Vide observações</t>
         </is>
       </c>
       <c r="AI19" s="1" t="n"/>
@@ -4583,7 +4649,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F465"/>
+  <dimension ref="A1:F508"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -18140,6 +18206,1342 @@
         </is>
       </c>
     </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>2026-04-20 14:48</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>1006.30.21</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>Crédito Presumido - PIS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>0,5775%</t>
+        </is>
+      </c>
+      <c r="F466" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>2026-04-20 14:48</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>1006.30.21</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>Crédito Presumido - COFINS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>2,66%</t>
+        </is>
+      </c>
+      <c r="F467" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>2026-04-20 14:48</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>1006.30.21</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>Crédito Presumido - Legislação</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>Cum: Lei nº 10.925/2004, artigo 8°, caput, e § 1° e artigo 15, § 2º | N.Cum: Lei nº 10.925/2004, artigo 8°, caput, e § 1° e artigo 15, § 2º</t>
+        </is>
+      </c>
+      <c r="F468" t="inlineStr">
+        <is>
+          <t>Cum: Lei nº 10.925/2004, artigo 8°, caput, e § 1° e artigo 15, § 2º | N.Cum: Lei nº 10.925/2004, artigo 8°, caput, e § 1° e artigo 15, § 2º; Lei Complementar nº 224/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>2026-04-20 14:48</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>1006.30.21</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>Crédito Presumido - Observações</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>ALÍQUOTA - O crédito presumido será determinado mediante a aplicação das alíquotas de 0,5775% (PIS) e 2,66% (COFINS) sobre o valor de aquisição dos produtos agropecuários utilizados como insumo na fabricação do produto pesquisado quando este é destinado à alimentação humana ou animal.
+O crédito presumido será apurado no caso dos produtos agropecuários: (Lei n° 10.925/2004, artigo 8°, caput e § 1°)
+- adquiridos de pessoa jurídica domiciliada no País, com suspensão da exigibilidade das contribuições na forma dos artigos 560 e 561 da IN RFB nº 2.121/2022;
+- adquiridos de pessoa física residente no País; ou
+- recebidos de cooperado, pessoa física ou jurídica, residente ou domiciliada no País.
+SIMPLES NACIONAL / REGIME CUMULATIVO - Não é concedido crédito presumido as pessoas jurídicas optantes pelo Simples Nacional e para as que apurem o PIS e COFINS pelo regime cumulativo. O crédito presumido é concedido nas aquisições do produto pesquisado pela indústria do regime não cumulativo, desde que cumpridos os requisitos legais.</t>
+        </is>
+      </c>
+      <c r="F469" t="inlineStr">
+        <is>
+          <t>ALÍQUOTA - O crédito presumido será determinado mediante a aplicação das alíquotas de 0,5775% (PIS) e 2,66% (COFINS) sobre o valor de aquisição dos produtos agropecuários utilizados como insumo na fabricação do produto pesquisado quando este é destinado à alimentação humana ou animal.
+O crédito presumido será apurado no caso dos produtos agropecuários: (Lei n° 10.925/2004, artigo 8°, caput e § 1°)
+- adquiridos de pessoa jurídica domiciliada no País, com suspensão da exigibilidade das contribuições na forma dos artigos 560 e 561 da IN RFB nº 2.121/2022;
+- adquiridos de pessoa física residente no País; ou
+- recebidos de cooperado, pessoa física ou jurídica, residente ou domiciliada no País.
+A partir de 01.04.2026, os incentivos e benefícios federais de natureza tributária são reduzidos, sendo aqueles de crédito presumido mediante aproveitamento limitado a 90% do valor original do crédito, cancelando-se o valor não aproveitado. (Lei Complementar nº 224/2025, artigo 4º, caput e § 4º, inciso IV)</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>2026-04-20 14:48</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>0402.21.10</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>Crédito Presumido - PIS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>0,99%</t>
+        </is>
+      </c>
+      <c r="F470" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>2026-04-20 14:48</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>0402.21.10</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>Crédito Presumido - COFINS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>4,56%</t>
+        </is>
+      </c>
+      <c r="F471" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>2026-04-20 14:48</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>0402.21.10</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>Crédito Presumido - Legislação</t>
+        </is>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>Cum: Lei nº 10.925/2004, artigo 8º; Lei nº 12.865/2013, artigo 30 | N.Cum: Lei nº 10.925/2004, artigo 8º; Lei nº 12.865/2013, artigo 30</t>
+        </is>
+      </c>
+      <c r="F472" t="inlineStr">
+        <is>
+          <t>Cum: Lei nº 10.925/2004, artigo 8º; Lei nº 12.865/2013, artigo 30 | N.Cum: Lei nº 10.925/2004, artigo 8º; Lei nº 12.865/2013, artigo 30; Lei Complementar nº 224/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>2026-04-20 14:48</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>0402.21.10</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>Crédito Presumido - Observações</t>
+        </is>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>ALÍQUOTA - O crédito presumido será determinado mediante a aplicação das alíquotas de 0,99% (PIS) e 4,56% (COFINS) sobre o valor de aquisição dos produtos agropecuários utilizados como insumo na fabricação do produto pesquisado quando este é destinado à alimentação humana ou animal.
+O crédito presumido será apurado no caso dos produtos agropecuários:
+- adquiridos de pessoa jurídica domiciliada no País, com suspensão da exigibilidade das contribuições na forma dos artigos 560 e 561 da IN RFB nº 2.121/2022;
+- adquiridos de pessoa física residente no País; ou
+- recebidos de cooperado, pessoa física ou jurídica, residente ou domiciliada no País (Lei nº 10.925/2004, artigo 8º; Lei nº 12.865/2013, artigo 30).
+SIMPLES NACIONAL / REGIME CUMULATIVO - Não é concedido crédito presumido as pessoas jurídicas optantes pelo Simples Nacional e para as que apurem o PIS e COFINS pelo regime cumulativo. O crédito presumido é concedido nas aquisições do produto pesquisado pela indústria do regime não cumulativo, desde que cumpridos os requisitos legais.</t>
+        </is>
+      </c>
+      <c r="F473" t="inlineStr">
+        <is>
+          <t>ALÍQUOTA - O crédito presumido será determinado mediante a aplicação das alíquotas de 0,99% (PIS) e 4,56% (COFINS) sobre o valor de aquisição dos produtos agropecuários utilizados como insumo na fabricação do produto pesquisado quando este é destinado à alimentação humana ou animal.
+O crédito presumido será apurado no caso dos produtos agropecuários:
+- adquiridos de pessoa jurídica domiciliada no País, com suspensão da exigibilidade das contribuições na forma dos artigos 560 e 561 da IN RFB nº 2.121/2022;
+- adquiridos de pessoa física residente no País; ou
+- recebidos de cooperado, pessoa física ou jurídica, residente ou domiciliada no País (Lei nº 10.925/2004, artigo 8º; Lei nº 12.865/2013, artigo 30).
+A partir de 01.04.2026, os incentivos e benefícios federais de natureza tributária são reduzidos, sendo aqueles de crédito presumido mediante aproveitamento limitado a 90% do valor original do crédito, cancelando-se o valor não aproveitado. (Lei Complementar nº 224/2025, artigo 4º, caput e § 4º, inciso IV)</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>8471.41.90</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>ZFM - PIS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>CRÉDITO ZONA FRANCA DE MANAUS - De acordo com o §§ 12, art. 3º da Lei nº 10.637/2002 e o § 17, art. 3º da Lei nº 10.833/2003, ressalvado o disposto no § 2° do referido artigo e nos §§ 1° a 3° do art. 2°, na aquisição de mercadoria produzida por pessoa jurídica estabelecida na ZFM, consoante projeto aprovado pela Suframa, o crédito será determinado mediante a aplicação da alíquota: PIS a) de alíquota de 1% e, b) de 1,65%, na situação de que trata a alínea ""b"" do inciso II do § 4° do art. 2° da Lei nº 10.637/2002. COFINS a) de 5,60%, nas operações com os bens referidos no inciso VI do art. 28 da Lei n° 11.196/2005; b) de 7,60%, na situação de que trata a alínea ""b"" do inciso II do § 5° do art. 2° desta Lei; e c) de 4,60%, nos demais casos. CRÉDITO ÁREA DE LIVRE COMÉRCIO - Segundo os §§ 15 e 16, art. 3º da Lei nº 10.637/2002 e §§ 23 e 24, art. 3º da Lei nº 10.833/2003, na hipótese de aquisição de mercadoria produzida por pessoa jurídica estabelecida nas Áreas de Livre Comércio, o crédito será determinado mediante a aplicação da alíquota: PIS - de 0,65%. COFINS - de 3%.</t>
+        </is>
+      </c>
+      <c r="F474" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>8471.41.90</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E475" t="inlineStr"/>
+      <c r="F475" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>3926.90.90</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>ZFM - PIS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>CRÉDITO ZONA FRANCA DE MANAUS - De acordo com o §§ 12, art. 3º da Lei nº 10.637/2002 e o § 17, art. 3º da Lei nº 10.833/2003, ressalvado o disposto no § 2° do referido artigo e nos §§ 1° a 3° do art. 2°, na aquisição de mercadoria produzida por pessoa jurídica estabelecida na ZFM, consoante projeto aprovado pela Suframa, o crédito será determinado mediante a aplicação da alíquota: PIS a) de alíquota de 1% e, b) de 1,65%, na situação de que trata a alínea ""b"" do inciso II do § 4° do art. 2° da Lei nº 10.637/2002. COFINS a) de 5,60%, nas operações com os bens referidos no inciso VI do art. 28 da Lei n° 11.196/2005; b) de 7,60%, na situação de que trata a alínea ""b"" do inciso II do § 5° do art. 2° desta Lei; e c) de 4,60%, nos demais casos. CRÉDITO ÁREA DE LIVRE COMÉRCIO - Segundo os §§ 15 e 16, art. 3º da Lei nº 10.637/2002 e §§ 23 e 24, art. 3º da Lei nº 10.833/2003, na hipótese de aquisição de mercadoria produzida por pessoa jurídica estabelecida nas Áreas de Livre Comércio, o crédito será determinado mediante a aplicação da alíquota: PIS - de 0,65%. COFINS - de 3%.</t>
+        </is>
+      </c>
+      <c r="F476" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>3926.90.90</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E477" t="inlineStr"/>
+      <c r="F477" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>6109.10.00</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>ZFM - PIS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E478" t="inlineStr">
+        <is>
+          <t>CRÉDITO ZONA FRANCA DE MANAUS - De acordo com o §§ 12, art. 3º da Lei nº 10.637/2002 e o § 17, art. 3º da Lei nº 10.833/2003, ressalvado o disposto no § 2° do referido artigo e nos §§ 1° a 3° do art. 2°, na aquisição de mercadoria produzida por pessoa jurídica estabelecida na ZFM, consoante projeto aprovado pela Suframa, o crédito será determinado mediante a aplicação da alíquota: PIS a) de alíquota de 1% e, b) de 1,65%, na situação de que trata a alínea ""b"" do inciso II do § 4° do art. 2° da Lei nº 10.637/2002. COFINS a) de 5,60%, nas operações com os bens referidos no inciso VI do art. 28 da Lei n° 11.196/2005; b) de 7,60%, na situação de que trata a alínea ""b"" do inciso II do § 5° do art. 2° desta Lei; e c) de 4,60%, nos demais casos. CRÉDITO ÁREA DE LIVRE COMÉRCIO - Segundo os §§ 15 e 16, art. 3º da Lei nº 10.637/2002 e §§ 23 e 24, art. 3º da Lei nº 10.833/2003, na hipótese de aquisição de mercadoria produzida por pessoa jurídica estabelecida nas Áreas de Livre Comércio, o crédito será determinado mediante a aplicação da alíquota: PIS - de 0,65%. COFINS - de 3%.</t>
+        </is>
+      </c>
+      <c r="F478" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>6109.10.00</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E479" t="inlineStr"/>
+      <c r="F479" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>2202.10.00</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>ZFM - PIS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t>CRÉDITO ZONA FRANCA DE MANAUS - De acordo com o §§ 12, art. 3º da Lei nº 10.637/2002 e o § 17, art. 3º da Lei nº 10.833/2003, ressalvado o disposto no § 2° do referido artigo e nos §§ 1° a 3° do art. 2°, na aquisição de mercadoria produzida por pessoa jurídica estabelecida na ZFM, consoante projeto aprovado pela Suframa, o crédito será determinado mediante a aplicação da alíquota: PIS a) de alíquota de 1% e, b) de 1,65%, na situação de que trata a alínea ""b"" do inciso II do § 4° do art. 2° da Lei nº 10.637/2002. COFINS a) de 5,60%, nas operações com os bens referidos no inciso VI do art. 28 da Lei n° 11.196/2005; b) de 7,60%, na situação de que trata a alínea ""b"" do inciso II do § 5° do art. 2° desta Lei; e c) de 4,60%, nos demais casos. CRÉDITO ÁREA DE LIVRE COMÉRCIO - Segundo os §§ 15 e 16, art. 3º da Lei nº 10.637/2002 e §§ 23 e 24, art. 3º da Lei nº 10.833/2003, na hipótese de aquisição de mercadoria produzida por pessoa jurídica estabelecida nas Áreas de Livre Comércio, o crédito será determinado mediante a aplicação da alíquota: PIS - de 0,65%. COFINS - de 3%.</t>
+        </is>
+      </c>
+      <c r="F480" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>2202.10.00</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E481" t="inlineStr"/>
+      <c r="F481" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>8481.80.99</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>ZFM - PIS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>CRÉDITO ZONA FRANCA DE MANAUS - De acordo com o §§ 12, art. 3º da Lei nº 10.637/2002 e o § 17, art. 3º da Lei nº 10.833/2003, ressalvado o disposto no § 2° do referido artigo e nos §§ 1° a 3° do art. 2°, na aquisição de mercadoria produzida por pessoa jurídica estabelecida na ZFM, consoante projeto aprovado pela Suframa, o crédito será determinado mediante a aplicação da alíquota: PIS a) de alíquota de 1% e, b) de 1,65%, na situação de que trata a alínea ""b"" do inciso II do § 4° do art. 2° da Lei nº 10.637/2002. COFINS a) de 5,60%, nas operações com os bens referidos no inciso VI do art. 28 da Lei n° 11.196/2005; b) de 7,60%, na situação de que trata a alínea ""b"" do inciso II do § 5° do art. 2° desta Lei; e c) de 4,60%, nos demais casos. CRÉDITO ÁREA DE LIVRE COMÉRCIO - Segundo os §§ 15 e 16, art. 3º da Lei nº 10.637/2002 e §§ 23 e 24, art. 3º da Lei nº 10.833/2003, na hipótese de aquisição de mercadoria produzida por pessoa jurídica estabelecida nas Áreas de Livre Comércio, o crédito será determinado mediante a aplicação da alíquota: PIS - de 0,65%. COFINS - de 3%.</t>
+        </is>
+      </c>
+      <c r="F482" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>8481.80.99</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E483" t="inlineStr"/>
+      <c r="F483" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>9403.60.90</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>ZFM - PIS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>CRÉDITO ZONA FRANCA DE MANAUS - De acordo com o §§ 12, art. 3º da Lei nº 10.637/2002 e o § 17, art. 3º da Lei nº 10.833/2003, ressalvado o disposto no § 2° do referido artigo e nos §§ 1° a 3° do art. 2°, na aquisição de mercadoria produzida por pessoa jurídica estabelecida na ZFM, consoante projeto aprovado pela Suframa, o crédito será determinado mediante a aplicação da alíquota: PIS a) de alíquota de 1% e, b) de 1,65%, na situação de que trata a alínea ""b"" do inciso II do § 4° do art. 2° da Lei nº 10.637/2002. COFINS a) de 5,60%, nas operações com os bens referidos no inciso VI do art. 28 da Lei n° 11.196/2005; b) de 7,60%, na situação de que trata a alínea ""b"" do inciso II do § 5° do art. 2° desta Lei; e c) de 4,60%, nos demais casos. CRÉDITO ÁREA DE LIVRE COMÉRCIO - Segundo os §§ 15 e 16, art. 3º da Lei nº 10.637/2002 e §§ 23 e 24, art. 3º da Lei nº 10.833/2003, na hipótese de aquisição de mercadoria produzida por pessoa jurídica estabelecida nas Áreas de Livre Comércio, o crédito será determinado mediante a aplicação da alíquota: PIS - de 0,65%. COFINS - de 3%.</t>
+        </is>
+      </c>
+      <c r="F484" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>9403.60.90</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E485" t="inlineStr"/>
+      <c r="F485" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>3004.90.99</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>ZFM - PIS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>CRÉDITO ZONA FRANCA DE MANAUS - De acordo com o §§ 12, art. 3º da Lei nº 10.637/2002 e o § 17, art. 3º da Lei nº 10.833/2003, ressalvado o disposto no § 2° do referido artigo e nos §§ 1° a 3° do art. 2°, na aquisição de mercadoria produzida por pessoa jurídica estabelecida na ZFM, consoante projeto aprovado pela Suframa, o crédito será determinado mediante a aplicação da alíquota: PIS a) de alíquota de 1% e, b) de 1,65%, na situação de que trata a alínea ""b"" do inciso II do § 4° do art. 2° da Lei nº 10.637/2002. COFINS a) de 5,60%, nas operações com os bens referidos no inciso VI do art. 28 da Lei n° 11.196/2005; b) de 7,60%, na situação de que trata a alínea ""b"" do inciso II do § 5° do art. 2° desta Lei; e c) de 4,60%, nos demais casos. CRÉDITO ÁREA DE LIVRE COMÉRCIO - Segundo os §§ 15 e 16, art. 3º da Lei nº 10.637/2002 e §§ 23 e 24, art. 3º da Lei nº 10.833/2003, na hipótese de aquisição de mercadoria produzida por pessoa jurídica estabelecida nas Áreas de Livre Comércio, o crédito será determinado mediante a aplicação da alíquota: PIS - de 0,65%. COFINS - de 3%.</t>
+        </is>
+      </c>
+      <c r="F486" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>3004.90.99</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E487" t="inlineStr"/>
+      <c r="F487" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>3004.90.99</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>Crédito Presumido - PIS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E488" t="inlineStr">
+        <is>
+          <t>Vide orientações do Registro F700 mencionado no campo NATUREZA DA DEDUÇÃO do item EFD-Contribuições a seguir.</t>
+        </is>
+      </c>
+      <c r="F488" t="inlineStr">
+        <is>
+          <t>2,10%</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>3004.90.99</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>Crédito Presumido - COFINS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E489" t="inlineStr"/>
+      <c r="F489" t="inlineStr">
+        <is>
+          <t>9,90%</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>3004.90.99</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>Crédito Presumido - Observações</t>
+        </is>
+      </c>
+      <c r="E490" t="inlineStr">
+        <is>
+          <t>CONDIÇÃO - Será concedido o regime especial de utilização de crédito presumido às pessoas jurídicas que procedam à industrialização ou à importação de medicamentos submetidos às alíquotas concentradas da Contribuição para o PIS e COFINS, sujeitos à prescrição médica e identificados por tarja vermelha ou preta, e que, visando assegurar a repercussão nos preços da redução da carga tributária tenham firmado com a União, compromisso de ajustamento de conduta, nos termos do § 6º do artigo 5º da Lei nº 7.347/85 ou que cumpram a sistemática estabelecida pela Câmara de Regulação do Mercado de Medicamentos (CMED) para utilização do crédito presumido na forma determinada pela Lei nº 10.742/2003 (Lei nº 10.147/2000, artigo 3º, § 2º).
+A concessão do regime especial depende de habilitação perante a CMED e a Receita Federal (RFB).
+ALÍQUOTA - O crédito presumido será determinado mediante a aplicação das alíquotas de 2,10% (PIS) e 9,90% (COFINS) sobre a receita bruta decorrente da venda desse medicamento (Lei nº 10.147/2000, artigo 3º, § 1º).
+A partir de 01/04/2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. No caso dos créditos presumidos, o aproveitamento fica limitado a 90% do valor original, sendo cancelada a parcela não utilizada. Desta forma, os contribuintes devem calcular o crédito presumido utilizando as alíquotas originais constantes na legislação, porém, apropriando valores correspondentes a 90% do crédito original. (Lei Complementar nº 224/2025, artigo 4º, caput e § 4º, inciso IV)
+REGIME CUMULATIVO / NÃO CUMULATIVO - São beneficiários do crédito presumido sobre o segmento farmacêutico as pessoas jurídicas que procedam à industrialização ou à importação dos produtos mencionados no artigo 3º da Lei nº 10.147/2000, optantes pelo regime cumulativo e não cumulativo.
+SIMPLES NACIONAL - Não é concedido crédito presumido as pessoas jurídicas optantes pelo Simples Nacional.</t>
+        </is>
+      </c>
+      <c r="F490" t="inlineStr">
+        <is>
+          <t>CONDIÇÃO - Será concedido o regime especial de utilização de crédito presumido às pessoas jurídicas que procedam à industrialização ou à importação de medicamentos submetidos às alíquotas concentradas da Contribuição para o PIS e COFINS, sujeitos à prescrição médica e identificados por tarja vermelha ou preta, e que, visando assegurar a repercussão nos preços da redução da carga tributária tenham firmado com a União, compromisso de ajustamento de conduta, nos termos do § 6º do artigo 5º da Lei nº 7.347/85 ou que cumpram a sistemática estabelecida pela Câmara de Regulação do Mercado de Medicamentos (CMED) para utilização do crédito presumido na forma determinada pela Lei nº 10.742/2003 (Lei nº 10.147/2000, artigo 3º, § 2º).
+A concessão do regime especial depende de habilitação perante a CMED e a Receita Federal (RFB).
+ALÍQUOTA - O crédito presumido será determinado mediante a aplicação das alíquotas de 2,10% (PIS) e 9,90% (COFINS) sobre a receita bruta decorrente da venda desse medicamento (Lei nº 10.147/2000, artigo 3º, § 1º).
+A partir de 01.04.2026, os incentivos e benefícios federais de natureza tributária são reduzidos, sendo aqueles de crédito presumido mediante aproveitamento limitado a 90% do valor original do crédito, cancelando-se o valor não aproveitado. (Lei Complementar nº 224/2025, artigo 4º, caput e § 4º, inciso IV)</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>8443.31.00</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>ZFM - PIS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E491" t="inlineStr">
+        <is>
+          <t>CRÉDITO ZONA FRANCA DE MANAUS - De acordo com o §§ 12, art. 3º da Lei nº 10.637/2002 e o § 17, art. 3º da Lei nº 10.833/2003, ressalvado o disposto no § 2° do referido artigo e nos §§ 1° a 3° do art. 2°, na aquisição de mercadoria produzida por pessoa jurídica estabelecida na ZFM, consoante projeto aprovado pela Suframa, o crédito será determinado mediante a aplicação da alíquota: PIS a) de alíquota de 1% e, b) de 1,65%, na situação de que trata a alínea ""b"" do inciso II do § 4° do art. 2° da Lei nº 10.637/2002. COFINS a) de 5,60%, nas operações com os bens referidos no inciso VI do art. 28 da Lei n° 11.196/2005; b) de 7,60%, na situação de que trata a alínea ""b"" do inciso II do § 5° do art. 2° desta Lei; e c) de 4,60%, nos demais casos. CRÉDITO ÁREA DE LIVRE COMÉRCIO - Segundo os §§ 15 e 16, art. 3º da Lei nº 10.637/2002 e §§ 23 e 24, art. 3º da Lei nº 10.833/2003, na hipótese de aquisição de mercadoria produzida por pessoa jurídica estabelecida nas Áreas de Livre Comércio, o crédito será determinado mediante a aplicação da alíquota: PIS - de 0,65%. COFINS - de 3%.</t>
+        </is>
+      </c>
+      <c r="F491" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>8443.31.00</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E492" t="inlineStr"/>
+      <c r="F492" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>1006.30.21</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>ZFM - PIS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E493" t="inlineStr">
+        <is>
+          <t>CRÉDITO ZONA FRANCA DE MANAUS - De acordo com o §§ 12, art. 3º da Lei nº 10.637/2002 e o § 17, art. 3º da Lei nº 10.833/2003, ressalvado o disposto no § 2° do referido artigo e nos §§ 1° a 3° do art. 2°, na aquisição de mercadoria produzida por pessoa jurídica estabelecida na ZFM, consoante projeto aprovado pela Suframa, o crédito será determinado mediante a aplicação da alíquota: PIS a) de alíquota de 1% e, b) de 1,65%, na situação de que trata a alínea ""b"" do inciso II do § 4° do art. 2° da Lei nº 10.637/2002. COFINS a) de 5,60%, nas operações com os bens referidos no inciso VI do art. 28 da Lei n° 11.196/2005; b) de 7,60%, na situação de que trata a alínea ""b"" do inciso II do § 5° do art. 2° desta Lei; e c) de 4,60%, nos demais casos. CRÉDITO ÁREA DE LIVRE COMÉRCIO - Segundo os §§ 15 e 16, art. 3º da Lei nº 10.637/2002 e §§ 23 e 24, art. 3º da Lei nº 10.833/2003, na hipótese de aquisição de mercadoria produzida por pessoa jurídica estabelecida nas Áreas de Livre Comércio, o crédito será determinado mediante a aplicação da alíquota: PIS - de 0,65%. COFINS - de 3%.</t>
+        </is>
+      </c>
+      <c r="F493" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>1006.30.21</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E494" t="inlineStr"/>
+      <c r="F494" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>0207.14.00</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>ZFM - PIS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E495" t="inlineStr">
+        <is>
+          <t>CRÉDITO ZONA FRANCA DE MANAUS - De acordo com o §§ 12, art. 3º da Lei nº 10.637/2002 e o § 17, art. 3º da Lei nº 10.833/2003, ressalvado o disposto no § 2° do referido artigo e nos §§ 1° a 3° do art. 2°, na aquisição de mercadoria produzida por pessoa jurídica estabelecida na ZFM, consoante projeto aprovado pela Suframa, o crédito será determinado mediante a aplicação da alíquota: PIS a) de alíquota de 1% e, b) de 1,65%, na situação de que trata a alínea ""b"" do inciso II do § 4° do art. 2° da Lei nº 10.637/2002. COFINS a) de 5,60%, nas operações com os bens referidos no inciso VI do art. 28 da Lei n° 11.196/2005; b) de 7,60%, na situação de que trata a alínea ""b"" do inciso II do § 5° do art. 2° desta Lei; e c) de 4,60%, nos demais casos. CRÉDITO ÁREA DE LIVRE COMÉRCIO - Segundo os §§ 15 e 16, art. 3º da Lei nº 10.637/2002 e §§ 23 e 24, art. 3º da Lei nº 10.833/2003, na hipótese de aquisição de mercadoria produzida por pessoa jurídica estabelecida nas Áreas de Livre Comércio, o crédito será determinado mediante a aplicação da alíquota: PIS - de 0,65%. COFINS - de 3%.</t>
+        </is>
+      </c>
+      <c r="F495" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>0207.14.00</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E496" t="inlineStr"/>
+      <c r="F496" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>1507.90.11</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>ZFM - PIS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E497" t="inlineStr">
+        <is>
+          <t>CRÉDITO ZONA FRANCA DE MANAUS - De acordo com o §§ 12, art. 3º da Lei nº 10.637/2002 e o § 17, art. 3º da Lei nº 10.833/2003, ressalvado o disposto no § 2° do referido artigo e nos §§ 1° a 3° do art. 2°, na aquisição de mercadoria produzida por pessoa jurídica estabelecida na ZFM, consoante projeto aprovado pela Suframa, o crédito será determinado mediante a aplicação da alíquota: PIS a) de alíquota de 1% e, b) de 1,65%, na situação de que trata a alínea ""b"" do inciso II do § 4° do art. 2° da Lei nº 10.637/2002. COFINS a) de 5,60%, nas operações com os bens referidos no inciso VI do art. 28 da Lei n° 11.196/2005; b) de 7,60%, na situação de que trata a alínea ""b"" do inciso II do § 5° do art. 2° desta Lei; e c) de 4,60%, nos demais casos. CRÉDITO ÁREA DE LIVRE COMÉRCIO - Segundo os §§ 15 e 16, art. 3º da Lei nº 10.637/2002 e §§ 23 e 24, art. 3º da Lei nº 10.833/2003, na hipótese de aquisição de mercadoria produzida por pessoa jurídica estabelecida nas Áreas de Livre Comércio, o crédito será determinado mediante a aplicação da alíquota: PIS - de 0,65%. COFINS - de 3%.</t>
+        </is>
+      </c>
+      <c r="F497" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>1507.90.11</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E498" t="inlineStr"/>
+      <c r="F498" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>2710.19.32</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>ZFM - PIS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E499" t="inlineStr">
+        <is>
+          <t>CRÉDITO ZONA FRANCA DE MANAUS - De acordo com o §§ 12, art. 3º da Lei nº 10.637/2002 e o § 17, art. 3º da Lei nº 10.833/2003, ressalvado o disposto no § 2° do referido artigo e nos §§ 1° a 3° do art. 2°, na aquisição de mercadoria produzida por pessoa jurídica estabelecida na ZFM, consoante projeto aprovado pela Suframa, o crédito será determinado mediante a aplicação da alíquota: PIS a) de alíquota de 1% e, b) de 1,65%, na situação de que trata a alínea ""b"" do inciso II do § 4° do art. 2° da Lei nº 10.637/2002. COFINS a) de 5,60%, nas operações com os bens referidos no inciso VI do art. 28 da Lei n° 11.196/2005; b) de 7,60%, na situação de que trata a alínea ""b"" do inciso II do § 5° do art. 2° desta Lei; e c) de 4,60%, nos demais casos. CRÉDITO ÁREA DE LIVRE COMÉRCIO - Segundo os §§ 15 e 16, art. 3º da Lei nº 10.637/2002 e §§ 23 e 24, art. 3º da Lei nº 10.833/2003, na hipótese de aquisição de mercadoria produzida por pessoa jurídica estabelecida nas Áreas de Livre Comércio, o crédito será determinado mediante a aplicação da alíquota: PIS - de 0,65%. COFINS - de 3%.</t>
+        </is>
+      </c>
+      <c r="F499" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>2710.19.32</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E500" t="inlineStr"/>
+      <c r="F500" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>3926.90.90</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>ZFM - PIS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>CRÉDITO ZONA FRANCA DE MANAUS - De acordo com o §§ 12, art. 3º da Lei nº 10.637/2002 e o § 17, art. 3º da Lei nº 10.833/2003, ressalvado o disposto no § 2° do referido artigo e nos §§ 1° a 3° do art. 2°, na aquisição de mercadoria produzida por pessoa jurídica estabelecida na ZFM, consoante projeto aprovado pela Suframa, o crédito será determinado mediante a aplicação da alíquota: PIS a) de alíquota de 1% e, b) de 1,65%, na situação de que trata a alínea ""b"" do inciso II do § 4° do art. 2° da Lei nº 10.637/2002. COFINS a) de 5,60%, nas operações com os bens referidos no inciso VI do art. 28 da Lei n° 11.196/2005; b) de 7,60%, na situação de que trata a alínea ""b"" do inciso II do § 5° do art. 2° desta Lei; e c) de 4,60%, nos demais casos. CRÉDITO ÁREA DE LIVRE COMÉRCIO - Segundo os §§ 15 e 16, art. 3º da Lei nº 10.637/2002 e §§ 23 e 24, art. 3º da Lei nº 10.833/2003, na hipótese de aquisição de mercadoria produzida por pessoa jurídica estabelecida nas Áreas de Livre Comércio, o crédito será determinado mediante a aplicação da alíquota: PIS - de 0,65%. COFINS - de 3%.</t>
+        </is>
+      </c>
+      <c r="F501" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>3926.90.90</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E502" t="inlineStr"/>
+      <c r="F502" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>9403.60.00</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>ZFM - PIS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E503" t="inlineStr">
+        <is>
+          <t>CRÉDITO ZONA FRANCA DE MANAUS - De acordo com o §§ 12, art. 3º da Lei nº 10.637/2002 e o § 17, art. 3º da Lei nº 10.833/2003, ressalvado o disposto no § 2° do referido artigo e nos §§ 1° a 3° do art. 2°, na aquisição de mercadoria produzida por pessoa jurídica estabelecida na ZFM, consoante projeto aprovado pela Suframa, o crédito será determinado mediante a aplicação da alíquota: PIS a) de alíquota de 1% e, b) de 1,65%, na situação de que trata a alínea ""b"" do inciso II do § 4° do art. 2° da Lei nº 10.637/2002. COFINS a) de 5,60%, nas operações com os bens referidos no inciso VI do art. 28 da Lei n° 11.196/2005; b) de 7,60%, na situação de que trata a alínea ""b"" do inciso II do § 5° do art. 2° desta Lei; e c) de 4,60%, nos demais casos. CRÉDITO ÁREA DE LIVRE COMÉRCIO - Segundo os §§ 15 e 16, art. 3º da Lei nº 10.637/2002 e §§ 23 e 24, art. 3º da Lei nº 10.833/2003, na hipótese de aquisição de mercadoria produzida por pessoa jurídica estabelecida nas Áreas de Livre Comércio, o crédito será determinado mediante a aplicação da alíquota: PIS - de 0,65%. COFINS - de 3%.</t>
+        </is>
+      </c>
+      <c r="F503" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>9403.60.00</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E504" t="inlineStr"/>
+      <c r="F504" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>8517.12.31</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>ZFM - PIS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E505" t="inlineStr">
+        <is>
+          <t>CRÉDITO ZONA FRANCA DE MANAUS - De acordo com o §§ 12, art. 3º da Lei nº 10.637/2002 e o § 17, art. 3º da Lei nº 10.833/2003, ressalvado o disposto no § 2° do referido artigo e nos §§ 1° a 3° do art. 2°, na aquisição de mercadoria produzida por pessoa jurídica estabelecida na ZFM, consoante projeto aprovado pela Suframa, o crédito será determinado mediante a aplicação da alíquota: PIS a) de alíquota de 1% e, b) de 1,65%, na situação de que trata a alínea ""b"" do inciso II do § 4° do art. 2° da Lei nº 10.637/2002. COFINS a) de 5,60%, nas operações com os bens referidos no inciso VI do art. 28 da Lei n° 11.196/2005; b) de 7,60%, na situação de que trata a alínea ""b"" do inciso II do § 5° do art. 2° desta Lei; e c) de 4,60%, nos demais casos. CRÉDITO ÁREA DE LIVRE COMÉRCIO - Segundo os §§ 15 e 16, art. 3º da Lei nº 10.637/2002 e §§ 23 e 24, art. 3º da Lei nº 10.833/2003, na hipótese de aquisição de mercadoria produzida por pessoa jurídica estabelecida nas Áreas de Livre Comércio, o crédito será determinado mediante a aplicação da alíquota: PIS - de 0,65%. COFINS - de 3%.</t>
+        </is>
+      </c>
+      <c r="F505" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>8517.12.31</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E506" t="inlineStr"/>
+      <c r="F506" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>0402.21.10</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>ZFM - PIS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E507" t="inlineStr">
+        <is>
+          <t>CRÉDITO ZONA FRANCA DE MANAUS - De acordo com o §§ 12, art. 3º da Lei nº 10.637/2002 e o § 17, art. 3º da Lei nº 10.833/2003, ressalvado o disposto no § 2° do referido artigo e nos §§ 1° a 3° do art. 2°, na aquisição de mercadoria produzida por pessoa jurídica estabelecida na ZFM, consoante projeto aprovado pela Suframa, o crédito será determinado mediante a aplicação da alíquota: PIS a) de alíquota de 1% e, b) de 1,65%, na situação de que trata a alínea ""b"" do inciso II do § 4° do art. 2° da Lei nº 10.637/2002. COFINS a) de 5,60%, nas operações com os bens referidos no inciso VI do art. 28 da Lei n° 11.196/2005; b) de 7,60%, na situação de que trata a alínea ""b"" do inciso II do § 5° do art. 2° desta Lei; e c) de 4,60%, nos demais casos. CRÉDITO ÁREA DE LIVRE COMÉRCIO - Segundo os §§ 15 e 16, art. 3º da Lei nº 10.637/2002 e §§ 23 e 24, art. 3º da Lei nº 10.833/2003, na hipótese de aquisição de mercadoria produzida por pessoa jurídica estabelecida nas Áreas de Livre Comércio, o crédito será determinado mediante a aplicação da alíquota: PIS - de 0,65%. COFINS - de 3%.</t>
+        </is>
+      </c>
+      <c r="F507" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:06</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>0402.21.10</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E508" t="inlineStr"/>
+      <c r="F508" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: ajuste de card no dashboard
</commit_message>
<xml_diff>
--- a/bcoDados.xlsx
+++ b/bcoDados.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BR27"/>
+  <dimension ref="A1:BR29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -834,7 +834,7 @@
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>0,00%</t>
+          <t>0,65%</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
@@ -5931,7 +5931,7 @@
       <c r="BQ26" s="1" t="n"/>
       <c r="BR26" s="1" t="n"/>
     </row>
-    <row r="27">
+    <row r="27" ht="409.6" customHeight="1">
       <c r="A27" s="1" t="n">
         <v>64041100</v>
       </c>
@@ -6090,6 +6090,387 @@
       <c r="BQ27" s="1" t="n"/>
       <c r="BR27" s="1" t="n"/>
     </row>
+    <row r="28">
+      <c r="A28" s="1" t="n">
+        <v>9012100</v>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
+        <is>
+          <t>0901.21.00</t>
+        </is>
+      </c>
+      <c r="C28" s="1" t="inlineStr">
+        <is>
+          <t>Café, mesmo torrado ou descafeinado; cascas e películas de café; sucedâneos do café que contenham café em qualquer proporção — Não descafeinado</t>
+        </is>
+      </c>
+      <c r="D28" s="1" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+      <c r="E28" s="1" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+      <c r="F28" s="1" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+      <c r="G28" s="1" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+      <c r="H28" s="1" t="inlineStr">
+        <is>
+          <t>Cumulativo / Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="I28" s="1" t="inlineStr">
+        <is>
+          <t>Cum: Lei nº 10.925/2004, artigo 1º, inciso XXI | N.Cum: Lei nº 10.925/2004, artigo 1º, inciso XXI</t>
+        </is>
+      </c>
+      <c r="J28" s="1" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+REGIME CUMULATIVO / NÃO CUMULATIVO - O produto está sujeito à alíquota zero do PIS e da COFINS (Lei nº 10.925/2004, artigo 1º, inciso XXI).</t>
+        </is>
+      </c>
+      <c r="K28" s="1" t="n"/>
+      <c r="L28" s="1" t="n"/>
+      <c r="M28" s="1" t="n"/>
+      <c r="N28" s="1" t="n"/>
+      <c r="O28" s="1" t="n"/>
+      <c r="P28" s="1" t="n"/>
+      <c r="Q28" s="1" t="inlineStr">
+        <is>
+          <t>Cum: Lei nº 10.996/2004, artigo 2º; Lei Complementar nº 224/2025 | N.Cum: Lei nº 10.996/2004, artigo 2º; Lei Complementar nº 224/2025</t>
+        </is>
+      </c>
+      <c r="R28" s="1" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+ZONA FRANCA DE MANAUS (ZFM) - Para os regimes cumulativo e não cumulativo, ficam reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas de vendas de mercadorias destinadas ao consumo (utilizadas diretamente ou para comercialização por atacado ou a varejo) ou à industrialização na Zona Franca de Manaus, por pessoa jurídica estabelecida fora da ZFM (Lei nº 10.996/2004, artigo 2º).
+Nas notas fiscais relativas à venda, deverá constar a expressão "Venda de mercadoria efetuada com alíquota zero da Contribuição para o PIS/Pasep e da COFINS - Lei nº 10.996/2004, artigo 2º".
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, terão a alíquota do PIS e da COFINS reduzidas a zero, exceto nas vendas de mercadorias que tenham como destinatárias pessoas jurídicas atacadistas e varejistas, sujeitas ao regime de apuração não cumulativa do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, §§ 3º e 4º). As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+MATÉRIAS-PRIMAS, PRODUTOS INTERMEDIÁRIOS E MATERIAIS DE EMBALAGEM - São reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas decorrentes da comercialização de matérias-primas, produtos intermediários e materiais de embalagem, produzidos na Zona Franca de Manaus para emprego em processo de industrialização por estabelecimentos industriais dos regimes cumulativo ou não cumulativo ali instalados, consoante projetos aprovados pelo Conselho de Administração da Superintendência da Zona Franca de Manaus (SUFRAMA) (Lei nº 10.637/2002, artigo 5º-A).
+REGIME NÃO CUMULATIVO - As alíquotas especiais para vendas realizadas por pessoa jurídica optante pelo regime não cumulativo estabelecida na Zona Franca de Manaus estão dispostas abaixo do item "Solução de Consulta".</t>
+        </is>
+      </c>
+      <c r="S28" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="T28" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="U28" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="V28" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="W28" s="1" t="inlineStr">
+        <is>
+          <t>Cum: Lei nº 10.925/2004, artigo 1º, inciso XXI | N.Cum: Lei nº 10.925/2004, artigo 1º, inciso XXI</t>
+        </is>
+      </c>
+      <c r="X28" s="1" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+REGIME CUMULATIVO / NÃO CUMULATIVO - O produto está sujeito à alíquota zero do PIS e da COFINS (Lei nº 10.925/2004, artigo 1º, inciso XXI).</t>
+        </is>
+      </c>
+      <c r="Y28" s="1" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+      <c r="Z28" s="1" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+      <c r="AA28" s="1" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+      <c r="AB28" s="1" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+      <c r="AC28" s="1" t="n"/>
+      <c r="AD28" s="1" t="n"/>
+      <c r="AE28" s="1" t="n"/>
+      <c r="AF28" s="1" t="n"/>
+      <c r="AG28" s="1" t="n"/>
+      <c r="AH28" s="1" t="n"/>
+      <c r="AI28" s="1" t="n"/>
+      <c r="AJ28" s="1" t="n"/>
+      <c r="AK28" s="1" t="n"/>
+      <c r="AL28" s="1" t="n"/>
+      <c r="AM28" s="1" t="n"/>
+      <c r="AN28" s="1" t="n"/>
+      <c r="AO28" s="1" t="n"/>
+      <c r="AP28" s="1" t="n"/>
+      <c r="AQ28" s="1" t="n"/>
+      <c r="AR28" s="1" t="n"/>
+      <c r="AS28" s="1" t="n"/>
+      <c r="AT28" s="1" t="n"/>
+      <c r="AU28" s="1" t="n"/>
+      <c r="AV28" s="1" t="n"/>
+      <c r="AW28" s="1" t="n"/>
+      <c r="AX28" s="1" t="n"/>
+      <c r="AY28" s="1" t="n"/>
+      <c r="AZ28" s="1" t="n"/>
+      <c r="BA28" s="1" t="n"/>
+      <c r="BB28" s="1" t="n"/>
+      <c r="BC28" s="1" t="n"/>
+      <c r="BD28" s="1" t="n"/>
+      <c r="BE28" s="1" t="n"/>
+      <c r="BF28" s="1" t="n"/>
+      <c r="BG28" s="1" t="n"/>
+      <c r="BH28" s="1" t="n"/>
+      <c r="BI28" s="1" t="n"/>
+      <c r="BJ28" s="1" t="n"/>
+      <c r="BK28" s="1" t="n"/>
+      <c r="BL28" s="1" t="n"/>
+      <c r="BM28" s="1" t="n"/>
+      <c r="BN28" s="1" t="n"/>
+      <c r="BO28" s="1" t="n"/>
+      <c r="BP28" s="1" t="n"/>
+      <c r="BQ28" s="1" t="n"/>
+      <c r="BR28" s="1" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="n">
+        <v>85285200</v>
+      </c>
+      <c r="B29" s="1" t="inlineStr">
+        <is>
+          <t>8528.52.00</t>
+        </is>
+      </c>
+      <c r="C29" s="1" t="inlineStr">
+        <is>
+          <t>Monitores e projetores, que não incorporem aparelho receptor de televisão; aparelhos receptores de televisão, mesmo que incorporem um aparelho receptor de radiodifusão ou um aparelho de gravação ou de reprodução de som ou de imagens — Capazes de serem conectados diretamente a uma máquina automática para processamento de dados da posição 84.71 e concebidos para serem utilizados com esta máquina</t>
+        </is>
+      </c>
+      <c r="D29" s="1" t="inlineStr">
+        <is>
+          <t>0,65%</t>
+        </is>
+      </c>
+      <c r="E29" s="1" t="inlineStr">
+        <is>
+          <t>3,00%</t>
+        </is>
+      </c>
+      <c r="F29" s="1" t="inlineStr">
+        <is>
+          <t>1,65%</t>
+        </is>
+      </c>
+      <c r="G29" s="1" t="inlineStr">
+        <is>
+          <t>7,60%</t>
+        </is>
+      </c>
+      <c r="H29" s="1" t="inlineStr">
+        <is>
+          <t>Cumulativo / Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="I29" s="1" t="inlineStr">
+        <is>
+          <t>Cum: Lei nº 9.715/98, artigo 8º, inciso I; Lei nº 9.718/98, artigo 8º | N.Cum: Lei nº 10.637/2002, artigo 2º; Lei nº 10.833/2003, artigo 2º</t>
+        </is>
+      </c>
+      <c r="J29" s="1" t="inlineStr">
+        <is>
+          <t>ALTERAÇÃO NA NCM - A reclassificação dos códigos NCM promovida pelo Decreto nº 11.158/2022 não faz com que o produto sofra alteração de tributação prevista na legislação mencionada anteriormente.
+Desta forma, a definição da NCM deverá seguir o disposto no artigo 16 do RIPI (Decreto nº 7.212/2010). Para verificar se houve reclassificação utilize a ferramenta Correlação da NCM.
+REGRA GERAL - O código NCM pesquisado não se encontra dentre os produtos com benefícios fiscais de PIS e COFINS previstos em legislação. Antes de aplicar as alíquotas correspondentes ao regime tributário da pessoa jurídica é recomendado analisar as outras guias.
+CONDIÇÃO DO ADQUIRENTE - Antes de aplicar a alíquota básica, é importante verificar se a pessoa jurídica adquirente é habilitada em algum regime especial, se está localizada na Zona Franca de Manaus (ZFM) ou em Área de Livre Comércio (ALC), e se a receita é proveniente de exportação de mercadorias.
+SIMPLES NACIONAL - A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+DARF - As empresas optantes pelo regime cumulativo recolherão o PIS e a COFINS em DARF, nos códigos 8109 e 2172, respectivamente.
+Para o regime não cumulativo os códigos serão 6912 e 5856.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
+      <c r="K29" s="1" t="inlineStr">
+        <is>
+          <t>Cum: Lei nº 12.599/2012, artigos 12 a 15; Decreto nº 7.729/2012; Lei Complementar nº 224/2025 | N.Cum: Lei nº 12.599/2012, artigos 12 a 15; Decreto nº 7.729/2012; Lei Complementar nº 224/2025</t>
+        </is>
+      </c>
+      <c r="L29" s="1" t="inlineStr">
+        <is>
+          <t>ALTERAÇÃO NA NCM - A reclassificação dos códigos NCM promovida pelo Decreto nº 11.158/2022 não faz com que o produto sofra alteração de tributação prevista na legislação mencionada anteriormente.
+Desta forma, a definição da NCM deverá seguir o disposto no artigo 16 do RIPI (Decreto nº 7.212/2010). Para verificar se houve reclassificação utilize a ferramenta Correlação da NCM.
+SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da suspensão do PIS e da COFINS sobre as receitas de vendas de mercadorias, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+REGIME CUMULATIVO / NÃO CUMULATIVO - Aplica-se a suspensão do PIS e da COFINS nos casos de venda realizada a pessoa jurídica inscrita no Regime Especial de Tributação para Desenvolvimento da Atividade de Exibição Cinematográfica (RECINE) (Lei nº 12.599/2012, artigos 12 a 15; Decreto nº 7.729/2012).
+Prazo de vigência do benefício do RECINE: Até 31.12.2029 (Lei nº 13.594/2018).
+A partir de 01.04.2026, os incentivos e benefícios federais de natureza tributária são reduzidos, sendo aqueles de alíquota zero mediante a aplicação de alíquota correspondente a 10% da alíquota do sistema padrão de tributação. Desta forma, tendo em vista que para o PIS e a Cofins existem dois regimes de tributação, as alíquotas devem corresponder a 10% das alíquotas padrão de cada um dos regimes:
+a) Regime cumulativo - PIS: 0,065%; Cofins: 0,3%;
+b) Regime não cumulativo - PIS: 0,165%; Cofins: 0,76%. (Lei Complementar nº 224/2025, artigo 4º, caput e § 4º, inciso I)
+Ressalta-se que o § 1°, do artigo 2°, da IN RFB n° 2.305/2025 limita a redução dos benefícios àqueles discriminados no demonstrativo de gastos tributários anexo à Lei Orçamentária Anual de 2026. O Recine está discriminado, sofrendo redução do benefício.
+Quanto à aplicação da redução dos benefícios, no caso da suspensão, o artigo 6°, da IN RFB n° 2.305/2025 estabelece que a redução não se aplica aos benefícios de suspensão em que se verifique apenas um diferimento temporal no recolhimento do tributo. Logo, tendo em vista que o inciso II, do § 3°, do artigo 14, da Lei n° 12.599/2012 estabelece que a suspensão do PIS/Cofins converte-se em alíquota zero após a incorporação do bem ou material de construção no ativo imobilizado ou sua utilização no complexo de exibição cinematográfica ou cinema itinerante, situação na qual a operação fica sujeita à redução do benefício disposto na Lei Complementar nº 224/2025.
+Preventivamente, a sugestão é de que no cálculo para demonstrar o aumento da carga deve ser aplicado 10% das alíquotas do sistema padrão de PIS/Cofins sobre as vendas ou importação, baseado no artigo 7° da IN RFB 2.305/2025. Tal sugestão é um entendimento que poderá ser confirmado ou reformulado mediante esclarecimento da RFB.
+Visto que essas informações não estão claras na legislação, recomenda-se ao contribuinte buscar o serviço do Receita Soluciona, por meio das Confederações Nacionais de Representação de Categorias Econômicas, às Centrais Sindicais, aos Órgãos de Registro de Classe com atuação nacional e Organizações Associativas Patronais e Empresarias.</t>
+        </is>
+      </c>
+      <c r="M29" s="1" t="inlineStr">
+        <is>
+          <t>0,065%</t>
+        </is>
+      </c>
+      <c r="N29" s="1" t="inlineStr">
+        <is>
+          <t>0,30%</t>
+        </is>
+      </c>
+      <c r="O29" s="1" t="inlineStr">
+        <is>
+          <t>0,165%</t>
+        </is>
+      </c>
+      <c r="P29" s="1" t="inlineStr">
+        <is>
+          <t>0,76%</t>
+        </is>
+      </c>
+      <c r="Q29" s="1" t="inlineStr">
+        <is>
+          <t>Cum: Lei nº 10.996/2004, artigo 2º; Lei Complementar nº 224/2025 | N.Cum: Lei nº 10.996/2004, artigo 2º; Lei Complementar nº 224/2025</t>
+        </is>
+      </c>
+      <c r="R29" s="1" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+ZONA FRANCA DE MANAUS (ZFM) - Para os regimes cumulativo e não cumulativo, ficam reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas de vendas de mercadorias destinadas ao consumo (utilizadas diretamente ou para comercialização por atacado ou a varejo) ou à industrialização na Zona Franca de Manaus, por pessoa jurídica estabelecida fora da ZFM (Lei nº 10.996/2004, artigo 2º).
+Nas notas fiscais relativas à venda, deverá constar a expressão "Venda de mercadoria efetuada com alíquota zero da Contribuição para o PIS/Pasep e da COFINS - Lei nº 10.996/2004, artigo 2º".
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, terão a alíquota do PIS e da COFINS reduzidas a zero, exceto nas vendas de mercadorias que tenham como destinatárias pessoas jurídicas atacadistas e varejistas, sujeitas ao regime de apuração não cumulativa do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, §§ 3º e 4º). As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+MATÉRIAS-PRIMAS, PRODUTOS INTERMEDIÁRIOS E MATERIAIS DE EMBALAGEM - São reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas decorrentes da comercialização de matérias-primas, produtos intermediários e materiais de embalagem, produzidos na Zona Franca de Manaus para emprego em processo de industrialização por estabelecimentos industriais dos regimes cumulativo ou não cumulativo ali instalados, consoante projetos aprovados pelo Conselho de Administração da Superintendência da Zona Franca de Manaus (SUFRAMA) (Lei nº 10.637/2002, artigo 5º-A).
+REGIME NÃO CUMULATIVO - As alíquotas especiais para vendas realizadas por pessoa jurídica optante pelo regime não cumulativo estabelecida na Zona Franca de Manaus estão dispostas abaixo do item "Solução de Consulta".</t>
+        </is>
+      </c>
+      <c r="S29" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="T29" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="U29" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="V29" s="1" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+      <c r="W29" s="1" t="n"/>
+      <c r="X29" s="1" t="n"/>
+      <c r="Y29" s="1" t="n"/>
+      <c r="Z29" s="1" t="n"/>
+      <c r="AA29" s="1" t="n"/>
+      <c r="AB29" s="1" t="n"/>
+      <c r="AC29" s="1" t="n"/>
+      <c r="AD29" s="1" t="n"/>
+      <c r="AE29" s="1" t="n"/>
+      <c r="AF29" s="1" t="n"/>
+      <c r="AG29" s="1" t="n"/>
+      <c r="AH29" s="1" t="n"/>
+      <c r="AI29" s="1" t="n"/>
+      <c r="AJ29" s="1" t="n"/>
+      <c r="AK29" s="1" t="n"/>
+      <c r="AL29" s="1" t="n"/>
+      <c r="AM29" s="1" t="n"/>
+      <c r="AN29" s="1" t="n"/>
+      <c r="AO29" s="1" t="n"/>
+      <c r="AP29" s="1" t="n"/>
+      <c r="AQ29" s="1" t="n"/>
+      <c r="AR29" s="1" t="n"/>
+      <c r="AS29" s="1" t="n"/>
+      <c r="AT29" s="1" t="n"/>
+      <c r="AU29" s="1" t="n"/>
+      <c r="AV29" s="1" t="n"/>
+      <c r="AW29" s="1" t="n"/>
+      <c r="AX29" s="1" t="n"/>
+      <c r="AY29" s="1" t="n"/>
+      <c r="AZ29" s="1" t="n"/>
+      <c r="BA29" s="1" t="n"/>
+      <c r="BB29" s="1" t="n"/>
+      <c r="BC29" s="1" t="n"/>
+      <c r="BD29" s="1" t="n"/>
+      <c r="BE29" s="1" t="n"/>
+      <c r="BF29" s="1" t="n"/>
+      <c r="BG29" s="1" t="n"/>
+      <c r="BH29" s="1" t="n"/>
+      <c r="BI29" s="1" t="n"/>
+      <c r="BJ29" s="1" t="n"/>
+      <c r="BK29" s="1" t="n"/>
+      <c r="BL29" s="1" t="n"/>
+      <c r="BM29" s="1" t="n"/>
+      <c r="BN29" s="1" t="n"/>
+      <c r="BO29" s="1" t="n"/>
+      <c r="BP29" s="1" t="n"/>
+      <c r="BQ29" s="1" t="n"/>
+      <c r="BR29" s="1" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -6104,7 +6485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F666"/>
+  <dimension ref="A1:F708"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -26301,6 +26682,1415 @@
         </is>
       </c>
     </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>8471.41.90</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D667" t="inlineStr">
+        <is>
+          <t>PIS Cumulativo</t>
+        </is>
+      </c>
+      <c r="E667" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+      <c r="F667" t="inlineStr">
+        <is>
+          <t>0,65%</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>6404.11.00</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>Atualização</t>
+        </is>
+      </c>
+      <c r="D668" t="inlineStr">
+        <is>
+          <t>PIS Cumulativo</t>
+        </is>
+      </c>
+      <c r="E668" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+      <c r="F668" t="inlineStr">
+        <is>
+          <t>0,65%</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>0901.21.00</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D669" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F669" t="inlineStr">
+        <is>
+          <t>Café, mesmo torrado ou descafeinado; cascas e películas de café; sucedâneos do café que contenham café em qualquer proporção — Não descafeinado</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>0901.21.00</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>PIS Cumulativo</t>
+        </is>
+      </c>
+      <c r="E670" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F670" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>0901.21.00</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D671" t="inlineStr">
+        <is>
+          <t>COFINS Cumulativo</t>
+        </is>
+      </c>
+      <c r="E671" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F671" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>0901.21.00</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>PIS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F672" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>0901.21.00</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D673" t="inlineStr">
+        <is>
+          <t>COFINS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F673" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>0901.21.00</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D674" t="inlineStr">
+        <is>
+          <t>Regime</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F674" t="inlineStr">
+        <is>
+          <t>Cumulativo / Não Cumulativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>0901.21.00</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D675" t="inlineStr">
+        <is>
+          <t>Legislação</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F675" t="inlineStr">
+        <is>
+          <t>Cum: Lei nº 10.925/2004, artigo 1º, inciso XXI | N.Cum: Lei nº 10.925/2004, artigo 1º, inciso XXI</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>0901.21.00</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D676" t="inlineStr">
+        <is>
+          <t>Observações (Regra Geral)</t>
+        </is>
+      </c>
+      <c r="E676" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F676" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+REGIME CUMULATIVO / NÃO CUMULATIVO - O produto está sujeito à alíquota zero do PIS e da COFINS (Lei nº 10.925/2004, artigo 1º, inciso XXI).</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>0901.21.00</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D677" t="inlineStr">
+        <is>
+          <t>Alíquota Zero - PIS Cumulativo</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F677" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>0901.21.00</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D678" t="inlineStr">
+        <is>
+          <t>Alíquota Zero - COFINS Cumulativo</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F678" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>0901.21.00</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D679" t="inlineStr">
+        <is>
+          <t>Alíquota Zero - PIS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F679" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>0901.21.00</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>Alíquota Zero - COFINS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F680" t="inlineStr">
+        <is>
+          <t>0,00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>0901.21.00</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D681" t="inlineStr">
+        <is>
+          <t>Alíquota Zero - Legislação</t>
+        </is>
+      </c>
+      <c r="E681" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F681" t="inlineStr">
+        <is>
+          <t>Cum: Lei nº 10.925/2004, artigo 1º, inciso XXI | N.Cum: Lei nº 10.925/2004, artigo 1º, inciso XXI</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>0901.21.00</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D682" t="inlineStr">
+        <is>
+          <t>Alíquota Zero - Observações</t>
+        </is>
+      </c>
+      <c r="E682" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F682" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+REGIME CUMULATIVO / NÃO CUMULATIVO - O produto está sujeito à alíquota zero do PIS e da COFINS (Lei nº 10.925/2004, artigo 1º, inciso XXI).</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>0901.21.00</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D683" t="inlineStr">
+        <is>
+          <t>ZFM - PIS Cumulativo</t>
+        </is>
+      </c>
+      <c r="E683" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F683" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>0901.21.00</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D684" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS Cumulativo</t>
+        </is>
+      </c>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F684" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>0901.21.00</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D685" t="inlineStr">
+        <is>
+          <t>ZFM - PIS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F685" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>0901.21.00</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D686" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E686" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F686" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>0901.21.00</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D687" t="inlineStr">
+        <is>
+          <t>ZFM - Legislação</t>
+        </is>
+      </c>
+      <c r="E687" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F687" t="inlineStr">
+        <is>
+          <t>Cum: Lei nº 10.996/2004, artigo 2º; Lei Complementar nº 224/2025 | N.Cum: Lei nº 10.996/2004, artigo 2º; Lei Complementar nº 224/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>0901.21.00</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D688" t="inlineStr">
+        <is>
+          <t>ZFM - Observações</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F688" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+ZONA FRANCA DE MANAUS (ZFM) - Para os regimes cumulativo e não cumulativo, ficam reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas de vendas de mercadorias destinadas ao consumo (utilizadas diretamente ou para comercialização por atacado ou a varejo) ou à industrialização na Zona Franca de Manaus, por pessoa jurídica estabelecida fora da ZFM (Lei nº 10.996/2004, artigo 2º).
+Nas notas fiscais relativas à venda, deverá constar a expressão "Venda de mercadoria efetuada com alíquota zero da Contribuição para o PIS/Pasep e da COFINS - Lei nº 10.996/2004, artigo 2º".
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, terão a alíquota do PIS e da COFINS reduzidas a zero, exceto nas vendas de mercadorias que tenham como destinatárias pessoas jurídicas atacadistas e varejistas, sujeitas ao regime de apuração não cumulativa do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, §§ 3º e 4º). As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+MATÉRIAS-PRIMAS, PRODUTOS INTERMEDIÁRIOS E MATERIAIS DE EMBALAGEM - São reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas decorrentes da comercialização de matérias-primas, produtos intermediários e materiais de embalagem, produzidos na Zona Franca de Manaus para emprego em processo de industrialização por estabelecimentos industriais dos regimes cumulativo ou não cumulativo ali instalados, consoante projetos aprovados pelo Conselho de Administração da Superintendência da Zona Franca de Manaus (SUFRAMA) (Lei nº 10.637/2002, artigo 5º-A).
+REGIME NÃO CUMULATIVO - As alíquotas especiais para vendas realizadas por pessoa jurídica optante pelo regime não cumulativo estabelecida na Zona Franca de Manaus estão dispostas abaixo do item "Solução de Consulta".</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>8528.52.00</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D689" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="E689" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F689" t="inlineStr">
+        <is>
+          <t>Monitores e projetores, que não incorporem aparelho receptor de televisão; aparelhos receptores de televisão, mesmo que incorporem um aparelho receptor de radiodifusão ou um aparelho de gravação ou de reprodução de som ou de imagens — Capazes de serem conectados diretamente a uma máquina automática para processamento de dados da posição 84.71 e concebidos para serem utilizados com esta máquina</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>8528.52.00</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D690" t="inlineStr">
+        <is>
+          <t>PIS Cumulativo</t>
+        </is>
+      </c>
+      <c r="E690" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F690" t="inlineStr">
+        <is>
+          <t>0,65%</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>8528.52.00</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D691" t="inlineStr">
+        <is>
+          <t>COFINS Cumulativo</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F691" t="inlineStr">
+        <is>
+          <t>3,00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>8528.52.00</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D692" t="inlineStr">
+        <is>
+          <t>PIS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F692" t="inlineStr">
+        <is>
+          <t>1,65%</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>8528.52.00</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D693" t="inlineStr">
+        <is>
+          <t>COFINS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F693" t="inlineStr">
+        <is>
+          <t>7,60%</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>8528.52.00</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D694" t="inlineStr">
+        <is>
+          <t>Regime</t>
+        </is>
+      </c>
+      <c r="E694" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F694" t="inlineStr">
+        <is>
+          <t>Cumulativo / Não Cumulativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>8528.52.00</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D695" t="inlineStr">
+        <is>
+          <t>Legislação</t>
+        </is>
+      </c>
+      <c r="E695" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F695" t="inlineStr">
+        <is>
+          <t>Cum: Lei nº 9.715/98, artigo 8º, inciso I; Lei nº 9.718/98, artigo 8º | N.Cum: Lei nº 10.637/2002, artigo 2º; Lei nº 10.833/2003, artigo 2º</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>8528.52.00</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D696" t="inlineStr">
+        <is>
+          <t>Observações (Regra Geral)</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F696" t="inlineStr">
+        <is>
+          <t>ALTERAÇÃO NA NCM - A reclassificação dos códigos NCM promovida pelo Decreto nº 11.158/2022 não faz com que o produto sofra alteração de tributação prevista na legislação mencionada anteriormente.
+Desta forma, a definição da NCM deverá seguir o disposto no artigo 16 do RIPI (Decreto nº 7.212/2010). Para verificar se houve reclassificação utilize a ferramenta Correlação da NCM.
+REGRA GERAL - O código NCM pesquisado não se encontra dentre os produtos com benefícios fiscais de PIS e COFINS previstos em legislação. Antes de aplicar as alíquotas correspondentes ao regime tributário da pessoa jurídica é recomendado analisar as outras guias.
+CONDIÇÃO DO ADQUIRENTE - Antes de aplicar a alíquota básica, é importante verificar se a pessoa jurídica adquirente é habilitada em algum regime especial, se está localizada na Zona Franca de Manaus (ZFM) ou em Área de Livre Comércio (ALC), e se a receita é proveniente de exportação de mercadorias.
+SIMPLES NACIONAL - A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+DARF - As empresas optantes pelo regime cumulativo recolherão o PIS e a COFINS em DARF, nos códigos 8109 e 2172, respectivamente.
+Para o regime não cumulativo os códigos serão 6912 e 5856.
+O pagamento do PIS e da COFINS deverão ser efetuados até o 25º dia do mês subsequente ao mês de ocorrência dos fatos geradores (Lei nº 11.933/2009, artigo 1º). Se o dia do vencimento não for dia útil, considerar-se-á antecipado o prazo para o primeiro dia útil que o anteceder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>8528.52.00</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D697" t="inlineStr">
+        <is>
+          <t>Suspensão - PIS Cumulativo</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F697" t="inlineStr">
+        <is>
+          <t>0,065%</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>8528.52.00</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D698" t="inlineStr">
+        <is>
+          <t>Suspensão - COFINS Cumulativo</t>
+        </is>
+      </c>
+      <c r="E698" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F698" t="inlineStr">
+        <is>
+          <t>0,30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>8528.52.00</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D699" t="inlineStr">
+        <is>
+          <t>Suspensão - PIS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E699" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F699" t="inlineStr">
+        <is>
+          <t>0,165%</t>
+        </is>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>8528.52.00</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D700" t="inlineStr">
+        <is>
+          <t>Suspensão - COFINS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E700" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F700" t="inlineStr">
+        <is>
+          <t>0,76%</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>8528.52.00</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D701" t="inlineStr">
+        <is>
+          <t>Suspensão - Legislação</t>
+        </is>
+      </c>
+      <c r="E701" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F701" t="inlineStr">
+        <is>
+          <t>Cum: Lei nº 12.599/2012, artigos 12 a 15; Decreto nº 7.729/2012; Lei Complementar nº 224/2025 | N.Cum: Lei nº 12.599/2012, artigos 12 a 15; Decreto nº 7.729/2012; Lei Complementar nº 224/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>8528.52.00</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D702" t="inlineStr">
+        <is>
+          <t>Suspensão - Observações</t>
+        </is>
+      </c>
+      <c r="E702" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F702" t="inlineStr">
+        <is>
+          <t>ALTERAÇÃO NA NCM - A reclassificação dos códigos NCM promovida pelo Decreto nº 11.158/2022 não faz com que o produto sofra alteração de tributação prevista na legislação mencionada anteriormente.
+Desta forma, a definição da NCM deverá seguir o disposto no artigo 16 do RIPI (Decreto nº 7.212/2010). Para verificar se houve reclassificação utilize a ferramenta Correlação da NCM.
+SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da suspensão do PIS e da COFINS sobre as receitas de vendas de mercadorias, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+Nos casos de estabelecimento comercial importador e a saída das mercadorias seja de procedência estrangeira, estará equiparada a industrial pela legislação do IPI, tributando dessa forma pelo Anexo II, conforme o ADI RFB nº 01/2018.
+REGIME CUMULATIVO / NÃO CUMULATIVO - Aplica-se a suspensão do PIS e da COFINS nos casos de venda realizada a pessoa jurídica inscrita no Regime Especial de Tributação para Desenvolvimento da Atividade de Exibição Cinematográfica (RECINE) (Lei nº 12.599/2012, artigos 12 a 15; Decreto nº 7.729/2012).
+Prazo de vigência do benefício do RECINE: Até 31.12.2029 (Lei nº 13.594/2018).
+A partir de 01.04.2026, os incentivos e benefícios federais de natureza tributária são reduzidos, sendo aqueles de alíquota zero mediante a aplicação de alíquota correspondente a 10% da alíquota do sistema padrão de tributação. Desta forma, tendo em vista que para o PIS e a Cofins existem dois regimes de tributação, as alíquotas devem corresponder a 10% das alíquotas padrão de cada um dos regimes:
+a) Regime cumulativo - PIS: 0,065%; Cofins: 0,3%;
+b) Regime não cumulativo - PIS: 0,165%; Cofins: 0,76%. (Lei Complementar nº 224/2025, artigo 4º, caput e § 4º, inciso I)
+Ressalta-se que o § 1°, do artigo 2°, da IN RFB n° 2.305/2025 limita a redução dos benefícios àqueles discriminados no demonstrativo de gastos tributários anexo à Lei Orçamentária Anual de 2026. O Recine está discriminado, sofrendo redução do benefício.
+Quanto à aplicação da redução dos benefícios, no caso da suspensão, o artigo 6°, da IN RFB n° 2.305/2025 estabelece que a redução não se aplica aos benefícios de suspensão em que se verifique apenas um diferimento temporal no recolhimento do tributo. Logo, tendo em vista que o inciso II, do § 3°, do artigo 14, da Lei n° 12.599/2012 estabelece que a suspensão do PIS/Cofins converte-se em alíquota zero após a incorporação do bem ou material de construção no ativo imobilizado ou sua utilização no complexo de exibição cinematográfica ou cinema itinerante, situação na qual a operação fica sujeita à redução do benefício disposto na Lei Complementar nº 224/2025.
+Preventivamente, a sugestão é de que no cálculo para demonstrar o aumento da carga deve ser aplicado 10% das alíquotas do sistema padrão de PIS/Cofins sobre as vendas ou importação, baseado no artigo 7° da IN RFB 2.305/2025. Tal sugestão é um entendimento que poderá ser confirmado ou reformulado mediante esclarecimento da RFB.
+Visto que essas informações não estão claras na legislação, recomenda-se ao contribuinte buscar o serviço do Receita Soluciona, por meio das Confederações Nacionais de Representação de Categorias Econômicas, às Centrais Sindicais, aos Órgãos de Registro de Classe com atuação nacional e Organizações Associativas Patronais e Empresarias.</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>8528.52.00</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D703" t="inlineStr">
+        <is>
+          <t>ZFM - PIS Cumulativo</t>
+        </is>
+      </c>
+      <c r="E703" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F703" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>8528.52.00</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D704" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS Cumulativo</t>
+        </is>
+      </c>
+      <c r="E704" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F704" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>8528.52.00</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D705" t="inlineStr">
+        <is>
+          <t>ZFM - PIS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E705" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F705" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>8528.52.00</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D706" t="inlineStr">
+        <is>
+          <t>ZFM - COFINS Não Cumulativo</t>
+        </is>
+      </c>
+      <c r="E706" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F706" t="inlineStr">
+        <is>
+          <t>Vide observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>8528.52.00</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D707" t="inlineStr">
+        <is>
+          <t>ZFM - Legislação</t>
+        </is>
+      </c>
+      <c r="E707" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F707" t="inlineStr">
+        <is>
+          <t>Cum: Lei nº 10.996/2004, artigo 2º; Lei Complementar nº 224/2025 | N.Cum: Lei nº 10.996/2004, artigo 2º; Lei Complementar nº 224/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:21</t>
+        </is>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>8528.52.00</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>Registro Inicial</t>
+        </is>
+      </c>
+      <c r="D708" t="inlineStr">
+        <is>
+          <t>ZFM - Observações</t>
+        </is>
+      </c>
+      <c r="E708" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F708" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL - As microempresas e as empresas de pequeno porte optantes pelo Simples Nacional não se beneficiam da alíquota zero do PIS e da COFINS sobre as receitas de vendas de mercadorias à Zona Franca de Manaus ou Área de Livre Comércio, devido à impossibilidade em utilizar ou destinar qualquer valor a título de incentivo fiscal (Lei Complementar nº 123/2006, artigo 24).
+A tributação do PIS e da COFINS será determinada conforme os percentuais de repartição das referidas contribuições (aplicados sobre a alíquota efetiva utilizada para apuração do DAS) constantes no Anexo de enquadramento.
+ZONA FRANCA DE MANAUS (ZFM) - Para os regimes cumulativo e não cumulativo, ficam reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas de vendas de mercadorias destinadas ao consumo (utilizadas diretamente ou para comercialização por atacado ou a varejo) ou à industrialização na Zona Franca de Manaus, por pessoa jurídica estabelecida fora da ZFM (Lei nº 10.996/2004, artigo 2º).
+Nas notas fiscais relativas à venda, deverá constar a expressão "Venda de mercadoria efetuada com alíquota zero da Contribuição para o PIS/Pasep e da COFINS - Lei nº 10.996/2004, artigo 2º".
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+ÁREAS DE LIVRE COMÉRCIO - As vendas de mercadorias destinadas ao consumo ou à industrialização nas Áreas de Livre Comércio, por pessoa jurídica optante pelos regimes cumulativo ou não cumulativo estabelecida fora dessas áreas, terão a alíquota do PIS e da COFINS reduzidas a zero, exceto nas vendas de mercadorias que tenham como destinatárias pessoas jurídicas atacadistas e varejistas, sujeitas ao regime de apuração não cumulativa do PIS e da COFINS (Lei nº 10.996/2004, artigo 2º, §§ 3º e 4º). As áreas são:
+a) Área de Livre Comércio de Tabatinga (ALCT), no Estado do Amazonas (Lei nº 7.965/89);
+b) Área de Livre Comércio de Guajará-Mirim (ALCGM), no Estado de Rondônia (Lei nº 8.210/91);
+c) Áreas de Livre Comércio de Boa Vista e Pacaraima (ALCBV) e Bonfim (ALCB), no Estado de Roraima (Lei nº 8.256/91);
+d) Área de Livre Comércio de Macapá e Santana (ALCMS), no Estado do Amapá (Lei nº 8.387/91);
+e) Áreas de Livre Comércio de Brasiléia, com extensão para o Município de Epitaciolândia (ALCB) e de Cruzeiro do Sul (ALCCS), no Estado do Acre (Lei nº 8.857/94).
+A partir de 01.04.2026, os incentivos e benefícios fiscais federais de natureza tributária serão reduzidos. Uma das exceções é voltada aos benefícios concedidos às empresas estabelecidas na ZFM, relativos ao regime especial estabelecido nos termos do artigo 40, do ADCT, bem como nas ALC, de modo que nessas condições a empresa situada na região incentivada não será impactada pelo corte de benefícios.
+A RFB, ao regulamentar as exceções previstas no § 8°, do artigo 4°, da Lei Complementar n° 224/2025, apresentou no Anexo Único, da IN RFB n° 2.305/2025, uma listagem de benefícios previstos no DGT para os quais não se aplica a redução linear. (IN RFB n° 2.305/2025, artigo 17)
+Ocorre que, o Anexo Único, da IN RFB n° 2.305/2025 compreende quase todos os benefícios de PIS e Cofins relacionados à ZFM/ALC listados DGT, Anexo à PLOA de 2026, deixando de citar o benefício de empresas de fora da ZFM/ALC que vendem para a ZFM/ALC, previsto no artigo 2°, da Lei n° 10.996/04, no Decreto n° 5.310/04 e no artigo 65, da Lei n° 11.196/05.
+Assim, preventivamente interpretamos que cabe indicação da aplicação da alíquota correspondente a 10% da alíquota do sistema padrão de tributação, que, no regime cumulativo, resultará nas alíquotas de 0,065% de PIS e 0,3% de Cofins, ao passo que, no regime não cumulativo, resultará nas alíquotas de 0,165% de PIS e 0,76% de Cofins. Essa interpretação poderá ser confirmada ou reformulada mediante esclarecimento da RFB.
+MATÉRIAS-PRIMAS, PRODUTOS INTERMEDIÁRIOS E MATERIAIS DE EMBALAGEM - São reduzidas a zero as alíquotas do PIS e da COFINS incidentes sobre as receitas decorrentes da comercialização de matérias-primas, produtos intermediários e materiais de embalagem, produzidos na Zona Franca de Manaus para emprego em processo de industrialização por estabelecimentos industriais dos regimes cumulativo ou não cumulativo ali instalados, consoante projetos aprovados pelo Conselho de Administração da Superintendência da Zona Franca de Manaus (SUFRAMA) (Lei nº 10.637/2002, artigo 5º-A).
+REGIME NÃO CUMULATIVO - As alíquotas especiais para vendas realizadas por pessoa jurídica optante pelo regime não cumulativo estabelecida na Zona Franca de Manaus estão dispostas abaixo do item "Solução de Consulta".</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
add: adições no arquivo de teste e excel
</commit_message>
<xml_diff>
--- a/bcoDados.xlsx
+++ b/bcoDados.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BR29"/>
+  <dimension ref="A1:BR31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6471,6 +6471,20 @@
       <c r="BQ29" s="1" t="n"/>
       <c r="BR29" s="1" t="n"/>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>09012100</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>85076000</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>